<commit_message>
[ Version 0.0.31.1 ] - FSM first states code were writen.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -465,7 +465,7 @@
     <t xml:space="preserve">io_byte</t>
   </si>
   <si>
-    <t xml:space="preserve">tmp_byte</t>
+    <t xml:space="preserve">ctrl_byte</t>
   </si>
   <si>
     <t xml:space="preserve">BIT STRUCTURES</t>
@@ -480,10 +480,10 @@
     <t xml:space="preserve">DATA</t>
   </si>
   <si>
-    <t xml:space="preserve">BIN MASK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HEX MASK</t>
+    <t xml:space="preserve">READ BIN MASK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">READ HEX MASK</t>
   </si>
   <si>
     <t xml:space="preserve">B0</t>
@@ -763,7 +763,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="18">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -812,17 +812,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -1139,7 +1128,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="94">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1200,59 +1189,43 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="9" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="10" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="11" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="12" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="11" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="12" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1260,7 +1233,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1280,7 +1253,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1304,7 +1277,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1320,27 +1293,23 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="180" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1348,15 +1317,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1372,7 +1345,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1384,7 +1357,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1428,7 +1401,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1496,7 +1469,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4179,576 +4152,576 @@
         <v>38</v>
       </c>
       <c r="B63" s="4"/>
-      <c r="C63" s="15" t="s">
+      <c r="C63" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="D63" s="15" t="s">
+      <c r="D63" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="E63" s="15" t="s">
+      <c r="E63" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="F63" s="15"/>
-      <c r="G63" s="15" t="s">
+      <c r="F63" s="4"/>
+      <c r="G63" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="H63" s="15"/>
-      <c r="I63" s="15" t="s">
+      <c r="H63" s="4"/>
+      <c r="I63" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="J63" s="15"/>
+      <c r="J63" s="4"/>
       <c r="L63" s="4" t="s">
         <v>38</v>
       </c>
       <c r="M63" s="4"/>
-      <c r="N63" s="15" t="s">
+      <c r="N63" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="O63" s="15" t="s">
+      <c r="O63" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="P63" s="15" t="s">
+      <c r="P63" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="Q63" s="15"/>
-      <c r="R63" s="15" t="s">
+      <c r="Q63" s="4"/>
+      <c r="R63" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="S63" s="15"/>
-      <c r="T63" s="15" t="s">
+      <c r="S63" s="4"/>
+      <c r="T63" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="U63" s="15"/>
+      <c r="U63" s="4"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="16" t="n">
+      <c r="A64" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B64" s="16"/>
-      <c r="C64" s="16" t="n">
+      <c r="B64" s="9"/>
+      <c r="C64" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="E64" s="16" t="s">
+      <c r="E64" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F64" s="16"/>
-      <c r="G64" s="16"/>
-      <c r="H64" s="16"/>
-      <c r="I64" s="16"/>
-      <c r="J64" s="16"/>
-      <c r="L64" s="16" t="n">
+      <c r="F64" s="9"/>
+      <c r="G64" s="9"/>
+      <c r="H64" s="9"/>
+      <c r="I64" s="9"/>
+      <c r="J64" s="9"/>
+      <c r="L64" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="M64" s="16"/>
-      <c r="N64" s="16" t="n">
+      <c r="M64" s="9"/>
+      <c r="N64" s="9" t="n">
         <v>1</v>
       </c>
       <c r="O64" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="P64" s="17" t="s">
+      <c r="P64" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="Q64" s="17"/>
-      <c r="R64" s="17" t="s">
+      <c r="Q64" s="5"/>
+      <c r="R64" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="S64" s="17"/>
-      <c r="T64" s="17" t="s">
+      <c r="S64" s="5"/>
+      <c r="T64" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="U64" s="17"/>
+      <c r="U64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C65" s="16"/>
+      <c r="C65" s="9"/>
       <c r="D65" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="E65" s="16" t="s">
+      <c r="E65" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F65" s="16"/>
-      <c r="G65" s="16"/>
-      <c r="H65" s="16"/>
-      <c r="I65" s="16"/>
-      <c r="J65" s="16"/>
-      <c r="N65" s="16"/>
+      <c r="F65" s="9"/>
+      <c r="G65" s="9"/>
+      <c r="H65" s="9"/>
+      <c r="I65" s="9"/>
+      <c r="J65" s="9"/>
+      <c r="N65" s="9"/>
       <c r="O65" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="P65" s="17"/>
-      <c r="Q65" s="17"/>
-      <c r="R65" s="17"/>
-      <c r="S65" s="17"/>
-      <c r="T65" s="17"/>
-      <c r="U65" s="17"/>
+      <c r="P65" s="5"/>
+      <c r="Q65" s="5"/>
+      <c r="R65" s="5"/>
+      <c r="S65" s="5"/>
+      <c r="T65" s="5"/>
+      <c r="U65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
         <v>160</v>
       </c>
       <c r="B66" s="4"/>
-      <c r="C66" s="16"/>
+      <c r="C66" s="9"/>
       <c r="D66" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="E66" s="16" t="s">
+      <c r="E66" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F66" s="16"/>
-      <c r="G66" s="16"/>
-      <c r="H66" s="16"/>
-      <c r="I66" s="16"/>
-      <c r="J66" s="16"/>
+      <c r="F66" s="9"/>
+      <c r="G66" s="9"/>
+      <c r="H66" s="9"/>
+      <c r="I66" s="9"/>
+      <c r="J66" s="9"/>
       <c r="L66" s="4" t="s">
         <v>160</v>
       </c>
       <c r="M66" s="4"/>
-      <c r="N66" s="16"/>
+      <c r="N66" s="9"/>
       <c r="O66" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="P66" s="16" t="s">
+      <c r="P66" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="Q66" s="16"/>
-      <c r="R66" s="16"/>
-      <c r="S66" s="16"/>
-      <c r="T66" s="16"/>
-      <c r="U66" s="16"/>
+      <c r="Q66" s="9"/>
+      <c r="R66" s="9"/>
+      <c r="S66" s="9"/>
+      <c r="T66" s="9"/>
+      <c r="U66" s="9"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="18" t="s">
+      <c r="A67" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B67" s="18"/>
-      <c r="C67" s="16"/>
+      <c r="B67" s="5"/>
+      <c r="C67" s="9"/>
       <c r="D67" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="E67" s="16" t="s">
+      <c r="E67" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F67" s="16"/>
-      <c r="G67" s="16"/>
-      <c r="H67" s="16"/>
-      <c r="I67" s="16"/>
-      <c r="J67" s="16"/>
-      <c r="L67" s="18" t="s">
+      <c r="F67" s="9"/>
+      <c r="G67" s="9"/>
+      <c r="H67" s="9"/>
+      <c r="I67" s="9"/>
+      <c r="J67" s="9"/>
+      <c r="L67" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="M67" s="18"/>
-      <c r="N67" s="16"/>
+      <c r="M67" s="5"/>
+      <c r="N67" s="9"/>
       <c r="O67" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="P67" s="16" t="s">
+      <c r="P67" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="Q67" s="16"/>
-      <c r="R67" s="16"/>
-      <c r="S67" s="16"/>
-      <c r="T67" s="16"/>
-      <c r="U67" s="16"/>
+      <c r="Q67" s="9"/>
+      <c r="R67" s="9"/>
+      <c r="S67" s="9"/>
+      <c r="T67" s="9"/>
+      <c r="U67" s="9"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C68" s="16"/>
+      <c r="C68" s="9"/>
       <c r="D68" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="E68" s="16" t="s">
+      <c r="E68" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F68" s="16"/>
-      <c r="G68" s="16"/>
-      <c r="H68" s="16"/>
-      <c r="I68" s="16"/>
-      <c r="J68" s="16"/>
-      <c r="N68" s="16"/>
+      <c r="F68" s="9"/>
+      <c r="G68" s="9"/>
+      <c r="H68" s="9"/>
+      <c r="I68" s="9"/>
+      <c r="J68" s="9"/>
+      <c r="N68" s="9"/>
       <c r="O68" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="P68" s="16" t="s">
+      <c r="P68" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="Q68" s="16"/>
-      <c r="R68" s="16" t="s">
+      <c r="Q68" s="9"/>
+      <c r="R68" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="S68" s="16"/>
-      <c r="T68" s="16" t="s">
+      <c r="S68" s="9"/>
+      <c r="T68" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="U68" s="16"/>
+      <c r="U68" s="9"/>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="15" t="s">
+      <c r="A69" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B69" s="15"/>
-      <c r="C69" s="16"/>
+      <c r="B69" s="4"/>
+      <c r="C69" s="9"/>
       <c r="D69" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="E69" s="16" t="s">
+      <c r="E69" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F69" s="16"/>
-      <c r="G69" s="16"/>
-      <c r="H69" s="16"/>
-      <c r="I69" s="16"/>
-      <c r="J69" s="16"/>
-      <c r="L69" s="15" t="s">
+      <c r="F69" s="9"/>
+      <c r="G69" s="9"/>
+      <c r="H69" s="9"/>
+      <c r="I69" s="9"/>
+      <c r="J69" s="9"/>
+      <c r="L69" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="M69" s="15"/>
-      <c r="N69" s="16"/>
+      <c r="M69" s="4"/>
+      <c r="N69" s="9"/>
       <c r="O69" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="P69" s="16" t="s">
+      <c r="P69" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="Q69" s="16"/>
-      <c r="R69" s="16" t="s">
+      <c r="Q69" s="9"/>
+      <c r="R69" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="S69" s="16"/>
-      <c r="T69" s="16" t="s">
+      <c r="S69" s="9"/>
+      <c r="T69" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="U69" s="16"/>
+      <c r="U69" s="9"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="18" t="s">
+      <c r="A70" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="B70" s="18"/>
-      <c r="C70" s="16"/>
+      <c r="B70" s="5"/>
+      <c r="C70" s="9"/>
       <c r="D70" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="E70" s="16" t="s">
+      <c r="E70" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F70" s="16"/>
-      <c r="G70" s="16"/>
-      <c r="H70" s="16"/>
-      <c r="I70" s="16"/>
-      <c r="J70" s="16"/>
-      <c r="L70" s="18" t="s">
+      <c r="F70" s="9"/>
+      <c r="G70" s="9"/>
+      <c r="H70" s="9"/>
+      <c r="I70" s="9"/>
+      <c r="J70" s="9"/>
+      <c r="L70" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="M70" s="18"/>
-      <c r="N70" s="16"/>
+      <c r="M70" s="5"/>
+      <c r="N70" s="9"/>
       <c r="O70" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="P70" s="16" t="s">
+      <c r="P70" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="Q70" s="16"/>
-      <c r="R70" s="16"/>
-      <c r="S70" s="16"/>
-      <c r="T70" s="16"/>
-      <c r="U70" s="16"/>
+      <c r="Q70" s="9"/>
+      <c r="R70" s="9"/>
+      <c r="S70" s="9"/>
+      <c r="T70" s="9"/>
+      <c r="U70" s="9"/>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C71" s="16"/>
+      <c r="C71" s="9"/>
       <c r="D71" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="E71" s="16" t="s">
+      <c r="E71" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F71" s="16"/>
-      <c r="G71" s="16"/>
-      <c r="H71" s="16"/>
-      <c r="I71" s="16"/>
-      <c r="J71" s="16"/>
-      <c r="N71" s="16"/>
+      <c r="F71" s="9"/>
+      <c r="G71" s="9"/>
+      <c r="H71" s="9"/>
+      <c r="I71" s="9"/>
+      <c r="J71" s="9"/>
+      <c r="N71" s="9"/>
       <c r="O71" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="P71" s="16" t="s">
+      <c r="P71" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="Q71" s="16"/>
-      <c r="R71" s="16"/>
-      <c r="S71" s="16"/>
-      <c r="T71" s="16"/>
-      <c r="U71" s="16"/>
+      <c r="Q71" s="9"/>
+      <c r="R71" s="9"/>
+      <c r="S71" s="9"/>
+      <c r="T71" s="9"/>
+      <c r="U71" s="9"/>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="15" t="s">
+      <c r="A72" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="B72" s="15"/>
-      <c r="C72" s="16" t="n">
+      <c r="B72" s="4"/>
+      <c r="C72" s="9" t="n">
         <v>2</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="E72" s="16" t="s">
+      <c r="E72" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F72" s="16"/>
-      <c r="G72" s="16"/>
-      <c r="H72" s="16"/>
-      <c r="I72" s="16"/>
-      <c r="J72" s="16"/>
-      <c r="L72" s="15" t="s">
+      <c r="F72" s="9"/>
+      <c r="G72" s="9"/>
+      <c r="H72" s="9"/>
+      <c r="I72" s="9"/>
+      <c r="J72" s="9"/>
+      <c r="L72" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="M72" s="15"/>
-      <c r="N72" s="16"/>
+      <c r="M72" s="4"/>
+      <c r="N72" s="9"/>
       <c r="O72" s="4"/>
-      <c r="P72" s="16"/>
-      <c r="Q72" s="16"/>
-      <c r="R72" s="16"/>
-      <c r="S72" s="16"/>
-      <c r="T72" s="16"/>
-      <c r="U72" s="16"/>
+      <c r="P72" s="9"/>
+      <c r="Q72" s="9"/>
+      <c r="R72" s="9"/>
+      <c r="S72" s="9"/>
+      <c r="T72" s="9"/>
+      <c r="U72" s="9"/>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="18" t="s">
+      <c r="A73" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="B73" s="18"/>
-      <c r="C73" s="16"/>
+      <c r="B73" s="5"/>
+      <c r="C73" s="9"/>
       <c r="D73" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="E73" s="16" t="s">
+      <c r="E73" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F73" s="16"/>
-      <c r="G73" s="16"/>
-      <c r="H73" s="16"/>
-      <c r="I73" s="16"/>
-      <c r="J73" s="16"/>
-      <c r="L73" s="18" t="s">
+      <c r="F73" s="9"/>
+      <c r="G73" s="9"/>
+      <c r="H73" s="9"/>
+      <c r="I73" s="9"/>
+      <c r="J73" s="9"/>
+      <c r="L73" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="M73" s="18"/>
-      <c r="N73" s="16"/>
+      <c r="M73" s="5"/>
+      <c r="N73" s="9"/>
       <c r="O73" s="4"/>
-      <c r="P73" s="16"/>
-      <c r="Q73" s="16"/>
-      <c r="R73" s="16"/>
-      <c r="S73" s="16"/>
-      <c r="T73" s="16"/>
-      <c r="U73" s="16"/>
+      <c r="P73" s="9"/>
+      <c r="Q73" s="9"/>
+      <c r="R73" s="9"/>
+      <c r="S73" s="9"/>
+      <c r="T73" s="9"/>
+      <c r="U73" s="9"/>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C74" s="16"/>
+      <c r="C74" s="9"/>
       <c r="D74" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="E74" s="16" t="s">
+      <c r="E74" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F74" s="16"/>
-      <c r="G74" s="16"/>
-      <c r="H74" s="16"/>
-      <c r="I74" s="16"/>
-      <c r="J74" s="16"/>
-      <c r="N74" s="16"/>
+      <c r="F74" s="9"/>
+      <c r="G74" s="9"/>
+      <c r="H74" s="9"/>
+      <c r="I74" s="9"/>
+      <c r="J74" s="9"/>
+      <c r="N74" s="9"/>
       <c r="O74" s="4"/>
-      <c r="P74" s="16"/>
-      <c r="Q74" s="16"/>
-      <c r="R74" s="16"/>
-      <c r="S74" s="16"/>
-      <c r="T74" s="16"/>
-      <c r="U74" s="16"/>
+      <c r="P74" s="9"/>
+      <c r="Q74" s="9"/>
+      <c r="R74" s="9"/>
+      <c r="S74" s="9"/>
+      <c r="T74" s="9"/>
+      <c r="U74" s="9"/>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C75" s="16"/>
+      <c r="C75" s="9"/>
       <c r="D75" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="E75" s="16" t="s">
+      <c r="E75" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F75" s="16"/>
-      <c r="G75" s="16"/>
-      <c r="H75" s="16"/>
-      <c r="I75" s="16"/>
-      <c r="J75" s="16"/>
-      <c r="N75" s="16"/>
+      <c r="F75" s="9"/>
+      <c r="G75" s="9"/>
+      <c r="H75" s="9"/>
+      <c r="I75" s="9"/>
+      <c r="J75" s="9"/>
+      <c r="N75" s="9"/>
       <c r="O75" s="4"/>
-      <c r="P75" s="16"/>
-      <c r="Q75" s="16"/>
-      <c r="R75" s="16"/>
-      <c r="S75" s="16"/>
-      <c r="T75" s="16"/>
-      <c r="U75" s="16"/>
+      <c r="P75" s="9"/>
+      <c r="Q75" s="9"/>
+      <c r="R75" s="9"/>
+      <c r="S75" s="9"/>
+      <c r="T75" s="9"/>
+      <c r="U75" s="9"/>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C76" s="16"/>
+      <c r="C76" s="9"/>
       <c r="D76" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="E76" s="16" t="s">
+      <c r="E76" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F76" s="16"/>
-      <c r="G76" s="16"/>
-      <c r="H76" s="16"/>
-      <c r="I76" s="16"/>
-      <c r="J76" s="16"/>
-      <c r="N76" s="16"/>
+      <c r="F76" s="9"/>
+      <c r="G76" s="9"/>
+      <c r="H76" s="9"/>
+      <c r="I76" s="9"/>
+      <c r="J76" s="9"/>
+      <c r="N76" s="9"/>
       <c r="O76" s="4"/>
-      <c r="P76" s="16"/>
-      <c r="Q76" s="16"/>
-      <c r="R76" s="16"/>
-      <c r="S76" s="16"/>
-      <c r="T76" s="16"/>
-      <c r="U76" s="16"/>
+      <c r="P76" s="9"/>
+      <c r="Q76" s="9"/>
+      <c r="R76" s="9"/>
+      <c r="S76" s="9"/>
+      <c r="T76" s="9"/>
+      <c r="U76" s="9"/>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C77" s="16"/>
+      <c r="C77" s="9"/>
       <c r="D77" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="E77" s="16" t="s">
+      <c r="E77" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F77" s="16"/>
-      <c r="G77" s="16"/>
-      <c r="H77" s="16"/>
-      <c r="I77" s="16"/>
-      <c r="J77" s="16"/>
-      <c r="N77" s="16"/>
+      <c r="F77" s="9"/>
+      <c r="G77" s="9"/>
+      <c r="H77" s="9"/>
+      <c r="I77" s="9"/>
+      <c r="J77" s="9"/>
+      <c r="N77" s="9"/>
       <c r="O77" s="4"/>
-      <c r="P77" s="16"/>
-      <c r="Q77" s="16"/>
-      <c r="R77" s="16"/>
-      <c r="S77" s="16"/>
-      <c r="T77" s="16"/>
-      <c r="U77" s="16"/>
+      <c r="P77" s="9"/>
+      <c r="Q77" s="9"/>
+      <c r="R77" s="9"/>
+      <c r="S77" s="9"/>
+      <c r="T77" s="9"/>
+      <c r="U77" s="9"/>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C78" s="16"/>
+      <c r="C78" s="9"/>
       <c r="D78" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="E78" s="16" t="s">
+      <c r="E78" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F78" s="16"/>
-      <c r="G78" s="16"/>
-      <c r="H78" s="16"/>
-      <c r="I78" s="16"/>
-      <c r="J78" s="16"/>
-      <c r="N78" s="16"/>
+      <c r="F78" s="9"/>
+      <c r="G78" s="9"/>
+      <c r="H78" s="9"/>
+      <c r="I78" s="9"/>
+      <c r="J78" s="9"/>
+      <c r="N78" s="9"/>
       <c r="O78" s="4"/>
-      <c r="P78" s="16"/>
-      <c r="Q78" s="16"/>
-      <c r="R78" s="16"/>
-      <c r="S78" s="16"/>
-      <c r="T78" s="16"/>
-      <c r="U78" s="16"/>
+      <c r="P78" s="9"/>
+      <c r="Q78" s="9"/>
+      <c r="R78" s="9"/>
+      <c r="S78" s="9"/>
+      <c r="T78" s="9"/>
+      <c r="U78" s="9"/>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C79" s="16"/>
+      <c r="C79" s="9"/>
       <c r="D79" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="E79" s="16" t="s">
+      <c r="E79" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F79" s="16"/>
-      <c r="G79" s="16"/>
-      <c r="H79" s="16"/>
-      <c r="I79" s="16"/>
-      <c r="J79" s="16"/>
-      <c r="N79" s="16"/>
+      <c r="F79" s="9"/>
+      <c r="G79" s="9"/>
+      <c r="H79" s="9"/>
+      <c r="I79" s="9"/>
+      <c r="J79" s="9"/>
+      <c r="N79" s="9"/>
       <c r="O79" s="4"/>
-      <c r="P79" s="16"/>
-      <c r="Q79" s="16"/>
-      <c r="R79" s="16"/>
-      <c r="S79" s="16"/>
-      <c r="T79" s="16"/>
-      <c r="U79" s="16"/>
+      <c r="P79" s="9"/>
+      <c r="Q79" s="9"/>
+      <c r="R79" s="9"/>
+      <c r="S79" s="9"/>
+      <c r="T79" s="9"/>
+      <c r="U79" s="9"/>
     </row>
     <row r="81" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="s">
         <v>38</v>
       </c>
       <c r="B81" s="4"/>
-      <c r="C81" s="15" t="s">
+      <c r="C81" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="D81" s="15" t="s">
+      <c r="D81" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="E81" s="15" t="s">
+      <c r="E81" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="F81" s="15"/>
-      <c r="G81" s="15" t="s">
+      <c r="F81" s="4"/>
+      <c r="G81" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="H81" s="15"/>
-      <c r="I81" s="15" t="s">
+      <c r="H81" s="4"/>
+      <c r="I81" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="J81" s="15"/>
-      <c r="L81" s="15" t="s">
+      <c r="J81" s="4"/>
+      <c r="L81" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="M81" s="15"/>
+      <c r="M81" s="4"/>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="16" t="n">
+      <c r="A82" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B82" s="16"/>
-      <c r="C82" s="16" t="n">
+      <c r="B82" s="9"/>
+      <c r="C82" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="E82" s="17" t="s">
+      <c r="E82" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="F82" s="17"/>
-      <c r="G82" s="17" t="s">
+      <c r="F82" s="5"/>
+      <c r="G82" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="H82" s="17"/>
-      <c r="I82" s="17" t="s">
+      <c r="H82" s="5"/>
+      <c r="I82" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="J82" s="17"/>
-      <c r="L82" s="16" t="n">
+      <c r="J82" s="5"/>
+      <c r="L82" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="M82" s="16" t="s">
+      <c r="M82" s="9" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C83" s="16"/>
+      <c r="C83" s="9"/>
       <c r="D83" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="E83" s="17"/>
-      <c r="F83" s="17"/>
-      <c r="G83" s="17"/>
-      <c r="H83" s="17"/>
-      <c r="I83" s="17"/>
-      <c r="J83" s="17"/>
-      <c r="L83" s="16" t="n">
+      <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
+      <c r="G83" s="5"/>
+      <c r="H83" s="5"/>
+      <c r="I83" s="5"/>
+      <c r="J83" s="5"/>
+      <c r="L83" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="M83" s="16" t="s">
+      <c r="M83" s="9" t="s">
         <v>188</v>
       </c>
     </row>
@@ -4757,206 +4730,206 @@
         <v>160</v>
       </c>
       <c r="B84" s="4"/>
-      <c r="C84" s="16"/>
+      <c r="C84" s="9"/>
       <c r="D84" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="E84" s="17"/>
-      <c r="F84" s="17"/>
-      <c r="G84" s="17"/>
-      <c r="H84" s="17"/>
-      <c r="I84" s="17"/>
-      <c r="J84" s="17"/>
-      <c r="L84" s="16" t="n">
+      <c r="E84" s="5"/>
+      <c r="F84" s="5"/>
+      <c r="G84" s="5"/>
+      <c r="H84" s="5"/>
+      <c r="I84" s="5"/>
+      <c r="J84" s="5"/>
+      <c r="L84" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="M84" s="16" t="s">
+      <c r="M84" s="9" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="18" t="s">
+      <c r="A85" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B85" s="18"/>
-      <c r="C85" s="16"/>
+      <c r="B85" s="5"/>
+      <c r="C85" s="9"/>
       <c r="D85" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="E85" s="17"/>
-      <c r="F85" s="17"/>
-      <c r="G85" s="17"/>
-      <c r="H85" s="17"/>
-      <c r="I85" s="17"/>
-      <c r="J85" s="17"/>
-      <c r="L85" s="16" t="n">
+      <c r="E85" s="5"/>
+      <c r="F85" s="5"/>
+      <c r="G85" s="5"/>
+      <c r="H85" s="5"/>
+      <c r="I85" s="5"/>
+      <c r="J85" s="5"/>
+      <c r="L85" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="M85" s="16" t="s">
+      <c r="M85" s="9" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C86" s="16"/>
+      <c r="C86" s="9"/>
       <c r="D86" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="E86" s="17" t="s">
+      <c r="E86" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="F86" s="17"/>
-      <c r="G86" s="17" t="s">
+      <c r="F86" s="5"/>
+      <c r="G86" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="H86" s="17"/>
-      <c r="I86" s="17" t="s">
+      <c r="H86" s="5"/>
+      <c r="I86" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="J86" s="17"/>
-      <c r="L86" s="16" t="n">
+      <c r="J86" s="5"/>
+      <c r="L86" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="M86" s="16" t="s">
+      <c r="M86" s="9" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="15" t="s">
+      <c r="A87" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B87" s="15"/>
-      <c r="C87" s="16"/>
+      <c r="B87" s="4"/>
+      <c r="C87" s="9"/>
       <c r="D87" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="E87" s="17"/>
-      <c r="F87" s="17"/>
-      <c r="G87" s="17"/>
-      <c r="H87" s="17"/>
-      <c r="I87" s="17"/>
-      <c r="J87" s="17"/>
-      <c r="L87" s="16" t="n">
+      <c r="E87" s="5"/>
+      <c r="F87" s="5"/>
+      <c r="G87" s="5"/>
+      <c r="H87" s="5"/>
+      <c r="I87" s="5"/>
+      <c r="J87" s="5"/>
+      <c r="L87" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="M87" s="16" t="s">
+      <c r="M87" s="9" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="18" t="s">
+      <c r="A88" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="B88" s="18"/>
-      <c r="C88" s="16"/>
+      <c r="B88" s="5"/>
+      <c r="C88" s="9"/>
       <c r="D88" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="E88" s="16"/>
-      <c r="F88" s="16"/>
-      <c r="G88" s="16"/>
-      <c r="H88" s="16"/>
-      <c r="I88" s="16"/>
-      <c r="J88" s="16"/>
+      <c r="E88" s="9"/>
+      <c r="F88" s="9"/>
+      <c r="G88" s="9"/>
+      <c r="H88" s="9"/>
+      <c r="I88" s="9"/>
+      <c r="J88" s="9"/>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C89" s="16"/>
+      <c r="C89" s="9"/>
       <c r="D89" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="E89" s="16"/>
-      <c r="F89" s="16"/>
-      <c r="G89" s="16"/>
-      <c r="H89" s="16"/>
-      <c r="I89" s="16"/>
-      <c r="J89" s="16"/>
+      <c r="E89" s="9"/>
+      <c r="F89" s="9"/>
+      <c r="G89" s="9"/>
+      <c r="H89" s="9"/>
+      <c r="I89" s="9"/>
+      <c r="J89" s="9"/>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="15" t="s">
+      <c r="A90" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="B90" s="15"/>
-      <c r="C90" s="16"/>
+      <c r="B90" s="4"/>
+      <c r="C90" s="9"/>
       <c r="D90" s="4"/>
-      <c r="E90" s="16"/>
-      <c r="F90" s="16"/>
-      <c r="G90" s="16"/>
-      <c r="H90" s="16"/>
-      <c r="I90" s="16"/>
-      <c r="J90" s="16"/>
+      <c r="E90" s="9"/>
+      <c r="F90" s="9"/>
+      <c r="G90" s="9"/>
+      <c r="H90" s="9"/>
+      <c r="I90" s="9"/>
+      <c r="J90" s="9"/>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="18" t="s">
+      <c r="A91" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="B91" s="18"/>
-      <c r="C91" s="16"/>
+      <c r="B91" s="5"/>
+      <c r="C91" s="9"/>
       <c r="D91" s="4"/>
-      <c r="E91" s="16"/>
-      <c r="F91" s="16"/>
-      <c r="G91" s="16"/>
-      <c r="H91" s="16"/>
-      <c r="I91" s="16"/>
-      <c r="J91" s="16"/>
+      <c r="E91" s="9"/>
+      <c r="F91" s="9"/>
+      <c r="G91" s="9"/>
+      <c r="H91" s="9"/>
+      <c r="I91" s="9"/>
+      <c r="J91" s="9"/>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C92" s="16"/>
+      <c r="C92" s="9"/>
       <c r="D92" s="4"/>
-      <c r="E92" s="16"/>
-      <c r="F92" s="16"/>
-      <c r="G92" s="16"/>
-      <c r="H92" s="16"/>
-      <c r="I92" s="16"/>
-      <c r="J92" s="16"/>
+      <c r="E92" s="9"/>
+      <c r="F92" s="9"/>
+      <c r="G92" s="9"/>
+      <c r="H92" s="9"/>
+      <c r="I92" s="9"/>
+      <c r="J92" s="9"/>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C93" s="16"/>
+      <c r="C93" s="9"/>
       <c r="D93" s="4"/>
-      <c r="E93" s="16"/>
-      <c r="F93" s="16"/>
-      <c r="G93" s="16"/>
-      <c r="H93" s="16"/>
-      <c r="I93" s="16"/>
-      <c r="J93" s="16"/>
+      <c r="E93" s="9"/>
+      <c r="F93" s="9"/>
+      <c r="G93" s="9"/>
+      <c r="H93" s="9"/>
+      <c r="I93" s="9"/>
+      <c r="J93" s="9"/>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C94" s="16"/>
+      <c r="C94" s="9"/>
       <c r="D94" s="4"/>
-      <c r="E94" s="16"/>
-      <c r="F94" s="16"/>
-      <c r="G94" s="16"/>
-      <c r="H94" s="16"/>
-      <c r="I94" s="16"/>
-      <c r="J94" s="16"/>
+      <c r="E94" s="9"/>
+      <c r="F94" s="9"/>
+      <c r="G94" s="9"/>
+      <c r="H94" s="9"/>
+      <c r="I94" s="9"/>
+      <c r="J94" s="9"/>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C95" s="16"/>
+      <c r="C95" s="9"/>
       <c r="D95" s="4"/>
-      <c r="E95" s="16"/>
-      <c r="F95" s="16"/>
-      <c r="G95" s="16"/>
-      <c r="H95" s="16"/>
-      <c r="I95" s="16"/>
-      <c r="J95" s="16"/>
+      <c r="E95" s="9"/>
+      <c r="F95" s="9"/>
+      <c r="G95" s="9"/>
+      <c r="H95" s="9"/>
+      <c r="I95" s="9"/>
+      <c r="J95" s="9"/>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C96" s="16"/>
+      <c r="C96" s="9"/>
       <c r="D96" s="4"/>
-      <c r="E96" s="16"/>
-      <c r="F96" s="16"/>
-      <c r="G96" s="16"/>
-      <c r="H96" s="16"/>
-      <c r="I96" s="16"/>
-      <c r="J96" s="16"/>
+      <c r="E96" s="9"/>
+      <c r="F96" s="9"/>
+      <c r="G96" s="9"/>
+      <c r="H96" s="9"/>
+      <c r="I96" s="9"/>
+      <c r="J96" s="9"/>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C97" s="16"/>
+      <c r="C97" s="9"/>
       <c r="D97" s="4"/>
-      <c r="E97" s="16"/>
-      <c r="F97" s="16"/>
-      <c r="G97" s="16"/>
-      <c r="H97" s="16"/>
-      <c r="I97" s="16"/>
-      <c r="J97" s="16"/>
+      <c r="E97" s="9"/>
+      <c r="F97" s="9"/>
+      <c r="G97" s="9"/>
+      <c r="H97" s="9"/>
+      <c r="I97" s="9"/>
+      <c r="J97" s="9"/>
     </row>
     <row r="98" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="2"/>
@@ -5036,70 +5009,70 @@
       <c r="A101" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B101" s="19"/>
+      <c r="B101" s="15"/>
       <c r="C101" s="9"/>
       <c r="D101" s="5" t="s">
         <v>201</v>
       </c>
       <c r="E101" s="5"/>
       <c r="F101" s="5"/>
-      <c r="H101" s="20" t="s">
+      <c r="H101" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="I101" s="21"/>
-      <c r="J101" s="22" t="s">
+      <c r="I101" s="17"/>
+      <c r="J101" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="K101" s="21"/>
-      <c r="L101" s="23" t="s">
+      <c r="K101" s="17"/>
+      <c r="L101" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="M101" s="21"/>
-      <c r="N101" s="24" t="s">
+      <c r="M101" s="17"/>
+      <c r="N101" s="20" t="s">
         <v>203</v>
       </c>
-      <c r="O101" s="21"/>
+      <c r="O101" s="17"/>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B102" s="19"/>
-      <c r="C102" s="19"/>
+      <c r="B102" s="15"/>
+      <c r="C102" s="15"/>
       <c r="D102" s="5" t="s">
         <v>204</v>
       </c>
       <c r="E102" s="5"/>
       <c r="F102" s="5"/>
-      <c r="H102" s="20" t="s">
+      <c r="H102" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="I102" s="25"/>
-      <c r="J102" s="22" t="s">
+      <c r="I102" s="21"/>
+      <c r="J102" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="K102" s="26"/>
-      <c r="L102" s="23" t="s">
+      <c r="K102" s="22"/>
+      <c r="L102" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="M102" s="27"/>
-      <c r="N102" s="24" t="s">
+      <c r="M102" s="23"/>
+      <c r="N102" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="O102" s="28"/>
+      <c r="O102" s="24"/>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B103" s="29"/>
+      <c r="B103" s="25"/>
       <c r="C103" s="9"/>
       <c r="D103" s="5" t="s">
         <v>201</v>
       </c>
       <c r="E103" s="5"/>
       <c r="F103" s="5"/>
-      <c r="O103" s="30" t="s">
+      <c r="O103" s="26" t="s">
         <v>206</v>
       </c>
     </row>
@@ -5107,38 +5080,38 @@
       <c r="A104" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B104" s="29"/>
-      <c r="C104" s="29"/>
+      <c r="B104" s="25"/>
+      <c r="C104" s="25"/>
       <c r="D104" s="5" t="s">
         <v>205</v>
       </c>
       <c r="E104" s="5"/>
       <c r="F104" s="5"/>
-      <c r="H104" s="31"/>
-      <c r="I104" s="32"/>
-      <c r="J104" s="32"/>
-      <c r="K104" s="31"/>
+      <c r="H104" s="27"/>
+      <c r="I104" s="28"/>
+      <c r="J104" s="28"/>
+      <c r="K104" s="27"/>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B105" s="33"/>
+      <c r="B105" s="29"/>
       <c r="C105" s="9"/>
       <c r="D105" s="5" t="s">
         <v>202</v>
       </c>
       <c r="E105" s="5"/>
       <c r="F105" s="5"/>
-      <c r="I105" s="32"/>
-      <c r="J105" s="32"/>
+      <c r="I105" s="28"/>
+      <c r="J105" s="28"/>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B106" s="33"/>
-      <c r="C106" s="33"/>
+      <c r="B106" s="29"/>
+      <c r="C106" s="29"/>
       <c r="D106" s="5" t="s">
         <v>49</v>
       </c>
@@ -5149,7 +5122,7 @@
       <c r="A107" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B107" s="34"/>
+      <c r="B107" s="30"/>
       <c r="C107" s="9"/>
       <c r="D107" s="5" t="s">
         <v>203</v>
@@ -5161,8 +5134,8 @@
       <c r="A108" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B108" s="34"/>
-      <c r="C108" s="34"/>
+      <c r="B108" s="30"/>
+      <c r="C108" s="30"/>
       <c r="D108" s="5" t="s">
         <v>49</v>
       </c>
@@ -5505,38 +5478,38 @@
       <c r="K119" s="4"/>
       <c r="L119" s="4"/>
       <c r="M119" s="4"/>
-      <c r="N119" s="35" t="s">
+      <c r="N119" s="31" t="s">
         <v>173</v>
       </c>
-      <c r="O119" s="35"/>
-      <c r="P119" s="35" t="s">
+      <c r="O119" s="31"/>
+      <c r="P119" s="31" t="s">
         <v>172</v>
       </c>
-      <c r="Q119" s="35"/>
-      <c r="R119" s="35" t="s">
+      <c r="Q119" s="31"/>
+      <c r="R119" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="S119" s="35"/>
-      <c r="T119" s="35" t="s">
+      <c r="S119" s="31"/>
+      <c r="T119" s="31" t="s">
         <v>163</v>
       </c>
-      <c r="U119" s="35"/>
-      <c r="V119" s="35" t="s">
+      <c r="U119" s="31"/>
+      <c r="V119" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="W119" s="35"/>
-      <c r="X119" s="35" t="s">
+      <c r="W119" s="31"/>
+      <c r="X119" s="31" t="s">
         <v>161</v>
       </c>
-      <c r="Y119" s="35"/>
-      <c r="Z119" s="35" t="s">
+      <c r="Y119" s="31"/>
+      <c r="Z119" s="31" t="s">
         <v>159</v>
       </c>
-      <c r="AA119" s="35"/>
-      <c r="AB119" s="35" t="s">
+      <c r="AA119" s="31"/>
+      <c r="AB119" s="31" t="s">
         <v>154</v>
       </c>
-      <c r="AC119" s="35"/>
+      <c r="AC119" s="31"/>
     </row>
     <row r="120" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="9" t="n">
@@ -6028,870 +6001,870 @@
   <dimension ref="A1:AH39"/>
   <sheetFormatPr defaultColWidth="6.48828125" defaultRowHeight="36" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="31" width="6.49"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="27" width="6.49"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="36"/>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="36"/>
-      <c r="T1" s="36"/>
-      <c r="U1" s="36"/>
-      <c r="V1" s="36"/>
-      <c r="W1" s="36"/>
+      <c r="A1" s="32"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+      <c r="O1" s="32"/>
+      <c r="P1" s="32"/>
+      <c r="Q1" s="32"/>
+      <c r="R1" s="32"/>
+      <c r="S1" s="32"/>
+      <c r="T1" s="32"/>
+      <c r="U1" s="32"/>
+      <c r="V1" s="32"/>
+      <c r="W1" s="32"/>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="36"/>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
-      <c r="T2" s="36"/>
-      <c r="U2" s="36"/>
-      <c r="V2" s="36"/>
-      <c r="W2" s="36"/>
+      <c r="A2" s="32"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
+      <c r="R2" s="32"/>
+      <c r="S2" s="32"/>
+      <c r="T2" s="32"/>
+      <c r="U2" s="32"/>
+      <c r="V2" s="32"/>
+      <c r="W2" s="32"/>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="36"/>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
-      <c r="M3" s="36"/>
-      <c r="N3" s="36"/>
-      <c r="O3" s="36"/>
-      <c r="P3" s="36"/>
-      <c r="Q3" s="36"/>
-      <c r="R3" s="36"/>
-      <c r="S3" s="36"/>
-      <c r="T3" s="36"/>
-      <c r="U3" s="36"/>
-      <c r="V3" s="36"/>
-      <c r="W3" s="36"/>
+      <c r="A3" s="32"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="32"/>
+      <c r="M3" s="32"/>
+      <c r="N3" s="32"/>
+      <c r="O3" s="32"/>
+      <c r="P3" s="32"/>
+      <c r="Q3" s="32"/>
+      <c r="R3" s="32"/>
+      <c r="S3" s="32"/>
+      <c r="T3" s="32"/>
+      <c r="U3" s="32"/>
+      <c r="V3" s="32"/>
+      <c r="W3" s="32"/>
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="36"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36"/>
-      <c r="O4" s="36"/>
-      <c r="P4" s="36"/>
-      <c r="Q4" s="36"/>
-      <c r="R4" s="36"/>
-      <c r="S4" s="36"/>
-      <c r="T4" s="36"/>
-      <c r="U4" s="36"/>
-      <c r="V4" s="36"/>
-      <c r="W4" s="36"/>
+      <c r="A4" s="32"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="32"/>
+      <c r="M4" s="32"/>
+      <c r="N4" s="32"/>
+      <c r="O4" s="32"/>
+      <c r="P4" s="32"/>
+      <c r="Q4" s="32"/>
+      <c r="R4" s="32"/>
+      <c r="S4" s="32"/>
+      <c r="T4" s="32"/>
+      <c r="U4" s="32"/>
+      <c r="V4" s="32"/>
+      <c r="W4" s="32"/>
     </row>
     <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="36"/>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
-      <c r="L5" s="36"/>
-      <c r="M5" s="36"/>
-      <c r="N5" s="36"/>
-      <c r="O5" s="36"/>
-      <c r="P5" s="36"/>
-      <c r="Q5" s="36"/>
-      <c r="R5" s="36"/>
-      <c r="S5" s="36"/>
-      <c r="T5" s="36"/>
-      <c r="U5" s="36"/>
-      <c r="V5" s="36"/>
-      <c r="W5" s="36"/>
+      <c r="A5" s="32"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="32"/>
+      <c r="N5" s="32"/>
+      <c r="O5" s="32"/>
+      <c r="P5" s="32"/>
+      <c r="Q5" s="32"/>
+      <c r="R5" s="32"/>
+      <c r="S5" s="32"/>
+      <c r="T5" s="32"/>
+      <c r="U5" s="32"/>
+      <c r="V5" s="32"/>
+      <c r="W5" s="32"/>
     </row>
     <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="36"/>
-      <c r="B6" s="36"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="36"/>
-      <c r="I6" s="36"/>
-      <c r="J6" s="36"/>
-      <c r="K6" s="36"/>
-      <c r="L6" s="36"/>
-      <c r="M6" s="36"/>
-      <c r="N6" s="36"/>
-      <c r="O6" s="36"/>
-      <c r="P6" s="36"/>
-      <c r="Q6" s="36"/>
-      <c r="R6" s="36"/>
-      <c r="S6" s="36"/>
-      <c r="T6" s="36"/>
-      <c r="U6" s="36"/>
-      <c r="V6" s="36"/>
-      <c r="W6" s="36"/>
+      <c r="A6" s="32"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="32"/>
+      <c r="N6" s="32"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="32"/>
+      <c r="Q6" s="32"/>
+      <c r="R6" s="32"/>
+      <c r="S6" s="32"/>
+      <c r="T6" s="32"/>
+      <c r="U6" s="32"/>
+      <c r="V6" s="32"/>
+      <c r="W6" s="32"/>
     </row>
     <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="36"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="36"/>
-      <c r="K7" s="36"/>
-      <c r="L7" s="36"/>
-      <c r="M7" s="36"/>
-      <c r="N7" s="36"/>
-      <c r="O7" s="36"/>
-      <c r="P7" s="36"/>
-      <c r="Q7" s="36"/>
-      <c r="R7" s="36"/>
-      <c r="S7" s="36"/>
-      <c r="T7" s="36"/>
-      <c r="U7" s="36"/>
-      <c r="V7" s="36"/>
-      <c r="W7" s="36"/>
+      <c r="A7" s="32"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
+      <c r="L7" s="32"/>
+      <c r="M7" s="32"/>
+      <c r="N7" s="32"/>
+      <c r="O7" s="32"/>
+      <c r="P7" s="32"/>
+      <c r="Q7" s="32"/>
+      <c r="R7" s="32"/>
+      <c r="S7" s="32"/>
+      <c r="T7" s="32"/>
+      <c r="U7" s="32"/>
+      <c r="V7" s="32"/>
+      <c r="W7" s="32"/>
     </row>
     <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="36"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="36"/>
-      <c r="J8" s="36"/>
-      <c r="K8" s="36"/>
-      <c r="L8" s="36"/>
-      <c r="M8" s="36"/>
-      <c r="N8" s="36"/>
-      <c r="O8" s="36"/>
-      <c r="P8" s="36"/>
-      <c r="Q8" s="36"/>
-      <c r="R8" s="36"/>
-      <c r="S8" s="36"/>
-      <c r="T8" s="36"/>
-      <c r="U8" s="36"/>
-      <c r="V8" s="36"/>
-      <c r="W8" s="36"/>
+      <c r="A8" s="32"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="32"/>
+      <c r="K8" s="32"/>
+      <c r="L8" s="32"/>
+      <c r="M8" s="32"/>
+      <c r="N8" s="32"/>
+      <c r="O8" s="32"/>
+      <c r="P8" s="32"/>
+      <c r="Q8" s="32"/>
+      <c r="R8" s="32"/>
+      <c r="S8" s="32"/>
+      <c r="T8" s="32"/>
+      <c r="U8" s="32"/>
+      <c r="V8" s="32"/>
+      <c r="W8" s="32"/>
     </row>
     <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="36"/>
-      <c r="K9" s="36"/>
-      <c r="L9" s="36"/>
-      <c r="M9" s="36"/>
-      <c r="N9" s="36"/>
-      <c r="O9" s="36"/>
-      <c r="P9" s="36"/>
-      <c r="Q9" s="36"/>
-      <c r="R9" s="36"/>
-      <c r="S9" s="36"/>
-      <c r="T9" s="36"/>
-      <c r="U9" s="36"/>
-      <c r="V9" s="36"/>
-      <c r="W9" s="36"/>
+      <c r="A9" s="32"/>
+      <c r="B9" s="32"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="32"/>
+      <c r="K9" s="32"/>
+      <c r="L9" s="32"/>
+      <c r="M9" s="32"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="32"/>
+      <c r="P9" s="32"/>
+      <c r="Q9" s="32"/>
+      <c r="R9" s="32"/>
+      <c r="S9" s="32"/>
+      <c r="T9" s="32"/>
+      <c r="U9" s="32"/>
+      <c r="V9" s="32"/>
+      <c r="W9" s="32"/>
     </row>
     <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36"/>
-      <c r="B10" s="36"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="38"/>
-      <c r="I10" s="38"/>
-      <c r="J10" s="38"/>
-      <c r="K10" s="38"/>
-      <c r="L10" s="38"/>
-      <c r="M10" s="38"/>
-      <c r="N10" s="38"/>
-      <c r="O10" s="38"/>
-      <c r="P10" s="38"/>
-      <c r="Q10" s="38"/>
-      <c r="R10" s="38"/>
-      <c r="S10" s="38"/>
-      <c r="T10" s="38"/>
-      <c r="U10" s="38"/>
-      <c r="V10" s="38"/>
-      <c r="W10" s="39"/>
+      <c r="A10" s="32"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="34"/>
+      <c r="K10" s="34"/>
+      <c r="L10" s="34"/>
+      <c r="M10" s="34"/>
+      <c r="N10" s="34"/>
+      <c r="O10" s="34"/>
+      <c r="P10" s="34"/>
+      <c r="Q10" s="34"/>
+      <c r="R10" s="34"/>
+      <c r="S10" s="34"/>
+      <c r="T10" s="34"/>
+      <c r="U10" s="34"/>
+      <c r="V10" s="34"/>
+      <c r="W10" s="35"/>
     </row>
     <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36"/>
-      <c r="B11" s="36"/>
-      <c r="C11" s="40"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="41" t="s">
+      <c r="A11" s="32"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="37" t="s">
         <v>218</v>
       </c>
-      <c r="F11" s="41"/>
-      <c r="G11" s="36"/>
-      <c r="H11" s="36"/>
-      <c r="I11" s="36"/>
-      <c r="J11" s="36"/>
-      <c r="K11" s="36"/>
-      <c r="L11" s="36"/>
-      <c r="M11" s="36"/>
-      <c r="N11" s="36"/>
-      <c r="O11" s="36"/>
-      <c r="P11" s="36"/>
-      <c r="Q11" s="36"/>
-      <c r="R11" s="36"/>
-      <c r="S11" s="36"/>
-      <c r="T11" s="36"/>
-      <c r="U11" s="36"/>
-      <c r="V11" s="36"/>
-      <c r="W11" s="42"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="32"/>
+      <c r="L11" s="32"/>
+      <c r="M11" s="32"/>
+      <c r="N11" s="32"/>
+      <c r="O11" s="32"/>
+      <c r="P11" s="32"/>
+      <c r="Q11" s="32"/>
+      <c r="R11" s="32"/>
+      <c r="S11" s="32"/>
+      <c r="T11" s="32"/>
+      <c r="U11" s="32"/>
+      <c r="V11" s="32"/>
+      <c r="W11" s="38"/>
     </row>
     <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36"/>
-      <c r="B12" s="36"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="36"/>
-      <c r="H12" s="36"/>
-      <c r="I12" s="36"/>
-      <c r="J12" s="36"/>
-      <c r="K12" s="36"/>
-      <c r="L12" s="36"/>
-      <c r="M12" s="36"/>
-      <c r="N12" s="36"/>
-      <c r="O12" s="36"/>
-      <c r="P12" s="36"/>
-      <c r="Q12" s="36"/>
-      <c r="R12" s="36"/>
-      <c r="S12" s="36"/>
-      <c r="T12" s="36"/>
-      <c r="U12" s="36"/>
-      <c r="V12" s="36"/>
-      <c r="W12" s="42"/>
+      <c r="A12" s="32"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="32"/>
+      <c r="K12" s="32"/>
+      <c r="L12" s="32"/>
+      <c r="M12" s="32"/>
+      <c r="N12" s="32"/>
+      <c r="O12" s="32"/>
+      <c r="P12" s="32"/>
+      <c r="Q12" s="32"/>
+      <c r="R12" s="32"/>
+      <c r="S12" s="32"/>
+      <c r="T12" s="32"/>
+      <c r="U12" s="32"/>
+      <c r="V12" s="32"/>
+      <c r="W12" s="38"/>
     </row>
     <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36"/>
-      <c r="B13" s="36"/>
-      <c r="C13" s="40"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="36"/>
-      <c r="H13" s="36"/>
-      <c r="I13" s="36"/>
-      <c r="J13" s="36"/>
-      <c r="K13" s="36"/>
-      <c r="L13" s="36"/>
-      <c r="M13" s="36"/>
-      <c r="N13" s="36"/>
-      <c r="O13" s="36"/>
-      <c r="P13" s="36"/>
-      <c r="Q13" s="36"/>
-      <c r="R13" s="36"/>
-      <c r="S13" s="36"/>
-      <c r="T13" s="36"/>
-      <c r="U13" s="36"/>
-      <c r="V13" s="36"/>
-      <c r="W13" s="42"/>
+      <c r="A13" s="32"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+      <c r="L13" s="32"/>
+      <c r="M13" s="32"/>
+      <c r="N13" s="32"/>
+      <c r="O13" s="32"/>
+      <c r="P13" s="32"/>
+      <c r="Q13" s="32"/>
+      <c r="R13" s="32"/>
+      <c r="S13" s="32"/>
+      <c r="T13" s="32"/>
+      <c r="U13" s="32"/>
+      <c r="V13" s="32"/>
+      <c r="W13" s="38"/>
     </row>
     <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36"/>
-      <c r="B14" s="36"/>
-      <c r="C14" s="40"/>
-      <c r="D14" s="45" t="s">
+      <c r="A14" s="32"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="41" t="s">
         <v>219</v>
       </c>
-      <c r="E14" s="46" t="s">
+      <c r="E14" s="42" t="s">
         <v>220</v>
       </c>
-      <c r="F14" s="47" t="s">
+      <c r="F14" s="43" t="s">
         <v>220</v>
       </c>
-      <c r="G14" s="36"/>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="36"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="36"/>
-      <c r="O14" s="36"/>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="36"/>
-      <c r="R14" s="36"/>
-      <c r="S14" s="36"/>
-      <c r="T14" s="36"/>
-      <c r="U14" s="36"/>
-      <c r="V14" s="36"/>
-      <c r="W14" s="42"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="32"/>
+      <c r="L14" s="32"/>
+      <c r="M14" s="32"/>
+      <c r="N14" s="32"/>
+      <c r="O14" s="32"/>
+      <c r="P14" s="32"/>
+      <c r="Q14" s="32"/>
+      <c r="R14" s="32"/>
+      <c r="S14" s="32"/>
+      <c r="T14" s="32"/>
+      <c r="U14" s="32"/>
+      <c r="V14" s="32"/>
+      <c r="W14" s="38"/>
     </row>
     <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="36"/>
-      <c r="B15" s="36"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="48" t="s">
+      <c r="A15" s="32"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="44" t="s">
         <v>220</v>
       </c>
-      <c r="F15" s="49" t="s">
+      <c r="F15" s="45" t="s">
         <v>220</v>
       </c>
-      <c r="G15" s="36"/>
-      <c r="H15" s="36"/>
-      <c r="I15" s="36"/>
-      <c r="J15" s="36"/>
-      <c r="K15" s="36"/>
-      <c r="L15" s="36"/>
-      <c r="M15" s="36"/>
-      <c r="N15" s="36"/>
-      <c r="O15" s="36"/>
-      <c r="P15" s="36"/>
-      <c r="Q15" s="36"/>
-      <c r="R15" s="36"/>
-      <c r="S15" s="36"/>
-      <c r="T15" s="36"/>
-      <c r="U15" s="36"/>
-      <c r="V15" s="36"/>
-      <c r="W15" s="42"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32"/>
+      <c r="K15" s="32"/>
+      <c r="L15" s="32"/>
+      <c r="M15" s="32"/>
+      <c r="N15" s="32"/>
+      <c r="O15" s="32"/>
+      <c r="P15" s="32"/>
+      <c r="Q15" s="32"/>
+      <c r="R15" s="32"/>
+      <c r="S15" s="32"/>
+      <c r="T15" s="32"/>
+      <c r="U15" s="32"/>
+      <c r="V15" s="32"/>
+      <c r="W15" s="38"/>
     </row>
     <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="36"/>
-      <c r="B16" s="36"/>
-      <c r="C16" s="40"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="50" t="s">
+      <c r="A16" s="32"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="46" t="s">
         <v>220</v>
       </c>
-      <c r="F16" s="51" t="s">
+      <c r="F16" s="47" t="s">
         <v>220</v>
       </c>
-      <c r="G16" s="36"/>
-      <c r="H16" s="36"/>
-      <c r="I16" s="36"/>
-      <c r="J16" s="36"/>
-      <c r="K16" s="36"/>
-      <c r="L16" s="36"/>
-      <c r="M16" s="36"/>
-      <c r="N16" s="36"/>
-      <c r="O16" s="36"/>
-      <c r="P16" s="36"/>
-      <c r="Q16" s="36"/>
-      <c r="R16" s="52" t="s">
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="32"/>
+      <c r="L16" s="32"/>
+      <c r="M16" s="32"/>
+      <c r="N16" s="32"/>
+      <c r="O16" s="32"/>
+      <c r="P16" s="32"/>
+      <c r="Q16" s="32"/>
+      <c r="R16" s="48" t="s">
         <v>221</v>
       </c>
-      <c r="S16" s="52"/>
-      <c r="T16" s="52"/>
-      <c r="U16" s="52"/>
-      <c r="V16" s="36"/>
-      <c r="W16" s="42"/>
+      <c r="S16" s="48"/>
+      <c r="T16" s="48"/>
+      <c r="U16" s="48"/>
+      <c r="V16" s="32"/>
+      <c r="W16" s="38"/>
     </row>
     <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="36"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="53" t="s">
+      <c r="B17" s="32"/>
+      <c r="C17" s="36"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="49" t="s">
         <v>220</v>
       </c>
-      <c r="F17" s="54" t="s">
+      <c r="F17" s="50" t="s">
         <v>220</v>
       </c>
-      <c r="G17" s="36"/>
-      <c r="H17" s="36"/>
-      <c r="I17" s="36"/>
-      <c r="J17" s="36"/>
-      <c r="K17" s="36"/>
-      <c r="L17" s="36"/>
-      <c r="M17" s="36"/>
-      <c r="N17" s="36"/>
-      <c r="O17" s="36"/>
-      <c r="P17" s="36"/>
-      <c r="Q17" s="36"/>
-      <c r="R17" s="36"/>
-      <c r="S17" s="36"/>
-      <c r="T17" s="36"/>
-      <c r="U17" s="36"/>
-      <c r="V17" s="36"/>
-      <c r="W17" s="42"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="32"/>
+      <c r="L17" s="32"/>
+      <c r="M17" s="32"/>
+      <c r="N17" s="32"/>
+      <c r="O17" s="32"/>
+      <c r="P17" s="32"/>
+      <c r="Q17" s="32"/>
+      <c r="R17" s="32"/>
+      <c r="S17" s="32"/>
+      <c r="T17" s="32"/>
+      <c r="U17" s="32"/>
+      <c r="V17" s="32"/>
+      <c r="W17" s="38"/>
     </row>
     <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="36"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="36"/>
-      <c r="K18" s="36"/>
-      <c r="L18" s="36"/>
-      <c r="M18" s="36"/>
-      <c r="N18" s="36"/>
-      <c r="O18" s="36"/>
-      <c r="P18" s="36"/>
-      <c r="Q18" s="36"/>
-      <c r="R18" s="36"/>
-      <c r="S18" s="36"/>
-      <c r="T18" s="36"/>
-      <c r="U18" s="36"/>
-      <c r="V18" s="36"/>
-      <c r="W18" s="42"/>
+      <c r="B18" s="32"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="32"/>
+      <c r="K18" s="32"/>
+      <c r="L18" s="32"/>
+      <c r="M18" s="32"/>
+      <c r="N18" s="32"/>
+      <c r="O18" s="32"/>
+      <c r="P18" s="32"/>
+      <c r="Q18" s="32"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="38"/>
     </row>
     <row r="19" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="36"/>
-      <c r="C19" s="40"/>
-      <c r="D19" s="45" t="s">
+      <c r="B19" s="32"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="41" t="s">
         <v>222</v>
       </c>
-      <c r="E19" s="53" t="s">
+      <c r="E19" s="49" t="s">
         <v>220</v>
       </c>
-      <c r="F19" s="54" t="s">
+      <c r="F19" s="50" t="s">
         <v>220</v>
       </c>
-      <c r="G19" s="36"/>
-      <c r="H19" s="36"/>
-      <c r="I19" s="36"/>
-      <c r="J19" s="36"/>
-      <c r="K19" s="36"/>
-      <c r="L19" s="36"/>
-      <c r="M19" s="36"/>
-      <c r="N19" s="36"/>
-      <c r="O19" s="36"/>
-      <c r="P19" s="36"/>
-      <c r="Q19" s="36"/>
-      <c r="R19" s="36"/>
-      <c r="S19" s="36"/>
-      <c r="T19" s="36"/>
-      <c r="U19" s="36"/>
-      <c r="V19" s="36"/>
-      <c r="W19" s="42"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+      <c r="L19" s="32"/>
+      <c r="M19" s="32"/>
+      <c r="N19" s="32"/>
+      <c r="O19" s="32"/>
+      <c r="P19" s="32"/>
+      <c r="Q19" s="32"/>
+      <c r="R19" s="32"/>
+      <c r="S19" s="32"/>
+      <c r="T19" s="32"/>
+      <c r="U19" s="32"/>
+      <c r="V19" s="32"/>
+      <c r="W19" s="38"/>
     </row>
     <row r="20" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C20" s="55"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="50" t="s">
+      <c r="C20" s="51"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="46" t="s">
         <v>220</v>
       </c>
-      <c r="F20" s="51" t="s">
+      <c r="F20" s="47" t="s">
         <v>220</v>
       </c>
-      <c r="W20" s="56"/>
+      <c r="W20" s="52"/>
     </row>
     <row r="21" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="36"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="48" t="s">
+      <c r="B21" s="32"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="44" t="s">
         <v>220</v>
       </c>
-      <c r="F21" s="49" t="s">
+      <c r="F21" s="45" t="s">
         <v>220</v>
       </c>
-      <c r="G21" s="36"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="36"/>
-      <c r="K21" s="36"/>
-      <c r="L21" s="36"/>
-      <c r="M21" s="36"/>
-      <c r="N21" s="36"/>
-      <c r="O21" s="36"/>
-      <c r="P21" s="36"/>
-      <c r="Q21" s="36"/>
-      <c r="R21" s="36"/>
-      <c r="S21" s="36"/>
-      <c r="U21" s="57"/>
-      <c r="V21" s="58" t="s">
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+      <c r="L21" s="32"/>
+      <c r="M21" s="32"/>
+      <c r="N21" s="32"/>
+      <c r="O21" s="32"/>
+      <c r="P21" s="32"/>
+      <c r="Q21" s="32"/>
+      <c r="R21" s="32"/>
+      <c r="S21" s="32"/>
+      <c r="U21" s="53"/>
+      <c r="V21" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="W21" s="56"/>
-      <c r="X21" s="36"/>
+      <c r="W21" s="52"/>
+      <c r="X21" s="32"/>
     </row>
     <row r="22" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="40"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="46" t="s">
+      <c r="C22" s="36"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="42" t="s">
         <v>220</v>
       </c>
-      <c r="F22" s="47" t="s">
+      <c r="F22" s="43" t="s">
         <v>220</v>
       </c>
-      <c r="G22" s="59"/>
-      <c r="H22" s="59"/>
-      <c r="I22" s="59"/>
-      <c r="J22" s="59"/>
-      <c r="K22" s="59"/>
-      <c r="L22" s="59"/>
-      <c r="M22" s="59"/>
-      <c r="N22" s="59"/>
-      <c r="O22" s="59"/>
-      <c r="P22" s="59"/>
-      <c r="Q22" s="59"/>
-      <c r="R22" s="59"/>
-      <c r="S22" s="59"/>
-      <c r="T22" s="59"/>
-      <c r="U22" s="60"/>
-      <c r="V22" s="58"/>
-      <c r="W22" s="56"/>
-      <c r="X22" s="36"/>
+      <c r="G22" s="55"/>
+      <c r="H22" s="55"/>
+      <c r="I22" s="55"/>
+      <c r="J22" s="55"/>
+      <c r="K22" s="55"/>
+      <c r="L22" s="55"/>
+      <c r="M22" s="55"/>
+      <c r="N22" s="55"/>
+      <c r="O22" s="55"/>
+      <c r="P22" s="55"/>
+      <c r="Q22" s="55"/>
+      <c r="R22" s="55"/>
+      <c r="S22" s="55"/>
+      <c r="T22" s="55"/>
+      <c r="U22" s="56"/>
+      <c r="V22" s="54"/>
+      <c r="W22" s="52"/>
+      <c r="X22" s="32"/>
     </row>
     <row r="23" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C23" s="40"/>
-      <c r="L23" s="61" t="s">
+      <c r="C23" s="36"/>
+      <c r="L23" s="57" t="s">
         <v>223</v>
       </c>
-      <c r="U23" s="36"/>
-      <c r="V23" s="36"/>
-      <c r="W23" s="56"/>
-      <c r="X23" s="36"/>
+      <c r="U23" s="32"/>
+      <c r="V23" s="32"/>
+      <c r="W23" s="52"/>
+      <c r="X23" s="32"/>
     </row>
     <row r="24" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C24" s="40"/>
-      <c r="I24" s="36"/>
-      <c r="J24" s="36"/>
-      <c r="K24" s="36"/>
-      <c r="L24" s="62" t="s">
+      <c r="C24" s="36"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="32"/>
+      <c r="L24" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="M24" s="63"/>
-      <c r="N24" s="63"/>
-      <c r="O24" s="63"/>
-      <c r="P24" s="63"/>
-      <c r="Q24" s="64"/>
-      <c r="V24" s="36"/>
-      <c r="W24" s="56"/>
-      <c r="X24" s="36"/>
+      <c r="M24" s="59"/>
+      <c r="N24" s="59"/>
+      <c r="O24" s="59"/>
+      <c r="P24" s="59"/>
+      <c r="Q24" s="60"/>
+      <c r="V24" s="32"/>
+      <c r="W24" s="52"/>
+      <c r="X24" s="32"/>
     </row>
     <row r="25" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C25" s="40"/>
-      <c r="I25" s="36"/>
-      <c r="J25" s="36"/>
-      <c r="K25" s="36"/>
-      <c r="L25" s="65" t="s">
+      <c r="C25" s="36"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+      <c r="L25" s="61" t="s">
         <v>224</v>
       </c>
-      <c r="M25" s="66"/>
-      <c r="N25" s="66"/>
-      <c r="O25" s="66"/>
-      <c r="P25" s="66"/>
-      <c r="Q25" s="67"/>
-      <c r="S25" s="36"/>
-      <c r="U25" s="57"/>
-      <c r="V25" s="58" t="s">
+      <c r="M25" s="62"/>
+      <c r="N25" s="62"/>
+      <c r="O25" s="62"/>
+      <c r="P25" s="62"/>
+      <c r="Q25" s="63"/>
+      <c r="S25" s="32"/>
+      <c r="U25" s="53"/>
+      <c r="V25" s="54" t="s">
         <v>44</v>
       </c>
-      <c r="W25" s="56"/>
-      <c r="X25" s="36"/>
+      <c r="W25" s="52"/>
+      <c r="X25" s="32"/>
     </row>
     <row r="26" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C26" s="40"/>
-      <c r="I26" s="36"/>
-      <c r="J26" s="36"/>
-      <c r="K26" s="36"/>
-      <c r="L26" s="68"/>
-      <c r="M26" s="69"/>
-      <c r="N26" s="69"/>
-      <c r="O26" s="69"/>
-      <c r="P26" s="69"/>
-      <c r="Q26" s="70" t="s">
+      <c r="C26" s="36"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="32"/>
+      <c r="K26" s="32"/>
+      <c r="L26" s="64"/>
+      <c r="M26" s="65"/>
+      <c r="N26" s="65"/>
+      <c r="O26" s="65"/>
+      <c r="P26" s="65"/>
+      <c r="Q26" s="66" t="s">
         <v>49</v>
       </c>
-      <c r="S26" s="36"/>
-      <c r="U26" s="71"/>
-      <c r="V26" s="58"/>
-      <c r="W26" s="56"/>
-      <c r="X26" s="36"/>
+      <c r="S26" s="32"/>
+      <c r="U26" s="67"/>
+      <c r="V26" s="54"/>
+      <c r="W26" s="52"/>
+      <c r="X26" s="32"/>
     </row>
     <row r="27" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="40"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="36"/>
-      <c r="I27" s="36"/>
-      <c r="L27" s="72" t="s">
+      <c r="C27" s="36"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="L27" s="68" t="s">
         <v>225</v>
       </c>
-      <c r="M27" s="72"/>
-      <c r="N27" s="72"/>
-      <c r="V27" s="36"/>
-      <c r="W27" s="56"/>
-      <c r="X27" s="36"/>
+      <c r="M27" s="68"/>
+      <c r="N27" s="68"/>
+      <c r="V27" s="32"/>
+      <c r="W27" s="52"/>
+      <c r="X27" s="32"/>
     </row>
     <row r="28" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="40"/>
-      <c r="G28" s="72" t="s">
+      <c r="C28" s="36"/>
+      <c r="G28" s="68" t="s">
         <v>226</v>
       </c>
-      <c r="H28" s="72"/>
-      <c r="I28" s="72"/>
-      <c r="L28" s="73" t="s">
+      <c r="H28" s="68"/>
+      <c r="I28" s="68"/>
+      <c r="L28" s="69" t="s">
         <v>49</v>
       </c>
-      <c r="M28" s="74"/>
-      <c r="N28" s="75"/>
-      <c r="V28" s="36"/>
-      <c r="W28" s="56"/>
-      <c r="X28" s="36"/>
-      <c r="AF28" s="36"/>
-      <c r="AG28" s="36"/>
-      <c r="AH28" s="36"/>
+      <c r="M28" s="70"/>
+      <c r="N28" s="71"/>
+      <c r="V28" s="32"/>
+      <c r="W28" s="52"/>
+      <c r="X28" s="32"/>
+      <c r="AF28" s="32"/>
+      <c r="AG28" s="32"/>
+      <c r="AH28" s="32"/>
     </row>
     <row r="29" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C29" s="40"/>
-      <c r="G29" s="76"/>
-      <c r="H29" s="77"/>
-      <c r="I29" s="78" t="s">
+      <c r="C29" s="36"/>
+      <c r="G29" s="72"/>
+      <c r="H29" s="73"/>
+      <c r="I29" s="74" t="s">
         <v>227</v>
       </c>
-      <c r="L29" s="79"/>
-      <c r="M29" s="80"/>
-      <c r="N29" s="81" t="s">
+      <c r="L29" s="75"/>
+      <c r="M29" s="76"/>
+      <c r="N29" s="77" t="s">
         <v>228</v>
       </c>
-      <c r="V29" s="36"/>
-      <c r="W29" s="56"/>
-      <c r="X29" s="36"/>
+      <c r="V29" s="32"/>
+      <c r="W29" s="52"/>
+      <c r="X29" s="32"/>
     </row>
     <row r="30" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C30" s="40"/>
-      <c r="G30" s="82"/>
-      <c r="H30" s="83"/>
-      <c r="I30" s="84"/>
-      <c r="L30" s="72" t="s">
+      <c r="C30" s="36"/>
+      <c r="G30" s="78"/>
+      <c r="H30" s="79"/>
+      <c r="I30" s="80"/>
+      <c r="L30" s="68" t="s">
         <v>229</v>
       </c>
-      <c r="M30" s="72"/>
-      <c r="N30" s="72"/>
-      <c r="R30" s="52" t="s">
+      <c r="M30" s="68"/>
+      <c r="N30" s="68"/>
+      <c r="R30" s="48" t="s">
         <v>230</v>
       </c>
-      <c r="S30" s="52"/>
-      <c r="T30" s="52"/>
-      <c r="V30" s="36"/>
-      <c r="W30" s="56"/>
-      <c r="X30" s="36"/>
+      <c r="S30" s="48"/>
+      <c r="T30" s="48"/>
+      <c r="V30" s="32"/>
+      <c r="W30" s="52"/>
+      <c r="X30" s="32"/>
     </row>
     <row r="31" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="40"/>
-      <c r="D31" s="45" t="s">
+      <c r="C31" s="36"/>
+      <c r="D31" s="41" t="s">
         <v>231</v>
       </c>
-      <c r="E31" s="85"/>
-      <c r="G31" s="82" t="s">
+      <c r="E31" s="81"/>
+      <c r="G31" s="78" t="s">
         <v>232</v>
       </c>
-      <c r="H31" s="83"/>
-      <c r="I31" s="84" t="s">
+      <c r="H31" s="79"/>
+      <c r="I31" s="80" t="s">
         <v>233</v>
       </c>
-      <c r="L31" s="73" t="s">
+      <c r="L31" s="69" t="s">
         <v>49</v>
       </c>
-      <c r="M31" s="74"/>
-      <c r="N31" s="75"/>
-      <c r="V31" s="36"/>
-      <c r="W31" s="56"/>
-      <c r="X31" s="36"/>
+      <c r="M31" s="70"/>
+      <c r="N31" s="71"/>
+      <c r="V31" s="32"/>
+      <c r="W31" s="52"/>
+      <c r="X31" s="32"/>
     </row>
     <row r="32" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="40"/>
-      <c r="D32" s="45"/>
-      <c r="E32" s="86"/>
-      <c r="G32" s="82" t="s">
+      <c r="C32" s="36"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="82"/>
+      <c r="G32" s="78" t="s">
         <v>234</v>
       </c>
-      <c r="H32" s="83"/>
-      <c r="I32" s="84" t="s">
+      <c r="H32" s="79"/>
+      <c r="I32" s="80" t="s">
         <v>235</v>
       </c>
-      <c r="L32" s="79"/>
-      <c r="M32" s="80"/>
-      <c r="N32" s="81" t="s">
+      <c r="L32" s="75"/>
+      <c r="M32" s="76"/>
+      <c r="N32" s="77" t="s">
         <v>228</v>
       </c>
-      <c r="V32" s="36"/>
-      <c r="W32" s="56"/>
-      <c r="X32" s="36"/>
+      <c r="V32" s="32"/>
+      <c r="W32" s="52"/>
+      <c r="X32" s="32"/>
     </row>
     <row r="33" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="40"/>
-      <c r="G33" s="82" t="s">
+      <c r="C33" s="36"/>
+      <c r="G33" s="78" t="s">
         <v>49</v>
       </c>
-      <c r="H33" s="83"/>
-      <c r="I33" s="84" t="s">
+      <c r="H33" s="79"/>
+      <c r="I33" s="80" t="s">
         <v>49</v>
       </c>
-      <c r="L33" s="72" t="s">
+      <c r="L33" s="68" t="s">
         <v>236</v>
       </c>
-      <c r="M33" s="72"/>
-      <c r="N33" s="72"/>
-      <c r="S33" s="87"/>
-      <c r="T33" s="88"/>
-      <c r="U33" s="44"/>
-      <c r="V33" s="89" t="s">
+      <c r="M33" s="68"/>
+      <c r="N33" s="68"/>
+      <c r="S33" s="83"/>
+      <c r="T33" s="84"/>
+      <c r="U33" s="40"/>
+      <c r="V33" s="85" t="s">
         <v>237</v>
       </c>
-      <c r="W33" s="56"/>
-      <c r="X33" s="36"/>
+      <c r="W33" s="52"/>
+      <c r="X33" s="32"/>
     </row>
     <row r="34" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="40"/>
-      <c r="G34" s="90" t="s">
+      <c r="C34" s="36"/>
+      <c r="G34" s="86" t="s">
         <v>238</v>
       </c>
-      <c r="H34" s="91"/>
-      <c r="I34" s="92"/>
-      <c r="L34" s="73"/>
-      <c r="M34" s="75" t="s">
+      <c r="H34" s="87"/>
+      <c r="I34" s="88"/>
+      <c r="L34" s="69"/>
+      <c r="M34" s="71" t="s">
         <v>228</v>
       </c>
-      <c r="S34" s="87"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="44"/>
-      <c r="V34" s="89" t="s">
+      <c r="S34" s="83"/>
+      <c r="T34" s="84"/>
+      <c r="U34" s="40"/>
+      <c r="V34" s="85" t="s">
         <v>239</v>
       </c>
-      <c r="W34" s="56"/>
-      <c r="X34" s="36"/>
+      <c r="W34" s="52"/>
+      <c r="X34" s="32"/>
     </row>
     <row r="35" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C35" s="40"/>
-      <c r="L35" s="93"/>
-      <c r="M35" s="94"/>
-      <c r="S35" s="87"/>
-      <c r="T35" s="88"/>
-      <c r="U35" s="44"/>
-      <c r="V35" s="89" t="s">
+      <c r="C35" s="36"/>
+      <c r="L35" s="89"/>
+      <c r="M35" s="90"/>
+      <c r="S35" s="83"/>
+      <c r="T35" s="84"/>
+      <c r="U35" s="40"/>
+      <c r="V35" s="85" t="s">
         <v>240</v>
       </c>
-      <c r="W35" s="56"/>
-      <c r="X35" s="36"/>
+      <c r="W35" s="52"/>
+      <c r="X35" s="32"/>
     </row>
     <row r="36" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C36" s="40"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="44"/>
-      <c r="L36" s="79" t="s">
+      <c r="C36" s="36"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="40"/>
+      <c r="L36" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="M36" s="81"/>
-      <c r="P36" s="43"/>
-      <c r="Q36" s="44"/>
-      <c r="S36" s="87"/>
-      <c r="T36" s="88"/>
-      <c r="U36" s="44"/>
-      <c r="V36" s="89" t="s">
+      <c r="M36" s="77"/>
+      <c r="P36" s="39"/>
+      <c r="Q36" s="40"/>
+      <c r="S36" s="83"/>
+      <c r="T36" s="84"/>
+      <c r="U36" s="40"/>
+      <c r="V36" s="85" t="s">
         <v>241</v>
       </c>
-      <c r="W36" s="56"/>
-      <c r="X36" s="36"/>
+      <c r="W36" s="52"/>
+      <c r="X36" s="32"/>
     </row>
     <row r="37" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C37" s="55"/>
-      <c r="E37" s="41" t="s">
+      <c r="C37" s="51"/>
+      <c r="E37" s="37" t="s">
         <v>242</v>
       </c>
-      <c r="F37" s="41"/>
-      <c r="P37" s="41" t="s">
+      <c r="F37" s="37"/>
+      <c r="P37" s="37" t="s">
         <v>243</v>
       </c>
-      <c r="Q37" s="41"/>
-      <c r="V37" s="36"/>
-      <c r="W37" s="56"/>
-      <c r="X37" s="36"/>
+      <c r="Q37" s="37"/>
+      <c r="V37" s="32"/>
+      <c r="W37" s="52"/>
+      <c r="X37" s="32"/>
     </row>
     <row r="38" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C38" s="95"/>
-      <c r="D38" s="96"/>
-      <c r="E38" s="96"/>
-      <c r="F38" s="96"/>
-      <c r="G38" s="96"/>
-      <c r="H38" s="96"/>
-      <c r="I38" s="96"/>
-      <c r="J38" s="96"/>
-      <c r="K38" s="96"/>
-      <c r="L38" s="96"/>
-      <c r="M38" s="96"/>
-      <c r="N38" s="96"/>
-      <c r="O38" s="96"/>
-      <c r="P38" s="96"/>
-      <c r="Q38" s="96"/>
-      <c r="R38" s="96"/>
-      <c r="S38" s="96"/>
-      <c r="T38" s="96"/>
-      <c r="U38" s="96"/>
-      <c r="V38" s="96"/>
-      <c r="W38" s="97"/>
-      <c r="X38" s="36"/>
+      <c r="C38" s="91"/>
+      <c r="D38" s="92"/>
+      <c r="E38" s="92"/>
+      <c r="F38" s="92"/>
+      <c r="G38" s="92"/>
+      <c r="H38" s="92"/>
+      <c r="I38" s="92"/>
+      <c r="J38" s="92"/>
+      <c r="K38" s="92"/>
+      <c r="L38" s="92"/>
+      <c r="M38" s="92"/>
+      <c r="N38" s="92"/>
+      <c r="O38" s="92"/>
+      <c r="P38" s="92"/>
+      <c r="Q38" s="92"/>
+      <c r="R38" s="92"/>
+      <c r="S38" s="92"/>
+      <c r="T38" s="92"/>
+      <c r="U38" s="92"/>
+      <c r="V38" s="92"/>
+      <c r="W38" s="93"/>
+      <c r="X38" s="32"/>
     </row>
     <row r="39" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="X39" s="36"/>
+      <c r="X39" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>

<commit_message>
[ Version 0.0.31.2 ] - FSM code was writen.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="247">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -429,16 +429,16 @@
     <t xml:space="preserve">Dataset structure which store drainage vent runtime properties.</t>
   </si>
   <si>
-    <t xml:space="preserve">v1_opn_tick</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v1_cls_tick</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v2_opn_tick</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v2_cls_tick</t>
+    <t xml:space="preserve">v1_opn_ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v1_cls_ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v2_opn_ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v2_cls_ms</t>
   </si>
   <si>
     <t xml:space="preserve">v1_opn_duty</t>
@@ -588,10 +588,19 @@
     <t xml:space="preserve">IDLE</t>
   </si>
   <si>
+    <t xml:space="preserve">OFF</t>
+  </si>
+  <si>
     <t xml:space="preserve">START 1</t>
   </si>
   <si>
+    <t xml:space="preserve">OPEN</t>
+  </si>
+  <si>
     <t xml:space="preserve">MOVING 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLOSE</t>
   </si>
   <si>
     <t xml:space="preserve">START 2</t>
@@ -3803,7 +3812,7 @@
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
       <c r="H50" s="5" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="I50" s="5"/>
       <c r="J50" s="5"/>
@@ -3830,7 +3839,7 @@
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
       <c r="H51" s="5" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="I51" s="5"/>
       <c r="J51" s="5"/>
@@ -3857,7 +3866,7 @@
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
       <c r="H52" s="5" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="I52" s="5"/>
       <c r="J52" s="5"/>
@@ -3884,7 +3893,7 @@
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
       <c r="H53" s="5" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="I53" s="5"/>
       <c r="J53" s="5"/>
@@ -4676,6 +4685,10 @@
         <v>183</v>
       </c>
       <c r="M81" s="4"/>
+      <c r="O81" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="P81" s="4"/>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="9" t="n">
@@ -4705,6 +4718,12 @@
       </c>
       <c r="M82" s="9" t="s">
         <v>187</v>
+      </c>
+      <c r="O82" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P82" s="9" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4722,7 +4741,13 @@
         <v>1</v>
       </c>
       <c r="M83" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
+      </c>
+      <c r="O83" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="P83" s="9" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4744,7 +4769,13 @@
         <v>2</v>
       </c>
       <c r="M84" s="9" t="s">
-        <v>189</v>
+        <v>191</v>
+      </c>
+      <c r="O84" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="P84" s="9" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4766,7 +4797,13 @@
         <v>3</v>
       </c>
       <c r="M85" s="9" t="s">
-        <v>190</v>
+        <v>193</v>
+      </c>
+      <c r="O85" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="P85" s="9" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4775,22 +4812,22 @@
         <v>163</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="F86" s="5"/>
       <c r="G86" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="H86" s="5"/>
       <c r="I86" s="5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="J86" s="5"/>
       <c r="L86" s="9" t="n">
         <v>4</v>
       </c>
       <c r="M86" s="9" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4812,7 +4849,7 @@
         <v>5</v>
       </c>
       <c r="M87" s="9" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4824,7 +4861,9 @@
       <c r="D88" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="E88" s="9"/>
+      <c r="E88" s="9" t="s">
+        <v>155</v>
+      </c>
       <c r="F88" s="9"/>
       <c r="G88" s="9"/>
       <c r="H88" s="9"/>
@@ -4836,7 +4875,9 @@
       <c r="D89" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="E89" s="9"/>
+      <c r="E89" s="9" t="s">
+        <v>155</v>
+      </c>
       <c r="F89" s="9"/>
       <c r="G89" s="9"/>
       <c r="H89" s="9"/>
@@ -4956,7 +4997,7 @@
     </row>
     <row r="99" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B99" s="6"/>
       <c r="C99" s="6"/>
@@ -4981,13 +5022,13 @@
     </row>
     <row r="100" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D100" s="4" t="s">
         <v>41</v>
@@ -4995,7 +5036,7 @@
       <c r="E100" s="4"/>
       <c r="F100" s="4"/>
       <c r="H100" s="4" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="I100" s="4"/>
       <c r="J100" s="4"/>
@@ -5012,24 +5053,24 @@
       <c r="B101" s="15"/>
       <c r="C101" s="9"/>
       <c r="D101" s="5" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="E101" s="5"/>
       <c r="F101" s="5"/>
       <c r="H101" s="16" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="I101" s="17"/>
       <c r="J101" s="18" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="K101" s="17"/>
       <c r="L101" s="19" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="M101" s="17"/>
       <c r="N101" s="20" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="O101" s="17"/>
     </row>
@@ -5040,16 +5081,16 @@
       <c r="B102" s="15"/>
       <c r="C102" s="15"/>
       <c r="D102" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E102" s="5"/>
       <c r="F102" s="5"/>
       <c r="H102" s="16" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="I102" s="21"/>
       <c r="J102" s="18" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="K102" s="22"/>
       <c r="L102" s="19" t="s">
@@ -5068,12 +5109,12 @@
       <c r="B103" s="25"/>
       <c r="C103" s="9"/>
       <c r="D103" s="5" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="E103" s="5"/>
       <c r="F103" s="5"/>
       <c r="O103" s="26" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5083,7 +5124,7 @@
       <c r="B104" s="25"/>
       <c r="C104" s="25"/>
       <c r="D104" s="5" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="E104" s="5"/>
       <c r="F104" s="5"/>
@@ -5099,7 +5140,7 @@
       <c r="B105" s="29"/>
       <c r="C105" s="9"/>
       <c r="D105" s="5" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="E105" s="5"/>
       <c r="F105" s="5"/>
@@ -5125,7 +5166,7 @@
       <c r="B107" s="30"/>
       <c r="C107" s="9"/>
       <c r="D107" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="E107" s="5"/>
       <c r="F107" s="5"/>
@@ -5255,7 +5296,7 @@
         <v>1</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C113" s="5"/>
       <c r="D113" s="5"/>
@@ -5265,7 +5306,7 @@
       <c r="F113" s="5"/>
       <c r="G113" s="5"/>
       <c r="H113" s="5" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="I113" s="5" t="s">
         <v>103</v>
@@ -5274,7 +5315,7 @@
         <v>103</v>
       </c>
       <c r="K113" s="5" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="L113" s="5" t="s">
         <v>103</v>
@@ -5283,7 +5324,7 @@
         <v>103</v>
       </c>
       <c r="N113" s="5" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="O113" s="5"/>
       <c r="P113" s="5"/>
@@ -5311,7 +5352,7 @@
         <v>103</v>
       </c>
       <c r="K114" s="5" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="L114" s="5" t="s">
         <v>103</v>
@@ -5346,7 +5387,7 @@
         <v>103</v>
       </c>
       <c r="K115" s="5" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="L115" s="5" t="s">
         <v>103</v>
@@ -5434,17 +5475,17 @@
       <c r="F118" s="4"/>
       <c r="G118" s="4"/>
       <c r="H118" s="4" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="I118" s="4"/>
       <c r="J118" s="4"/>
       <c r="K118" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="L118" s="4"/>
       <c r="M118" s="4"/>
       <c r="N118" s="4" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="O118" s="4"/>
       <c r="P118" s="4"/>
@@ -5460,7 +5501,7 @@
       <c r="Z118" s="4"/>
       <c r="AA118" s="4"/>
       <c r="AB118" s="4" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="AC118" s="4"/>
     </row>
@@ -5516,7 +5557,7 @@
         <v>1</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C120" s="5" t="s">
         <v>103</v>
@@ -5525,7 +5566,7 @@
         <v>103</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F120" s="5" t="s">
         <v>103</v>
@@ -5560,7 +5601,7 @@
       <c r="V120" s="5"/>
       <c r="W120" s="5"/>
       <c r="X120" s="5" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="Y120" s="5"/>
       <c r="Z120" s="5" t="s">
@@ -5594,7 +5635,7 @@
       <c r="U121" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="386">
+  <mergeCells count="387">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -5880,6 +5921,7 @@
     <mergeCell ref="G81:H81"/>
     <mergeCell ref="I81:J81"/>
     <mergeCell ref="L81:M81"/>
+    <mergeCell ref="O81:P81"/>
     <mergeCell ref="A82:B82"/>
     <mergeCell ref="C82:C89"/>
     <mergeCell ref="E82:F85"/>
@@ -6260,7 +6302,7 @@
       <c r="C11" s="36"/>
       <c r="D11" s="32"/>
       <c r="E11" s="37" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F11" s="37"/>
       <c r="G11" s="32"/>
@@ -6336,13 +6378,13 @@
       <c r="B14" s="32"/>
       <c r="C14" s="36"/>
       <c r="D14" s="41" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E14" s="42" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F14" s="43" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="G14" s="32"/>
       <c r="H14" s="32"/>
@@ -6368,10 +6410,10 @@
       <c r="C15" s="36"/>
       <c r="D15" s="41"/>
       <c r="E15" s="44" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F15" s="45" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="G15" s="32"/>
       <c r="H15" s="32"/>
@@ -6397,10 +6439,10 @@
       <c r="C16" s="36"/>
       <c r="D16" s="41"/>
       <c r="E16" s="46" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F16" s="47" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="G16" s="32"/>
       <c r="H16" s="32"/>
@@ -6414,7 +6456,7 @@
       <c r="P16" s="32"/>
       <c r="Q16" s="32"/>
       <c r="R16" s="48" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="S16" s="48"/>
       <c r="T16" s="48"/>
@@ -6427,10 +6469,10 @@
       <c r="C17" s="36"/>
       <c r="D17" s="41"/>
       <c r="E17" s="49" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F17" s="50" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="G17" s="32"/>
       <c r="H17" s="32"/>
@@ -6478,13 +6520,13 @@
       <c r="B19" s="32"/>
       <c r="C19" s="36"/>
       <c r="D19" s="41" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E19" s="49" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F19" s="50" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="G19" s="32"/>
       <c r="H19" s="32"/>
@@ -6508,10 +6550,10 @@
       <c r="C20" s="51"/>
       <c r="D20" s="41"/>
       <c r="E20" s="46" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F20" s="47" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="W20" s="52"/>
     </row>
@@ -6520,10 +6562,10 @@
       <c r="C21" s="36"/>
       <c r="D21" s="41"/>
       <c r="E21" s="44" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F21" s="45" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="G21" s="32"/>
       <c r="H21" s="32"/>
@@ -6549,10 +6591,10 @@
       <c r="C22" s="36"/>
       <c r="D22" s="41"/>
       <c r="E22" s="42" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F22" s="43" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="G22" s="55"/>
       <c r="H22" s="55"/>
@@ -6576,7 +6618,7 @@
     <row r="23" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C23" s="36"/>
       <c r="L23" s="57" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="U23" s="32"/>
       <c r="V23" s="32"/>
@@ -6606,7 +6648,7 @@
       <c r="J25" s="32"/>
       <c r="K25" s="32"/>
       <c r="L25" s="61" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M25" s="62"/>
       <c r="N25" s="62"/>
@@ -6646,7 +6688,7 @@
       <c r="H27" s="32"/>
       <c r="I27" s="32"/>
       <c r="L27" s="68" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="M27" s="68"/>
       <c r="N27" s="68"/>
@@ -6657,7 +6699,7 @@
     <row r="28" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="36"/>
       <c r="G28" s="68" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="H28" s="68"/>
       <c r="I28" s="68"/>
@@ -6678,12 +6720,12 @@
       <c r="G29" s="72"/>
       <c r="H29" s="73"/>
       <c r="I29" s="74" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="L29" s="75"/>
       <c r="M29" s="76"/>
       <c r="N29" s="77" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="V29" s="32"/>
       <c r="W29" s="52"/>
@@ -6695,12 +6737,12 @@
       <c r="H30" s="79"/>
       <c r="I30" s="80"/>
       <c r="L30" s="68" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="M30" s="68"/>
       <c r="N30" s="68"/>
       <c r="R30" s="48" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="S30" s="48"/>
       <c r="T30" s="48"/>
@@ -6711,15 +6753,15 @@
     <row r="31" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C31" s="36"/>
       <c r="D31" s="41" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E31" s="81"/>
       <c r="G31" s="78" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H31" s="79"/>
       <c r="I31" s="80" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="L31" s="69" t="s">
         <v>49</v>
@@ -6735,16 +6777,16 @@
       <c r="D32" s="41"/>
       <c r="E32" s="82"/>
       <c r="G32" s="78" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="H32" s="79"/>
       <c r="I32" s="80" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="L32" s="75"/>
       <c r="M32" s="76"/>
       <c r="N32" s="77" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="V32" s="32"/>
       <c r="W32" s="52"/>
@@ -6760,7 +6802,7 @@
         <v>49</v>
       </c>
       <c r="L33" s="68" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="M33" s="68"/>
       <c r="N33" s="68"/>
@@ -6768,7 +6810,7 @@
       <c r="T33" s="84"/>
       <c r="U33" s="40"/>
       <c r="V33" s="85" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="W33" s="52"/>
       <c r="X33" s="32"/>
@@ -6776,19 +6818,19 @@
     <row r="34" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="36"/>
       <c r="G34" s="86" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H34" s="87"/>
       <c r="I34" s="88"/>
       <c r="L34" s="69"/>
       <c r="M34" s="71" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="S34" s="83"/>
       <c r="T34" s="84"/>
       <c r="U34" s="40"/>
       <c r="V34" s="85" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="W34" s="52"/>
       <c r="X34" s="32"/>
@@ -6801,7 +6843,7 @@
       <c r="T35" s="84"/>
       <c r="U35" s="40"/>
       <c r="V35" s="85" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="W35" s="52"/>
       <c r="X35" s="32"/>
@@ -6820,7 +6862,7 @@
       <c r="T36" s="84"/>
       <c r="U36" s="40"/>
       <c r="V36" s="85" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="W36" s="52"/>
       <c r="X36" s="32"/>
@@ -6828,11 +6870,11 @@
     <row r="37" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C37" s="51"/>
       <c r="E37" s="37" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="F37" s="37"/>
       <c r="P37" s="37" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="Q37" s="37"/>
       <c r="V37" s="32"/>

</xml_diff>

<commit_message>
[ Version 0.0.32 ] - new GPIO pinout for roulette was created.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="253">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -273,22 +273,40 @@
     <t xml:space="preserve">DO for roulette R1 motor driver direction bit 2 – direction 1.</t>
   </si>
   <si>
-    <t xml:space="preserve">IN_ROULETTE_ESO1</t>
+    <t xml:space="preserve">IN_ROULETTE_TOP1</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO22</t>
   </si>
   <si>
-    <t xml:space="preserve">DI for roulette R1 open position end switches – end switch open 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ROULETTE_ESC1</t>
+    <t xml:space="preserve">DI for roulette R1 open position hall sensors – top 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_TOP2</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO23</t>
   </si>
   <si>
-    <t xml:space="preserve">DI for roulette R1 close position end switches – end switch close 1.</t>
+    <t xml:space="preserve">DI for roulette R1 open position hall sensors – top 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_BOT1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI for roulette R1 close position hall sensors – bottom 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_BOT2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI for roulette R1 close position hall sensors – bottom 2.</t>
   </si>
   <si>
     <t xml:space="preserve">ESP-IDF TIMERS</t>
@@ -2381,7 +2399,7 @@
     <tabColor rgb="FFFDD835"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AC121"/>
+  <dimension ref="A1:AC123"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2957,7 +2975,7 @@
     </row>
     <row r="20" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" s="13" t="s">
         <v>86</v>
@@ -2986,411 +3004,419 @@
       <c r="T20" s="13"/>
       <c r="U20" s="13"/>
     </row>
-    <row r="21" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="2"/>
-      <c r="S21" s="2"/>
-      <c r="T21" s="2"/>
-      <c r="U21" s="2"/>
-    </row>
-    <row r="22" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+    <row r="21" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="6"/>
-      <c r="M22" s="6"/>
-      <c r="N22" s="6"/>
-      <c r="O22" s="6"/>
-      <c r="P22" s="6"/>
-      <c r="Q22" s="6"/>
-      <c r="R22" s="6"/>
-      <c r="S22" s="6"/>
-      <c r="T22" s="6"/>
-      <c r="U22" s="6"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="13"/>
+      <c r="N21" s="13"/>
+      <c r="O21" s="13"/>
+      <c r="P21" s="13"/>
+      <c r="Q21" s="13"/>
+      <c r="R21" s="13"/>
+      <c r="S21" s="13"/>
+      <c r="T21" s="13"/>
+      <c r="U21" s="13"/>
+    </row>
+    <row r="22" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="13"/>
+      <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
+      <c r="P22" s="13"/>
+      <c r="Q22" s="13"/>
+      <c r="R22" s="13"/>
+      <c r="S22" s="13"/>
+      <c r="T22" s="13"/>
+      <c r="U22" s="13"/>
     </row>
     <row r="23" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
+      <c r="O23" s="2"/>
+      <c r="P23" s="2"/>
+      <c r="Q23" s="2"/>
+      <c r="R23" s="2"/>
+      <c r="S23" s="2"/>
+      <c r="T23" s="2"/>
+      <c r="U23" s="2"/>
+    </row>
+    <row r="24" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="6"/>
+      <c r="L24" s="6"/>
+      <c r="M24" s="6"/>
+      <c r="N24" s="6"/>
+      <c r="O24" s="6"/>
+      <c r="P24" s="6"/>
+      <c r="Q24" s="6"/>
+      <c r="R24" s="6"/>
+      <c r="S24" s="6"/>
+      <c r="T24" s="6"/>
+      <c r="U24" s="6"/>
+    </row>
+    <row r="25" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B25" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4" t="s">
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4" t="s">
+      <c r="F25" s="4"/>
+      <c r="G25" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
-      <c r="N23" s="4"/>
-      <c r="O23" s="4" t="s">
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="P23" s="4"/>
-      <c r="Q23" s="4"/>
-    </row>
-    <row r="24" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="n">
+      <c r="P25" s="4"/>
+      <c r="Q25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B24" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="11" t="s">
+      <c r="B26" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="11"/>
+      <c r="K26" s="11"/>
+      <c r="L26" s="11"/>
+      <c r="M26" s="11"/>
+      <c r="N26" s="11"/>
+      <c r="O26" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="P24" s="11"/>
-      <c r="Q24" s="11"/>
-    </row>
-    <row r="25" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
-      <c r="R25" s="2"/>
-      <c r="S25" s="2"/>
-      <c r="T25" s="2"/>
-      <c r="U25" s="2"/>
-    </row>
-    <row r="26" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="6"/>
-      <c r="L26" s="6"/>
-      <c r="M26" s="6"/>
-      <c r="N26" s="6"/>
-      <c r="O26" s="6"/>
-      <c r="P26" s="6"/>
-      <c r="Q26" s="6"/>
-      <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
-      <c r="T26" s="6"/>
-      <c r="U26" s="6"/>
+      <c r="P26" s="11"/>
+      <c r="Q26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
+      <c r="L27" s="2"/>
+      <c r="M27" s="2"/>
+      <c r="N27" s="2"/>
+      <c r="O27" s="2"/>
+      <c r="P27" s="2"/>
+      <c r="Q27" s="2"/>
+      <c r="R27" s="2"/>
+      <c r="S27" s="2"/>
+      <c r="T27" s="2"/>
+      <c r="U27" s="2"/>
+    </row>
+    <row r="28" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="6"/>
+      <c r="K28" s="6"/>
+      <c r="L28" s="6"/>
+      <c r="M28" s="6"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="6"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6"/>
+      <c r="R28" s="6"/>
+      <c r="S28" s="6"/>
+      <c r="T28" s="6"/>
+      <c r="U28" s="6"/>
+    </row>
+    <row r="29" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B29" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4" t="s">
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4" t="s">
+      <c r="F29" s="4"/>
+      <c r="G29" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
-      <c r="M27" s="4"/>
-      <c r="N27" s="4"/>
-      <c r="O27" s="4" t="s">
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="P27" s="4"/>
-      <c r="Q27" s="4"/>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="n">
+      <c r="P29" s="4"/>
+      <c r="Q29" s="4"/>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B28" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="H28" s="11"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="11"/>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
-      <c r="N28" s="11"/>
-      <c r="O28" s="11" t="s">
+      <c r="B30" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+      <c r="J30" s="11"/>
+      <c r="K30" s="11"/>
+      <c r="L30" s="11"/>
+      <c r="M30" s="11"/>
+      <c r="N30" s="11"/>
+      <c r="O30" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="P28" s="11"/>
-      <c r="Q28" s="11"/>
-    </row>
-    <row r="29" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2"/>
-      <c r="P29" s="2"/>
-      <c r="Q29" s="2"/>
-      <c r="R29" s="2"/>
-      <c r="S29" s="2"/>
-      <c r="T29" s="2"/>
-      <c r="U29" s="2"/>
-    </row>
-    <row r="30" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="14"/>
-      <c r="J30" s="14"/>
-      <c r="K30" s="14"/>
-      <c r="L30" s="14"/>
-      <c r="M30" s="14"/>
-      <c r="N30" s="14"/>
-      <c r="O30" s="14"/>
-      <c r="P30" s="14"/>
-      <c r="Q30" s="14"/>
-      <c r="R30" s="14"/>
-      <c r="S30" s="14"/>
-      <c r="T30" s="14"/>
-      <c r="U30" s="14"/>
-    </row>
-    <row r="31" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
-      <c r="I31" s="6"/>
-      <c r="J31" s="6"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="6"/>
-      <c r="M31" s="6"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="6"/>
-      <c r="P31" s="6"/>
-      <c r="Q31" s="6"/>
-      <c r="R31" s="6"/>
-      <c r="S31" s="6"/>
-      <c r="T31" s="6"/>
-      <c r="U31" s="6"/>
-    </row>
-    <row r="32" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="P30" s="11"/>
+      <c r="Q30" s="11"/>
+    </row>
+    <row r="31" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+      <c r="L31" s="2"/>
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
+      <c r="O31" s="2"/>
+      <c r="P31" s="2"/>
+      <c r="Q31" s="2"/>
+      <c r="R31" s="2"/>
+      <c r="S31" s="2"/>
+      <c r="T31" s="2"/>
+      <c r="U31" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="I32" s="14"/>
+      <c r="J32" s="14"/>
+      <c r="K32" s="14"/>
+      <c r="L32" s="14"/>
+      <c r="M32" s="14"/>
+      <c r="N32" s="14"/>
+      <c r="O32" s="14"/>
+      <c r="P32" s="14"/>
+      <c r="Q32" s="14"/>
+      <c r="R32" s="14"/>
+      <c r="S32" s="14"/>
+      <c r="T32" s="14"/>
+      <c r="U32" s="14"/>
+    </row>
+    <row r="33" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6"/>
+      <c r="K33" s="6"/>
+      <c r="L33" s="6"/>
+      <c r="M33" s="6"/>
+      <c r="N33" s="6"/>
+      <c r="O33" s="6"/>
+      <c r="P33" s="6"/>
+      <c r="Q33" s="6"/>
+      <c r="R33" s="6"/>
+      <c r="S33" s="6"/>
+      <c r="T33" s="6"/>
+      <c r="U33" s="6"/>
+    </row>
+    <row r="34" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B34" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="L32" s="4"/>
-      <c r="M32" s="4"/>
-      <c r="N32" s="4" t="s">
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="O32" s="4"/>
-      <c r="P32" s="4"/>
-      <c r="Q32" s="4"/>
-      <c r="R32" s="4"/>
-      <c r="S32" s="4"/>
-      <c r="T32" s="4"/>
-      <c r="U32" s="4"/>
-    </row>
-    <row r="33" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="9" t="n">
+      <c r="O34" s="4"/>
+      <c r="P34" s="4"/>
+      <c r="Q34" s="4"/>
+      <c r="R34" s="4"/>
+      <c r="S34" s="4"/>
+      <c r="T34" s="4"/>
+      <c r="U34" s="4"/>
+    </row>
+    <row r="35" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="L33" s="5"/>
-      <c r="M33" s="5"/>
-      <c r="N33" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="O33" s="5"/>
-      <c r="P33" s="5"/>
-      <c r="Q33" s="5"/>
-      <c r="R33" s="5"/>
-      <c r="S33" s="5"/>
-      <c r="T33" s="5"/>
-      <c r="U33" s="5"/>
-    </row>
-    <row r="34" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="9"/>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5" t="s">
+      <c r="B35" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="I34" s="5"/>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="L34" s="5"/>
-      <c r="M34" s="5"/>
-      <c r="N34" s="5"/>
-      <c r="O34" s="5"/>
-      <c r="P34" s="5"/>
-      <c r="Q34" s="5"/>
-      <c r="R34" s="5"/>
-      <c r="S34" s="5"/>
-      <c r="T34" s="5"/>
-      <c r="U34" s="5"/>
-    </row>
-    <row r="35" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="9"/>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
+      <c r="D35" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="F35" s="5"/>
       <c r="G35" s="5"/>
       <c r="H35" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
       <c r="K35" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L35" s="5"/>
       <c r="M35" s="5"/>
-      <c r="N35" s="5"/>
+      <c r="N35" s="5" t="s">
+        <v>113</v>
+      </c>
       <c r="O35" s="5"/>
       <c r="P35" s="5"/>
       <c r="Q35" s="5"/>
@@ -3408,12 +3434,12 @@
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
       <c r="H36" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I36" s="5"/>
       <c r="J36" s="5"/>
       <c r="K36" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="L36" s="5"/>
       <c r="M36" s="5"/>
@@ -3435,12 +3461,12 @@
       <c r="F37" s="5"/>
       <c r="G37" s="5"/>
       <c r="H37" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
       <c r="K37" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="L37" s="5"/>
       <c r="M37" s="5"/>
@@ -3454,30 +3480,24 @@
       <c r="U37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>116</v>
-      </c>
+      <c r="A38" s="9"/>
+      <c r="B38" s="5"/>
       <c r="C38" s="5"/>
       <c r="D38" s="5"/>
       <c r="E38" s="5"/>
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
       <c r="H38" s="5" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
       <c r="K38" s="5" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="L38" s="5"/>
       <c r="M38" s="5"/>
-      <c r="N38" s="5" t="s">
-        <v>117</v>
-      </c>
+      <c r="N38" s="5"/>
       <c r="O38" s="5"/>
       <c r="P38" s="5"/>
       <c r="Q38" s="5"/>
@@ -3495,12 +3515,12 @@
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
       <c r="H39" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
       <c r="K39" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="L39" s="5"/>
       <c r="M39" s="5"/>
@@ -3514,24 +3534,30 @@
       <c r="U39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="9"/>
-      <c r="B40" s="5"/>
+      <c r="A40" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>122</v>
+      </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
       <c r="E40" s="5"/>
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
       <c r="H40" s="5" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
       <c r="K40" s="5" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="L40" s="5"/>
       <c r="M40" s="5"/>
-      <c r="N40" s="5"/>
+      <c r="N40" s="5" t="s">
+        <v>123</v>
+      </c>
       <c r="O40" s="5"/>
       <c r="P40" s="5"/>
       <c r="Q40" s="5"/>
@@ -3549,12 +3575,12 @@
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
       <c r="H41" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
       <c r="K41" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="L41" s="5"/>
       <c r="M41" s="5"/>
@@ -3576,12 +3602,12 @@
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
       <c r="H42" s="5" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
       <c r="K42" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="L42" s="5"/>
       <c r="M42" s="5"/>
@@ -3603,12 +3629,12 @@
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
       <c r="H43" s="5" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
       <c r="K43" s="5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="L43" s="5"/>
       <c r="M43" s="5"/>
@@ -3630,12 +3656,12 @@
       <c r="F44" s="5"/>
       <c r="G44" s="5"/>
       <c r="H44" s="5" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="I44" s="5"/>
       <c r="J44" s="5"/>
       <c r="K44" s="5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L44" s="5"/>
       <c r="M44" s="5"/>
@@ -3649,32 +3675,24 @@
       <c r="U44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>127</v>
-      </c>
+      <c r="A45" s="9"/>
+      <c r="B45" s="5"/>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
-      <c r="E45" s="5" t="s">
-        <v>33</v>
-      </c>
+      <c r="E45" s="5"/>
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
       <c r="H45" s="5" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
       <c r="K45" s="5" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="L45" s="5"/>
       <c r="M45" s="5"/>
-      <c r="N45" s="5" t="s">
-        <v>129</v>
-      </c>
+      <c r="N45" s="5"/>
       <c r="O45" s="5"/>
       <c r="P45" s="5"/>
       <c r="Q45" s="5"/>
@@ -3692,12 +3710,12 @@
       <c r="F46" s="5"/>
       <c r="G46" s="5"/>
       <c r="H46" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
       <c r="K46" s="5" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="L46" s="5"/>
       <c r="M46" s="5"/>
@@ -3711,24 +3729,32 @@
       <c r="U46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="9"/>
-      <c r="B47" s="5"/>
+      <c r="A47" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>133</v>
+      </c>
       <c r="C47" s="5"/>
       <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
+      <c r="E47" s="5" t="s">
+        <v>33</v>
+      </c>
       <c r="F47" s="5"/>
       <c r="G47" s="5"/>
       <c r="H47" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
       <c r="K47" s="5" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="L47" s="5"/>
       <c r="M47" s="5"/>
-      <c r="N47" s="5"/>
+      <c r="N47" s="5" t="s">
+        <v>135</v>
+      </c>
       <c r="O47" s="5"/>
       <c r="P47" s="5"/>
       <c r="Q47" s="5"/>
@@ -3746,12 +3772,12 @@
       <c r="F48" s="5"/>
       <c r="G48" s="5"/>
       <c r="H48" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I48" s="5"/>
       <c r="J48" s="5"/>
       <c r="K48" s="5" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="L48" s="5"/>
       <c r="M48" s="5"/>
@@ -3765,36 +3791,24 @@
       <c r="U48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="E49" s="5" t="s">
-        <v>18</v>
-      </c>
+      <c r="A49" s="9"/>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
       <c r="H49" s="5" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
       <c r="K49" s="5" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="L49" s="5"/>
       <c r="M49" s="5"/>
-      <c r="N49" s="5" t="s">
-        <v>134</v>
-      </c>
+      <c r="N49" s="5"/>
       <c r="O49" s="5"/>
       <c r="P49" s="5"/>
       <c r="Q49" s="5"/>
@@ -3812,12 +3826,12 @@
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
       <c r="H50" s="5" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="I50" s="5"/>
       <c r="J50" s="5"/>
       <c r="K50" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L50" s="5"/>
       <c r="M50" s="5"/>
@@ -3831,24 +3845,36 @@
       <c r="U50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="9"/>
-      <c r="B51" s="5"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
+      <c r="A51" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>18</v>
+      </c>
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
       <c r="H51" s="5" t="s">
-        <v>112</v>
+        <v>138</v>
       </c>
       <c r="I51" s="5"/>
       <c r="J51" s="5"/>
       <c r="K51" s="5" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="L51" s="5"/>
       <c r="M51" s="5"/>
-      <c r="N51" s="5"/>
+      <c r="N51" s="5" t="s">
+        <v>140</v>
+      </c>
       <c r="O51" s="5"/>
       <c r="P51" s="5"/>
       <c r="Q51" s="5"/>
@@ -3866,12 +3892,12 @@
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
       <c r="H52" s="5" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="I52" s="5"/>
       <c r="J52" s="5"/>
       <c r="K52" s="5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="L52" s="5"/>
       <c r="M52" s="5"/>
@@ -3893,12 +3919,12 @@
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
       <c r="H53" s="5" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="I53" s="5"/>
       <c r="J53" s="5"/>
       <c r="K53" s="5" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="L53" s="5"/>
       <c r="M53" s="5"/>
@@ -3920,12 +3946,12 @@
       <c r="F54" s="5"/>
       <c r="G54" s="5"/>
       <c r="H54" s="5" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="I54" s="5"/>
       <c r="J54" s="5"/>
       <c r="K54" s="5" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="L54" s="5"/>
       <c r="M54" s="5"/>
@@ -3947,12 +3973,12 @@
       <c r="F55" s="5"/>
       <c r="G55" s="5"/>
       <c r="H55" s="5" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="I55" s="5"/>
       <c r="J55" s="5"/>
       <c r="K55" s="5" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="L55" s="5"/>
       <c r="M55" s="5"/>
@@ -3974,12 +4000,12 @@
       <c r="F56" s="5"/>
       <c r="G56" s="5"/>
       <c r="H56" s="5" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="I56" s="5"/>
       <c r="J56" s="5"/>
       <c r="K56" s="5" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L56" s="5"/>
       <c r="M56" s="5"/>
@@ -4001,12 +4027,12 @@
       <c r="F57" s="5"/>
       <c r="G57" s="5"/>
       <c r="H57" s="5" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="I57" s="5"/>
       <c r="J57" s="5"/>
       <c r="K57" s="5" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="L57" s="5"/>
       <c r="M57" s="5"/>
@@ -4028,12 +4054,12 @@
       <c r="F58" s="5"/>
       <c r="G58" s="5"/>
       <c r="H58" s="5" t="s">
-        <v>143</v>
+        <v>118</v>
       </c>
       <c r="I58" s="5"/>
       <c r="J58" s="5"/>
       <c r="K58" s="5" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="L58" s="5"/>
       <c r="M58" s="5"/>
@@ -4055,12 +4081,12 @@
       <c r="F59" s="5"/>
       <c r="G59" s="5"/>
       <c r="H59" s="5" t="s">
-        <v>145</v>
+        <v>118</v>
       </c>
       <c r="I59" s="5"/>
       <c r="J59" s="5"/>
       <c r="K59" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="L59" s="5"/>
       <c r="M59" s="5"/>
@@ -4082,12 +4108,12 @@
       <c r="F60" s="5"/>
       <c r="G60" s="5"/>
       <c r="H60" s="5" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="I60" s="5"/>
       <c r="J60" s="5"/>
       <c r="K60" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="L60" s="5"/>
       <c r="M60" s="5"/>
@@ -4100,396 +4126,392 @@
       <c r="T60" s="5"/>
       <c r="U60" s="5"/>
     </row>
-    <row r="61" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
-      <c r="F61" s="2"/>
-      <c r="G61" s="2"/>
-      <c r="H61" s="2"/>
-      <c r="I61" s="2"/>
-      <c r="J61" s="2"/>
-      <c r="K61" s="2"/>
-      <c r="L61" s="2"/>
-      <c r="M61" s="2"/>
-      <c r="N61" s="2"/>
-      <c r="O61" s="2"/>
-      <c r="P61" s="2"/>
-      <c r="Q61" s="2"/>
-      <c r="R61" s="2"/>
-      <c r="S61" s="2"/>
-      <c r="T61" s="2"/>
-      <c r="U61" s="2"/>
-    </row>
-    <row r="62" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="B62" s="6"/>
-      <c r="C62" s="6"/>
-      <c r="D62" s="6"/>
-      <c r="E62" s="6"/>
-      <c r="F62" s="6"/>
-      <c r="G62" s="6"/>
-      <c r="H62" s="6"/>
-      <c r="I62" s="6"/>
-      <c r="J62" s="6"/>
-      <c r="K62" s="6"/>
-      <c r="L62" s="6"/>
-      <c r="M62" s="6"/>
-      <c r="N62" s="6"/>
-      <c r="O62" s="6"/>
-      <c r="P62" s="6"/>
-      <c r="Q62" s="6"/>
-      <c r="R62" s="6"/>
-      <c r="S62" s="6"/>
-      <c r="T62" s="6"/>
-      <c r="U62" s="6"/>
-      <c r="V62" s="6"/>
-      <c r="W62" s="6"/>
-      <c r="X62" s="6"/>
-      <c r="Y62" s="6"/>
-      <c r="Z62" s="6"/>
-      <c r="AA62" s="6"/>
-      <c r="AB62" s="6"/>
-      <c r="AC62" s="6"/>
+    <row r="61" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="9"/>
+      <c r="B61" s="5"/>
+      <c r="C61" s="5"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="I61" s="5"/>
+      <c r="J61" s="5"/>
+      <c r="K61" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="L61" s="5"/>
+      <c r="M61" s="5"/>
+      <c r="N61" s="5"/>
+      <c r="O61" s="5"/>
+      <c r="P61" s="5"/>
+      <c r="Q61" s="5"/>
+      <c r="R61" s="5"/>
+      <c r="S61" s="5"/>
+      <c r="T61" s="5"/>
+      <c r="U61" s="5"/>
+    </row>
+    <row r="62" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="9"/>
+      <c r="B62" s="5"/>
+      <c r="C62" s="5"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+      <c r="G62" s="5"/>
+      <c r="H62" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="I62" s="5"/>
+      <c r="J62" s="5"/>
+      <c r="K62" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="L62" s="5"/>
+      <c r="M62" s="5"/>
+      <c r="N62" s="5"/>
+      <c r="O62" s="5"/>
+      <c r="P62" s="5"/>
+      <c r="Q62" s="5"/>
+      <c r="R62" s="5"/>
+      <c r="S62" s="5"/>
+      <c r="T62" s="5"/>
+      <c r="U62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="4" t="s">
+      <c r="A63" s="2"/>
+      <c r="B63" s="2"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2"/>
+      <c r="G63" s="2"/>
+      <c r="H63" s="2"/>
+      <c r="I63" s="2"/>
+      <c r="J63" s="2"/>
+      <c r="K63" s="2"/>
+      <c r="L63" s="2"/>
+      <c r="M63" s="2"/>
+      <c r="N63" s="2"/>
+      <c r="O63" s="2"/>
+      <c r="P63" s="2"/>
+      <c r="Q63" s="2"/>
+      <c r="R63" s="2"/>
+      <c r="S63" s="2"/>
+      <c r="T63" s="2"/>
+      <c r="U63" s="2"/>
+    </row>
+    <row r="64" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="B64" s="6"/>
+      <c r="C64" s="6"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="6"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="6"/>
+      <c r="H64" s="6"/>
+      <c r="I64" s="6"/>
+      <c r="J64" s="6"/>
+      <c r="K64" s="6"/>
+      <c r="L64" s="6"/>
+      <c r="M64" s="6"/>
+      <c r="N64" s="6"/>
+      <c r="O64" s="6"/>
+      <c r="P64" s="6"/>
+      <c r="Q64" s="6"/>
+      <c r="R64" s="6"/>
+      <c r="S64" s="6"/>
+      <c r="T64" s="6"/>
+      <c r="U64" s="6"/>
+      <c r="V64" s="6"/>
+      <c r="W64" s="6"/>
+      <c r="X64" s="6"/>
+      <c r="Y64" s="6"/>
+      <c r="Z64" s="6"/>
+      <c r="AA64" s="6"/>
+      <c r="AB64" s="6"/>
+      <c r="AC64" s="6"/>
+    </row>
+    <row r="65" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B63" s="4"/>
-      <c r="C63" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="E63" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="F63" s="4"/>
-      <c r="G63" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="H63" s="4"/>
-      <c r="I63" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="J63" s="4"/>
-      <c r="L63" s="4" t="s">
+      <c r="B65" s="4"/>
+      <c r="C65" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="E65" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="F65" s="4"/>
+      <c r="G65" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H65" s="4"/>
+      <c r="I65" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="J65" s="4"/>
+      <c r="L65" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="M63" s="4"/>
-      <c r="N63" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="O63" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="P63" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="Q63" s="4"/>
-      <c r="R63" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="S63" s="4"/>
-      <c r="T63" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="U63" s="4"/>
-    </row>
-    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="9" t="n">
+      <c r="M65" s="4"/>
+      <c r="N65" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="O65" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="P65" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q65" s="4"/>
+      <c r="R65" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="S65" s="4"/>
+      <c r="T65" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="U65" s="4"/>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B64" s="9"/>
-      <c r="C64" s="9" t="n">
+      <c r="B66" s="9"/>
+      <c r="C66" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="D64" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="E64" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="F64" s="9"/>
-      <c r="G64" s="9"/>
-      <c r="H64" s="9"/>
-      <c r="I64" s="9"/>
-      <c r="J64" s="9"/>
-      <c r="L64" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="M64" s="9"/>
-      <c r="N64" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="O64" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="P64" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="Q64" s="5"/>
-      <c r="R64" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="S64" s="5"/>
-      <c r="T64" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="U64" s="5"/>
-    </row>
-    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C65" s="9"/>
-      <c r="D65" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="E65" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="F65" s="9"/>
-      <c r="G65" s="9"/>
-      <c r="H65" s="9"/>
-      <c r="I65" s="9"/>
-      <c r="J65" s="9"/>
-      <c r="N65" s="9"/>
-      <c r="O65" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="P65" s="5"/>
-      <c r="Q65" s="5"/>
-      <c r="R65" s="5"/>
-      <c r="S65" s="5"/>
-      <c r="T65" s="5"/>
-      <c r="U65" s="5"/>
-    </row>
-    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="4" t="s">
+      <c r="D66" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="B66" s="4"/>
-      <c r="C66" s="9"/>
-      <c r="D66" s="4" t="s">
+      <c r="E66" s="9" t="s">
         <v>161</v>
-      </c>
-      <c r="E66" s="9" t="s">
-        <v>155</v>
       </c>
       <c r="F66" s="9"/>
       <c r="G66" s="9"/>
       <c r="H66" s="9"/>
       <c r="I66" s="9"/>
       <c r="J66" s="9"/>
-      <c r="L66" s="4" t="s">
+      <c r="L66" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="M66" s="9"/>
+      <c r="N66" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O66" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="M66" s="4"/>
-      <c r="N66" s="9"/>
-      <c r="O66" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="P66" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q66" s="9"/>
-      <c r="R66" s="9"/>
-      <c r="S66" s="9"/>
-      <c r="T66" s="9"/>
-      <c r="U66" s="9"/>
+      <c r="P66" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q66" s="5"/>
+      <c r="R66" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="S66" s="5"/>
+      <c r="T66" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="U66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="B67" s="5"/>
       <c r="C67" s="9"/>
       <c r="D67" s="4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F67" s="9"/>
       <c r="G67" s="9"/>
       <c r="H67" s="9"/>
       <c r="I67" s="9"/>
       <c r="J67" s="9"/>
-      <c r="L67" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="M67" s="5"/>
       <c r="N67" s="9"/>
       <c r="O67" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="P67" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q67" s="9"/>
-      <c r="R67" s="9"/>
-      <c r="S67" s="9"/>
-      <c r="T67" s="9"/>
-      <c r="U67" s="9"/>
+        <v>165</v>
+      </c>
+      <c r="P67" s="5"/>
+      <c r="Q67" s="5"/>
+      <c r="R67" s="5"/>
+      <c r="S67" s="5"/>
+      <c r="T67" s="5"/>
+      <c r="U67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B68" s="4"/>
       <c r="C68" s="9"/>
       <c r="D68" s="4" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F68" s="9"/>
       <c r="G68" s="9"/>
       <c r="H68" s="9"/>
       <c r="I68" s="9"/>
       <c r="J68" s="9"/>
+      <c r="L68" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="M68" s="4"/>
       <c r="N68" s="9"/>
       <c r="O68" s="4" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="P68" s="9" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="Q68" s="9"/>
-      <c r="R68" s="9" t="s">
-        <v>165</v>
-      </c>
+      <c r="R68" s="9"/>
       <c r="S68" s="9"/>
-      <c r="T68" s="9" t="s">
-        <v>166</v>
-      </c>
+      <c r="T68" s="9"/>
       <c r="U68" s="9"/>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="B69" s="4"/>
+      <c r="A69" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B69" s="5"/>
       <c r="C69" s="9"/>
       <c r="D69" s="4" t="s">
         <v>168</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F69" s="9"/>
       <c r="G69" s="9"/>
       <c r="H69" s="9"/>
       <c r="I69" s="9"/>
       <c r="J69" s="9"/>
-      <c r="L69" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="M69" s="4"/>
+      <c r="L69" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="M69" s="5"/>
       <c r="N69" s="9"/>
       <c r="O69" s="4" t="s">
         <v>168</v>
       </c>
       <c r="P69" s="9" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="Q69" s="9"/>
-      <c r="R69" s="9" t="s">
-        <v>170</v>
-      </c>
+      <c r="R69" s="9"/>
       <c r="S69" s="9"/>
-      <c r="T69" s="9" t="s">
-        <v>171</v>
-      </c>
+      <c r="T69" s="9"/>
       <c r="U69" s="9"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="B70" s="5"/>
       <c r="C70" s="9"/>
       <c r="D70" s="4" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E70" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F70" s="9"/>
       <c r="G70" s="9"/>
       <c r="H70" s="9"/>
       <c r="I70" s="9"/>
       <c r="J70" s="9"/>
-      <c r="L70" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="M70" s="5"/>
       <c r="N70" s="9"/>
       <c r="O70" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="P70" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="Q70" s="9"/>
+      <c r="R70" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="S70" s="9"/>
+      <c r="T70" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="P70" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q70" s="9"/>
-      <c r="R70" s="9"/>
-      <c r="S70" s="9"/>
-      <c r="T70" s="9"/>
       <c r="U70" s="9"/>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B71" s="4"/>
       <c r="C71" s="9"/>
       <c r="D71" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F71" s="9"/>
       <c r="G71" s="9"/>
       <c r="H71" s="9"/>
       <c r="I71" s="9"/>
       <c r="J71" s="9"/>
+      <c r="L71" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="M71" s="4"/>
       <c r="N71" s="9"/>
       <c r="O71" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="P71" s="9" t="s">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="Q71" s="9"/>
-      <c r="R71" s="9"/>
+      <c r="R71" s="9" t="s">
+        <v>176</v>
+      </c>
       <c r="S71" s="9"/>
-      <c r="T71" s="9"/>
+      <c r="T71" s="9" t="s">
+        <v>177</v>
+      </c>
       <c r="U71" s="9"/>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B72" s="4"/>
-      <c r="C72" s="9" t="n">
-        <v>2</v>
-      </c>
+      <c r="A72" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B72" s="5"/>
+      <c r="C72" s="9"/>
       <c r="D72" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="E72" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F72" s="9"/>
       <c r="G72" s="9"/>
       <c r="H72" s="9"/>
       <c r="I72" s="9"/>
       <c r="J72" s="9"/>
-      <c r="L72" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="M72" s="4"/>
+      <c r="L72" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="M72" s="5"/>
       <c r="N72" s="9"/>
-      <c r="O72" s="4"/>
-      <c r="P72" s="9"/>
+      <c r="O72" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="P72" s="9" t="s">
+        <v>161</v>
+      </c>
       <c r="Q72" s="9"/>
       <c r="R72" s="9"/>
       <c r="S72" s="9"/>
@@ -4497,29 +4519,25 @@
       <c r="U72" s="9"/>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="B73" s="5"/>
       <c r="C73" s="9"/>
       <c r="D73" s="4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
       <c r="H73" s="9"/>
       <c r="I73" s="9"/>
       <c r="J73" s="9"/>
-      <c r="L73" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="M73" s="5"/>
       <c r="N73" s="9"/>
-      <c r="O73" s="4"/>
-      <c r="P73" s="9"/>
+      <c r="O73" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="P73" s="9" t="s">
+        <v>161</v>
+      </c>
       <c r="Q73" s="9"/>
       <c r="R73" s="9"/>
       <c r="S73" s="9"/>
@@ -4527,18 +4545,28 @@
       <c r="U73" s="9"/>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C74" s="9"/>
+      <c r="A74" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B74" s="4"/>
+      <c r="C74" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="D74" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
       <c r="H74" s="9"/>
       <c r="I74" s="9"/>
       <c r="J74" s="9"/>
+      <c r="L74" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="M74" s="4"/>
       <c r="N74" s="9"/>
       <c r="O74" s="4"/>
       <c r="P74" s="9"/>
@@ -4549,18 +4577,26 @@
       <c r="U74" s="9"/>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B75" s="5"/>
       <c r="C75" s="9"/>
       <c r="D75" s="4" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F75" s="9"/>
       <c r="G75" s="9"/>
       <c r="H75" s="9"/>
       <c r="I75" s="9"/>
       <c r="J75" s="9"/>
+      <c r="L75" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="M75" s="5"/>
       <c r="N75" s="9"/>
       <c r="O75" s="4"/>
       <c r="P75" s="9"/>
@@ -4573,10 +4609,10 @@
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C76" s="9"/>
       <c r="D76" s="4" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="E76" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F76" s="9"/>
       <c r="G76" s="9"/>
@@ -4595,10 +4631,10 @@
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C77" s="9"/>
       <c r="D77" s="4" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
@@ -4617,10 +4653,10 @@
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C78" s="9"/>
       <c r="D78" s="4" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="E78" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
@@ -4639,10 +4675,10 @@
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C79" s="9"/>
       <c r="D79" s="4" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
@@ -4658,134 +4694,122 @@
       <c r="T79" s="9"/>
       <c r="U79" s="9"/>
     </row>
-    <row r="81" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="4" t="s">
+    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C80" s="9"/>
+      <c r="D80" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E80" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F80" s="9"/>
+      <c r="G80" s="9"/>
+      <c r="H80" s="9"/>
+      <c r="I80" s="9"/>
+      <c r="J80" s="9"/>
+      <c r="N80" s="9"/>
+      <c r="O80" s="4"/>
+      <c r="P80" s="9"/>
+      <c r="Q80" s="9"/>
+      <c r="R80" s="9"/>
+      <c r="S80" s="9"/>
+      <c r="T80" s="9"/>
+      <c r="U80" s="9"/>
+    </row>
+    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C81" s="9"/>
+      <c r="D81" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="E81" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F81" s="9"/>
+      <c r="G81" s="9"/>
+      <c r="H81" s="9"/>
+      <c r="I81" s="9"/>
+      <c r="J81" s="9"/>
+      <c r="N81" s="9"/>
+      <c r="O81" s="4"/>
+      <c r="P81" s="9"/>
+      <c r="Q81" s="9"/>
+      <c r="R81" s="9"/>
+      <c r="S81" s="9"/>
+      <c r="T81" s="9"/>
+      <c r="U81" s="9"/>
+    </row>
+    <row r="83" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B81" s="4"/>
-      <c r="C81" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="D81" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="E81" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="F81" s="4"/>
-      <c r="G81" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="H81" s="4"/>
-      <c r="I81" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="J81" s="4"/>
-      <c r="L81" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="M81" s="4"/>
-      <c r="O81" s="4" t="s">
+      <c r="B83" s="4"/>
+      <c r="C83" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D83" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="P81" s="4"/>
-    </row>
-    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="9" t="n">
+      <c r="E83" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="F83" s="4"/>
+      <c r="G83" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H83" s="4"/>
+      <c r="I83" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="J83" s="4"/>
+      <c r="L83" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="M83" s="4"/>
+      <c r="O83" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="P83" s="4"/>
+    </row>
+    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B82" s="9"/>
-      <c r="C82" s="9" t="n">
+      <c r="B84" s="9"/>
+      <c r="C84" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="D82" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="F82" s="5"/>
-      <c r="G82" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="H82" s="5"/>
-      <c r="I82" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="J82" s="5"/>
-      <c r="L82" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M82" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="O82" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P82" s="9" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C83" s="9"/>
-      <c r="D83" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="E83" s="5"/>
-      <c r="F83" s="5"/>
-      <c r="G83" s="5"/>
-      <c r="H83" s="5"/>
-      <c r="I83" s="5"/>
-      <c r="J83" s="5"/>
-      <c r="L83" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="M83" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="O83" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="P83" s="9" t="s">
+      <c r="D84" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E84" s="5" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="B84" s="4"/>
-      <c r="C84" s="9"/>
-      <c r="D84" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="E84" s="5"/>
       <c r="F84" s="5"/>
-      <c r="G84" s="5"/>
+      <c r="G84" s="5" t="s">
+        <v>191</v>
+      </c>
       <c r="H84" s="5"/>
-      <c r="I84" s="5"/>
+      <c r="I84" s="5" t="s">
+        <v>192</v>
+      </c>
       <c r="J84" s="5"/>
       <c r="L84" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M84" s="9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="O84" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P84" s="9" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="B85" s="5"/>
       <c r="C85" s="9"/>
       <c r="D85" s="4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E85" s="5"/>
       <c r="F85" s="5"/>
@@ -4794,47 +4818,51 @@
       <c r="I85" s="5"/>
       <c r="J85" s="5"/>
       <c r="L85" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M85" s="9" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="O85" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P85" s="9" t="s">
-        <v>155</v>
+        <v>196</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B86" s="4"/>
       <c r="C86" s="9"/>
       <c r="D86" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="E86" s="5" t="s">
-        <v>194</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="E86" s="5"/>
       <c r="F86" s="5"/>
-      <c r="G86" s="5" t="s">
-        <v>195</v>
-      </c>
+      <c r="G86" s="5"/>
       <c r="H86" s="5"/>
-      <c r="I86" s="5" t="s">
-        <v>196</v>
-      </c>
+      <c r="I86" s="5"/>
       <c r="J86" s="5"/>
       <c r="L86" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M86" s="9" t="s">
         <v>197</v>
       </c>
+      <c r="O86" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="P86" s="9" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="B87" s="4"/>
+      <c r="A87" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B87" s="5"/>
       <c r="C87" s="9"/>
       <c r="D87" s="4" t="s">
         <v>168</v>
@@ -4846,52 +4874,76 @@
       <c r="I87" s="5"/>
       <c r="J87" s="5"/>
       <c r="L87" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M87" s="9" t="s">
-        <v>198</v>
+        <v>199</v>
+      </c>
+      <c r="O87" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="P87" s="9" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="B88" s="5"/>
       <c r="C88" s="9"/>
       <c r="D88" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="E88" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="F88" s="9"/>
-      <c r="G88" s="9"/>
-      <c r="H88" s="9"/>
-      <c r="I88" s="9"/>
-      <c r="J88" s="9"/>
+        <v>169</v>
+      </c>
+      <c r="E88" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="F88" s="5"/>
+      <c r="G88" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="H88" s="5"/>
+      <c r="I88" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="J88" s="5"/>
+      <c r="L88" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M88" s="9" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B89" s="4"/>
       <c r="C89" s="9"/>
       <c r="D89" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="E89" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="F89" s="9"/>
-      <c r="G89" s="9"/>
-      <c r="H89" s="9"/>
-      <c r="I89" s="9"/>
-      <c r="J89" s="9"/>
+        <v>174</v>
+      </c>
+      <c r="E89" s="5"/>
+      <c r="F89" s="5"/>
+      <c r="G89" s="5"/>
+      <c r="H89" s="5"/>
+      <c r="I89" s="5"/>
+      <c r="J89" s="5"/>
+      <c r="L89" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="M89" s="9" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B90" s="4"/>
+      <c r="A90" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B90" s="5"/>
       <c r="C90" s="9"/>
-      <c r="D90" s="4"/>
-      <c r="E90" s="9"/>
+      <c r="D90" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="E90" s="9" t="s">
+        <v>161</v>
+      </c>
       <c r="F90" s="9"/>
       <c r="G90" s="9"/>
       <c r="H90" s="9"/>
@@ -4899,13 +4951,13 @@
       <c r="J90" s="9"/>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="B91" s="5"/>
       <c r="C91" s="9"/>
-      <c r="D91" s="4"/>
-      <c r="E91" s="9"/>
+      <c r="D91" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="E91" s="9" t="s">
+        <v>161</v>
+      </c>
       <c r="F91" s="9"/>
       <c r="G91" s="9"/>
       <c r="H91" s="9"/>
@@ -4913,6 +4965,10 @@
       <c r="J91" s="9"/>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B92" s="4"/>
       <c r="C92" s="9"/>
       <c r="D92" s="4"/>
       <c r="E92" s="9"/>
@@ -4923,6 +4979,10 @@
       <c r="J92" s="9"/>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="B93" s="5"/>
       <c r="C93" s="9"/>
       <c r="D93" s="4"/>
       <c r="E93" s="9"/>
@@ -4972,430 +5032,380 @@
       <c r="I97" s="9"/>
       <c r="J97" s="9"/>
     </row>
-    <row r="98" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A98" s="2"/>
-      <c r="B98" s="2"/>
-      <c r="C98" s="2"/>
-      <c r="D98" s="2"/>
-      <c r="E98" s="2"/>
-      <c r="F98" s="2"/>
-      <c r="G98" s="2"/>
-      <c r="H98" s="2"/>
-      <c r="I98" s="2"/>
-      <c r="J98" s="2"/>
-      <c r="K98" s="2"/>
-      <c r="L98" s="2"/>
-      <c r="M98" s="2"/>
-      <c r="N98" s="2"/>
-      <c r="O98" s="2"/>
-      <c r="P98" s="2"/>
-      <c r="Q98" s="2"/>
-      <c r="R98" s="2"/>
-      <c r="S98" s="2"/>
-      <c r="T98" s="2"/>
-      <c r="U98" s="2"/>
-    </row>
-    <row r="99" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A99" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="B99" s="6"/>
-      <c r="C99" s="6"/>
-      <c r="D99" s="6"/>
-      <c r="E99" s="6"/>
-      <c r="F99" s="6"/>
-      <c r="G99" s="6"/>
-      <c r="H99" s="6"/>
-      <c r="I99" s="6"/>
-      <c r="J99" s="6"/>
-      <c r="K99" s="6"/>
-      <c r="L99" s="6"/>
-      <c r="M99" s="6"/>
-      <c r="N99" s="6"/>
-      <c r="O99" s="6"/>
-      <c r="P99" s="6"/>
-      <c r="Q99" s="6"/>
-      <c r="R99" s="6"/>
-      <c r="S99" s="6"/>
-      <c r="T99" s="6"/>
-      <c r="U99" s="6"/>
+    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C98" s="9"/>
+      <c r="D98" s="4"/>
+      <c r="E98" s="9"/>
+      <c r="F98" s="9"/>
+      <c r="G98" s="9"/>
+      <c r="H98" s="9"/>
+      <c r="I98" s="9"/>
+      <c r="J98" s="9"/>
+    </row>
+    <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C99" s="9"/>
+      <c r="D99" s="4"/>
+      <c r="E99" s="9"/>
+      <c r="F99" s="9"/>
+      <c r="G99" s="9"/>
+      <c r="H99" s="9"/>
+      <c r="I99" s="9"/>
+      <c r="J99" s="9"/>
     </row>
     <row r="100" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A100" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="B100" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="C100" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="D100" s="4" t="s">
+      <c r="A100" s="2"/>
+      <c r="B100" s="2"/>
+      <c r="C100" s="2"/>
+      <c r="D100" s="2"/>
+      <c r="E100" s="2"/>
+      <c r="F100" s="2"/>
+      <c r="G100" s="2"/>
+      <c r="H100" s="2"/>
+      <c r="I100" s="2"/>
+      <c r="J100" s="2"/>
+      <c r="K100" s="2"/>
+      <c r="L100" s="2"/>
+      <c r="M100" s="2"/>
+      <c r="N100" s="2"/>
+      <c r="O100" s="2"/>
+      <c r="P100" s="2"/>
+      <c r="Q100" s="2"/>
+      <c r="R100" s="2"/>
+      <c r="S100" s="2"/>
+      <c r="T100" s="2"/>
+      <c r="U100" s="2"/>
+    </row>
+    <row r="101" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A101" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="B101" s="6"/>
+      <c r="C101" s="6"/>
+      <c r="D101" s="6"/>
+      <c r="E101" s="6"/>
+      <c r="F101" s="6"/>
+      <c r="G101" s="6"/>
+      <c r="H101" s="6"/>
+      <c r="I101" s="6"/>
+      <c r="J101" s="6"/>
+      <c r="K101" s="6"/>
+      <c r="L101" s="6"/>
+      <c r="M101" s="6"/>
+      <c r="N101" s="6"/>
+      <c r="O101" s="6"/>
+      <c r="P101" s="6"/>
+      <c r="Q101" s="6"/>
+      <c r="R101" s="6"/>
+      <c r="S101" s="6"/>
+      <c r="T101" s="6"/>
+      <c r="U101" s="6"/>
+    </row>
+    <row r="102" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D102" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E100" s="4"/>
-      <c r="F100" s="4"/>
-      <c r="H100" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="I100" s="4"/>
-      <c r="J100" s="4"/>
-      <c r="K100" s="4"/>
-      <c r="L100" s="4"/>
-      <c r="M100" s="4"/>
-      <c r="N100" s="4"/>
-      <c r="O100" s="4"/>
-    </row>
-    <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B101" s="15"/>
-      <c r="C101" s="9"/>
-      <c r="D101" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="E101" s="5"/>
-      <c r="F101" s="5"/>
-      <c r="H101" s="16" t="s">
-        <v>204</v>
-      </c>
-      <c r="I101" s="17"/>
-      <c r="J101" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="K101" s="17"/>
-      <c r="L101" s="19" t="s">
-        <v>205</v>
-      </c>
-      <c r="M101" s="17"/>
-      <c r="N101" s="20" t="s">
-        <v>206</v>
-      </c>
-      <c r="O101" s="17"/>
-    </row>
-    <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B102" s="15"/>
-      <c r="C102" s="15"/>
-      <c r="D102" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="E102" s="5"/>
-      <c r="F102" s="5"/>
-      <c r="H102" s="16" t="s">
-        <v>207</v>
-      </c>
-      <c r="I102" s="21"/>
-      <c r="J102" s="18" t="s">
-        <v>208</v>
-      </c>
-      <c r="K102" s="22"/>
-      <c r="L102" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="M102" s="23"/>
-      <c r="N102" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="O102" s="24"/>
+      <c r="E102" s="4"/>
+      <c r="F102" s="4"/>
+      <c r="H102" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="I102" s="4"/>
+      <c r="J102" s="4"/>
+      <c r="K102" s="4"/>
+      <c r="L102" s="4"/>
+      <c r="M102" s="4"/>
+      <c r="N102" s="4"/>
+      <c r="O102" s="4"/>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B103" s="25"/>
+        <v>1</v>
+      </c>
+      <c r="B103" s="15"/>
       <c r="C103" s="9"/>
       <c r="D103" s="5" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="E103" s="5"/>
       <c r="F103" s="5"/>
-      <c r="O103" s="26" t="s">
-        <v>209</v>
-      </c>
+      <c r="H103" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="I103" s="17"/>
+      <c r="J103" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="K103" s="17"/>
+      <c r="L103" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="M103" s="17"/>
+      <c r="N103" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="O103" s="17"/>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B104" s="25"/>
-      <c r="C104" s="25"/>
+        <v>2</v>
+      </c>
+      <c r="B104" s="15"/>
+      <c r="C104" s="15"/>
       <c r="D104" s="5" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="E104" s="5"/>
       <c r="F104" s="5"/>
-      <c r="H104" s="27"/>
-      <c r="I104" s="28"/>
-      <c r="J104" s="28"/>
-      <c r="K104" s="27"/>
+      <c r="H104" s="16" t="s">
+        <v>213</v>
+      </c>
+      <c r="I104" s="21"/>
+      <c r="J104" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="K104" s="22"/>
+      <c r="L104" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="M104" s="23"/>
+      <c r="N104" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="O104" s="24"/>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B105" s="29"/>
+        <v>3</v>
+      </c>
+      <c r="B105" s="25"/>
       <c r="C105" s="9"/>
       <c r="D105" s="5" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E105" s="5"/>
       <c r="F105" s="5"/>
-      <c r="I105" s="28"/>
-      <c r="J105" s="28"/>
-    </row>
-    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="O105" s="26" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B106" s="29"/>
-      <c r="C106" s="29"/>
+        <v>4</v>
+      </c>
+      <c r="B106" s="25"/>
+      <c r="C106" s="25"/>
       <c r="D106" s="5" t="s">
-        <v>49</v>
+        <v>214</v>
       </c>
       <c r="E106" s="5"/>
       <c r="F106" s="5"/>
-    </row>
-    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H106" s="27"/>
+      <c r="I106" s="28"/>
+      <c r="J106" s="28"/>
+      <c r="K106" s="27"/>
+    </row>
+    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B107" s="30"/>
+        <v>5</v>
+      </c>
+      <c r="B107" s="29"/>
       <c r="C107" s="9"/>
       <c r="D107" s="5" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="E107" s="5"/>
       <c r="F107" s="5"/>
+      <c r="I107" s="28"/>
+      <c r="J107" s="28"/>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B108" s="30"/>
-      <c r="C108" s="30"/>
+        <v>6</v>
+      </c>
+      <c r="B108" s="29"/>
+      <c r="C108" s="29"/>
       <c r="D108" s="5" t="s">
         <v>49</v>
       </c>
       <c r="E108" s="5"/>
       <c r="F108" s="5"/>
     </row>
-    <row r="109" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A109" s="2"/>
-      <c r="B109" s="2"/>
-      <c r="C109" s="2"/>
-      <c r="D109" s="2"/>
-      <c r="E109" s="2"/>
-      <c r="F109" s="2"/>
-      <c r="G109" s="2"/>
-      <c r="H109" s="2"/>
-      <c r="I109" s="2"/>
-      <c r="J109" s="2"/>
-      <c r="K109" s="2"/>
-      <c r="L109" s="2"/>
-      <c r="M109" s="2"/>
-      <c r="N109" s="2"/>
-      <c r="O109" s="2"/>
-      <c r="P109" s="2"/>
-      <c r="Q109" s="2"/>
-      <c r="R109" s="2"/>
-      <c r="S109" s="2"/>
-      <c r="T109" s="2"/>
-      <c r="U109" s="2"/>
-    </row>
-    <row r="110" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A110" s="14" t="s">
+    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B109" s="30"/>
+      <c r="C109" s="9"/>
+      <c r="D109" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="E109" s="5"/>
+      <c r="F109" s="5"/>
+    </row>
+    <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A110" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B110" s="30"/>
+      <c r="C110" s="30"/>
+      <c r="D110" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E110" s="5"/>
+      <c r="F110" s="5"/>
+    </row>
+    <row r="111" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A111" s="2"/>
+      <c r="B111" s="2"/>
+      <c r="C111" s="2"/>
+      <c r="D111" s="2"/>
+      <c r="E111" s="2"/>
+      <c r="F111" s="2"/>
+      <c r="G111" s="2"/>
+      <c r="H111" s="2"/>
+      <c r="I111" s="2"/>
+      <c r="J111" s="2"/>
+      <c r="K111" s="2"/>
+      <c r="L111" s="2"/>
+      <c r="M111" s="2"/>
+      <c r="N111" s="2"/>
+      <c r="O111" s="2"/>
+      <c r="P111" s="2"/>
+      <c r="Q111" s="2"/>
+      <c r="R111" s="2"/>
+      <c r="S111" s="2"/>
+      <c r="T111" s="2"/>
+      <c r="U111" s="2"/>
+    </row>
+    <row r="112" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A112" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="B110" s="14"/>
-      <c r="C110" s="14"/>
-      <c r="D110" s="14"/>
-      <c r="E110" s="14"/>
-      <c r="F110" s="14"/>
-      <c r="G110" s="14"/>
-      <c r="H110" s="14"/>
-      <c r="I110" s="14"/>
-      <c r="J110" s="14"/>
-      <c r="K110" s="14"/>
-      <c r="L110" s="14"/>
-      <c r="M110" s="14"/>
-      <c r="N110" s="14"/>
-      <c r="O110" s="14"/>
-      <c r="P110" s="14"/>
-      <c r="Q110" s="14"/>
-      <c r="R110" s="14"/>
-      <c r="S110" s="14"/>
-      <c r="T110" s="14"/>
-      <c r="U110" s="14"/>
-    </row>
-    <row r="111" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A111" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B111" s="6"/>
-      <c r="C111" s="6"/>
-      <c r="D111" s="6"/>
-      <c r="E111" s="6"/>
-      <c r="F111" s="6"/>
-      <c r="G111" s="6"/>
-      <c r="H111" s="6"/>
-      <c r="I111" s="6"/>
-      <c r="J111" s="6"/>
-      <c r="K111" s="6"/>
-      <c r="L111" s="6"/>
-      <c r="M111" s="6"/>
-      <c r="N111" s="6"/>
-      <c r="O111" s="6"/>
-      <c r="P111" s="6"/>
-      <c r="Q111" s="6"/>
-      <c r="R111" s="6"/>
-      <c r="S111" s="6"/>
-      <c r="T111" s="6"/>
-      <c r="U111" s="6"/>
-    </row>
-    <row r="112" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A112" s="4" t="s">
+      <c r="B112" s="14"/>
+      <c r="C112" s="14"/>
+      <c r="D112" s="14"/>
+      <c r="E112" s="14"/>
+      <c r="F112" s="14"/>
+      <c r="G112" s="14"/>
+      <c r="H112" s="14"/>
+      <c r="I112" s="14"/>
+      <c r="J112" s="14"/>
+      <c r="K112" s="14"/>
+      <c r="L112" s="14"/>
+      <c r="M112" s="14"/>
+      <c r="N112" s="14"/>
+      <c r="O112" s="14"/>
+      <c r="P112" s="14"/>
+      <c r="Q112" s="14"/>
+      <c r="R112" s="14"/>
+      <c r="S112" s="14"/>
+      <c r="T112" s="14"/>
+      <c r="U112" s="14"/>
+    </row>
+    <row r="113" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A113" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B113" s="6"/>
+      <c r="C113" s="6"/>
+      <c r="D113" s="6"/>
+      <c r="E113" s="6"/>
+      <c r="F113" s="6"/>
+      <c r="G113" s="6"/>
+      <c r="H113" s="6"/>
+      <c r="I113" s="6"/>
+      <c r="J113" s="6"/>
+      <c r="K113" s="6"/>
+      <c r="L113" s="6"/>
+      <c r="M113" s="6"/>
+      <c r="N113" s="6"/>
+      <c r="O113" s="6"/>
+      <c r="P113" s="6"/>
+      <c r="Q113" s="6"/>
+      <c r="R113" s="6"/>
+      <c r="S113" s="6"/>
+      <c r="T113" s="6"/>
+      <c r="U113" s="6"/>
+    </row>
+    <row r="114" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A114" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B112" s="4" t="s">
+      <c r="B114" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C112" s="4"/>
-      <c r="D112" s="4"/>
-      <c r="E112" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="F112" s="4"/>
-      <c r="G112" s="4"/>
-      <c r="H112" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="I112" s="4"/>
-      <c r="J112" s="4"/>
-      <c r="K112" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="L112" s="4"/>
-      <c r="M112" s="4"/>
-      <c r="N112" s="4" t="s">
+      <c r="C114" s="4"/>
+      <c r="D114" s="4"/>
+      <c r="E114" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F114" s="4"/>
+      <c r="G114" s="4"/>
+      <c r="H114" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="I114" s="4"/>
+      <c r="J114" s="4"/>
+      <c r="K114" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="L114" s="4"/>
+      <c r="M114" s="4"/>
+      <c r="N114" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="O112" s="4"/>
-      <c r="P112" s="4"/>
-      <c r="Q112" s="4"/>
-      <c r="R112" s="4"/>
-      <c r="S112" s="4"/>
-      <c r="T112" s="4"/>
-      <c r="U112" s="4"/>
-    </row>
-    <row r="113" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A113" s="9" t="n">
+      <c r="O114" s="4"/>
+      <c r="P114" s="4"/>
+      <c r="Q114" s="4"/>
+      <c r="R114" s="4"/>
+      <c r="S114" s="4"/>
+      <c r="T114" s="4"/>
+      <c r="U114" s="4"/>
+    </row>
+    <row r="115" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A115" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B113" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="C113" s="5"/>
-      <c r="D113" s="5"/>
-      <c r="E113" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F113" s="5"/>
-      <c r="G113" s="5"/>
-      <c r="H113" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="I113" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="J113" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="K113" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="L113" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="M113" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="N113" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="O113" s="5"/>
-      <c r="P113" s="5"/>
-      <c r="Q113" s="5"/>
-      <c r="R113" s="5"/>
-      <c r="S113" s="5"/>
-      <c r="T113" s="5"/>
-      <c r="U113" s="5"/>
-    </row>
-    <row r="114" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A114" s="9"/>
-      <c r="B114" s="5"/>
-      <c r="C114" s="5"/>
-      <c r="D114" s="5"/>
-      <c r="E114" s="5"/>
-      <c r="F114" s="5"/>
-      <c r="G114" s="5"/>
-      <c r="H114" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="I114" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="J114" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="K114" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="L114" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="M114" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="N114" s="5"/>
-      <c r="O114" s="5"/>
-      <c r="P114" s="5"/>
-      <c r="Q114" s="5"/>
-      <c r="R114" s="5"/>
-      <c r="S114" s="5"/>
-      <c r="T114" s="5"/>
-      <c r="U114" s="5"/>
-    </row>
-    <row r="115" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A115" s="9"/>
-      <c r="B115" s="5"/>
+      <c r="B115" s="5" t="s">
+        <v>216</v>
+      </c>
       <c r="C115" s="5"/>
       <c r="D115" s="5"/>
-      <c r="E115" s="5"/>
+      <c r="E115" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="F115" s="5"/>
       <c r="G115" s="5"/>
       <c r="H115" s="5" t="s">
-        <v>145</v>
+        <v>217</v>
       </c>
       <c r="I115" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="J115" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="K115" s="5" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="L115" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="M115" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="N115" s="5"/>
+        <v>109</v>
+      </c>
+      <c r="N115" s="5" t="s">
+        <v>219</v>
+      </c>
       <c r="O115" s="5"/>
       <c r="P115" s="5"/>
       <c r="Q115" s="5"/>
@@ -5404,238 +5414,308 @@
       <c r="T115" s="5"/>
       <c r="U115" s="5"/>
     </row>
-    <row r="116" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A116" s="2"/>
-      <c r="B116" s="2"/>
-      <c r="C116" s="2"/>
-      <c r="D116" s="2"/>
-      <c r="E116" s="2"/>
-      <c r="F116" s="2"/>
-      <c r="G116" s="2"/>
-      <c r="H116" s="2"/>
-      <c r="I116" s="2"/>
-      <c r="J116" s="2"/>
-      <c r="K116" s="2"/>
-      <c r="L116" s="2"/>
-      <c r="M116" s="2"/>
-      <c r="N116" s="2"/>
-      <c r="O116" s="2"/>
-      <c r="P116" s="2"/>
-      <c r="Q116" s="2"/>
-      <c r="R116" s="2"/>
-      <c r="S116" s="2"/>
-      <c r="T116" s="2"/>
-      <c r="U116" s="2"/>
-    </row>
-    <row r="117" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A117" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="B117" s="6"/>
-      <c r="C117" s="6"/>
-      <c r="D117" s="6"/>
-      <c r="E117" s="6"/>
-      <c r="F117" s="6"/>
-      <c r="G117" s="6"/>
-      <c r="H117" s="6"/>
-      <c r="I117" s="6"/>
-      <c r="J117" s="6"/>
-      <c r="K117" s="6"/>
-      <c r="L117" s="6"/>
-      <c r="M117" s="6"/>
-      <c r="N117" s="6"/>
-      <c r="O117" s="6"/>
-      <c r="P117" s="6"/>
-      <c r="Q117" s="6"/>
-      <c r="R117" s="6"/>
-      <c r="S117" s="6"/>
-      <c r="T117" s="6"/>
-      <c r="U117" s="6"/>
-      <c r="V117" s="6"/>
-      <c r="W117" s="6"/>
-      <c r="X117" s="6"/>
-      <c r="Y117" s="6"/>
-      <c r="Z117" s="6"/>
-      <c r="AA117" s="6"/>
-      <c r="AB117" s="6"/>
-      <c r="AC117" s="6"/>
+    <row r="116" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A116" s="9"/>
+      <c r="B116" s="5"/>
+      <c r="C116" s="5"/>
+      <c r="D116" s="5"/>
+      <c r="E116" s="5"/>
+      <c r="F116" s="5"/>
+      <c r="G116" s="5"/>
+      <c r="H116" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I116" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="J116" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="K116" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="L116" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="M116" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="N116" s="5"/>
+      <c r="O116" s="5"/>
+      <c r="P116" s="5"/>
+      <c r="Q116" s="5"/>
+      <c r="R116" s="5"/>
+      <c r="S116" s="5"/>
+      <c r="T116" s="5"/>
+      <c r="U116" s="5"/>
+    </row>
+    <row r="117" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A117" s="9"/>
+      <c r="B117" s="5"/>
+      <c r="C117" s="5"/>
+      <c r="D117" s="5"/>
+      <c r="E117" s="5"/>
+      <c r="F117" s="5"/>
+      <c r="G117" s="5"/>
+      <c r="H117" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="I117" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="J117" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="K117" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="L117" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="M117" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="N117" s="5"/>
+      <c r="O117" s="5"/>
+      <c r="P117" s="5"/>
+      <c r="Q117" s="5"/>
+      <c r="R117" s="5"/>
+      <c r="S117" s="5"/>
+      <c r="T117" s="5"/>
+      <c r="U117" s="5"/>
     </row>
     <row r="118" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="4" t="s">
+      <c r="A118" s="2"/>
+      <c r="B118" s="2"/>
+      <c r="C118" s="2"/>
+      <c r="D118" s="2"/>
+      <c r="E118" s="2"/>
+      <c r="F118" s="2"/>
+      <c r="G118" s="2"/>
+      <c r="H118" s="2"/>
+      <c r="I118" s="2"/>
+      <c r="J118" s="2"/>
+      <c r="K118" s="2"/>
+      <c r="L118" s="2"/>
+      <c r="M118" s="2"/>
+      <c r="N118" s="2"/>
+      <c r="O118" s="2"/>
+      <c r="P118" s="2"/>
+      <c r="Q118" s="2"/>
+      <c r="R118" s="2"/>
+      <c r="S118" s="2"/>
+      <c r="T118" s="2"/>
+      <c r="U118" s="2"/>
+    </row>
+    <row r="119" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A119" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="B119" s="6"/>
+      <c r="C119" s="6"/>
+      <c r="D119" s="6"/>
+      <c r="E119" s="6"/>
+      <c r="F119" s="6"/>
+      <c r="G119" s="6"/>
+      <c r="H119" s="6"/>
+      <c r="I119" s="6"/>
+      <c r="J119" s="6"/>
+      <c r="K119" s="6"/>
+      <c r="L119" s="6"/>
+      <c r="M119" s="6"/>
+      <c r="N119" s="6"/>
+      <c r="O119" s="6"/>
+      <c r="P119" s="6"/>
+      <c r="Q119" s="6"/>
+      <c r="R119" s="6"/>
+      <c r="S119" s="6"/>
+      <c r="T119" s="6"/>
+      <c r="U119" s="6"/>
+      <c r="V119" s="6"/>
+      <c r="W119" s="6"/>
+      <c r="X119" s="6"/>
+      <c r="Y119" s="6"/>
+      <c r="Z119" s="6"/>
+      <c r="AA119" s="6"/>
+      <c r="AB119" s="6"/>
+      <c r="AC119" s="6"/>
+    </row>
+    <row r="120" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A120" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B118" s="4" t="s">
+      <c r="B120" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="C120" s="4"/>
+      <c r="D120" s="4"/>
+      <c r="E120" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="F120" s="4"/>
+      <c r="G120" s="4"/>
+      <c r="H120" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="I120" s="4"/>
+      <c r="J120" s="4"/>
+      <c r="K120" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="L120" s="4"/>
+      <c r="M120" s="4"/>
+      <c r="N120" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="O120" s="4"/>
+      <c r="P120" s="4"/>
+      <c r="Q120" s="4"/>
+      <c r="R120" s="4"/>
+      <c r="S120" s="4"/>
+      <c r="T120" s="4"/>
+      <c r="U120" s="4"/>
+      <c r="V120" s="4"/>
+      <c r="W120" s="4"/>
+      <c r="X120" s="4"/>
+      <c r="Y120" s="4"/>
+      <c r="Z120" s="4"/>
+      <c r="AA120" s="4"/>
+      <c r="AB120" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="AC120" s="4"/>
+    </row>
+    <row r="121" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A121" s="4"/>
+      <c r="B121" s="4"/>
+      <c r="C121" s="4"/>
+      <c r="D121" s="4"/>
+      <c r="E121" s="4"/>
+      <c r="F121" s="4"/>
+      <c r="G121" s="4"/>
+      <c r="H121" s="4"/>
+      <c r="I121" s="4"/>
+      <c r="J121" s="4"/>
+      <c r="K121" s="4"/>
+      <c r="L121" s="4"/>
+      <c r="M121" s="4"/>
+      <c r="N121" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="O121" s="31"/>
+      <c r="P121" s="31" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q121" s="31"/>
+      <c r="R121" s="31" t="s">
+        <v>174</v>
+      </c>
+      <c r="S121" s="31"/>
+      <c r="T121" s="31" t="s">
+        <v>169</v>
+      </c>
+      <c r="U121" s="31"/>
+      <c r="V121" s="31" t="s">
+        <v>168</v>
+      </c>
+      <c r="W121" s="31"/>
+      <c r="X121" s="31" t="s">
+        <v>167</v>
+      </c>
+      <c r="Y121" s="31"/>
+      <c r="Z121" s="31" t="s">
+        <v>165</v>
+      </c>
+      <c r="AA121" s="31"/>
+      <c r="AB121" s="31" t="s">
         <v>160</v>
       </c>
-      <c r="C118" s="4"/>
-      <c r="D118" s="4"/>
-      <c r="E118" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="F118" s="4"/>
-      <c r="G118" s="4"/>
-      <c r="H118" s="4" t="s">
+      <c r="AC121" s="31"/>
+    </row>
+    <row r="122" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A122" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B122" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="I118" s="4"/>
-      <c r="J118" s="4"/>
-      <c r="K118" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="L118" s="4"/>
-      <c r="M118" s="4"/>
-      <c r="N118" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="O118" s="4"/>
-      <c r="P118" s="4"/>
-      <c r="Q118" s="4"/>
-      <c r="R118" s="4"/>
-      <c r="S118" s="4"/>
-      <c r="T118" s="4"/>
-      <c r="U118" s="4"/>
-      <c r="V118" s="4"/>
-      <c r="W118" s="4"/>
-      <c r="X118" s="4"/>
-      <c r="Y118" s="4"/>
-      <c r="Z118" s="4"/>
-      <c r="AA118" s="4"/>
-      <c r="AB118" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="AC118" s="4"/>
-    </row>
-    <row r="119" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A119" s="4"/>
-      <c r="B119" s="4"/>
-      <c r="C119" s="4"/>
-      <c r="D119" s="4"/>
-      <c r="E119" s="4"/>
-      <c r="F119" s="4"/>
-      <c r="G119" s="4"/>
-      <c r="H119" s="4"/>
-      <c r="I119" s="4"/>
-      <c r="J119" s="4"/>
-      <c r="K119" s="4"/>
-      <c r="L119" s="4"/>
-      <c r="M119" s="4"/>
-      <c r="N119" s="31" t="s">
-        <v>173</v>
-      </c>
-      <c r="O119" s="31"/>
-      <c r="P119" s="31" t="s">
-        <v>172</v>
-      </c>
-      <c r="Q119" s="31"/>
-      <c r="R119" s="31" t="s">
-        <v>168</v>
-      </c>
-      <c r="S119" s="31"/>
-      <c r="T119" s="31" t="s">
-        <v>163</v>
-      </c>
-      <c r="U119" s="31"/>
-      <c r="V119" s="31" t="s">
+      <c r="C122" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E122" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="F122" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="G122" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="H122" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I122" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="J122" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="K122" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L122" s="5"/>
+      <c r="M122" s="5"/>
+      <c r="N122" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="O122" s="5"/>
+      <c r="P122" s="5"/>
+      <c r="Q122" s="5"/>
+      <c r="R122" s="5"/>
+      <c r="S122" s="5"/>
+      <c r="T122" s="5"/>
+      <c r="U122" s="5"/>
+      <c r="V122" s="5"/>
+      <c r="W122" s="5"/>
+      <c r="X122" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="Y122" s="5"/>
+      <c r="Z122" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="W119" s="31"/>
-      <c r="X119" s="31" t="s">
-        <v>161</v>
-      </c>
-      <c r="Y119" s="31"/>
-      <c r="Z119" s="31" t="s">
-        <v>159</v>
-      </c>
-      <c r="AA119" s="31"/>
-      <c r="AB119" s="31" t="s">
-        <v>154</v>
-      </c>
-      <c r="AC119" s="31"/>
-    </row>
-    <row r="120" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A120" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B120" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="C120" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="D120" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="E120" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="F120" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="G120" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="H120" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I120" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="J120" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="K120" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L120" s="5"/>
-      <c r="M120" s="5"/>
-      <c r="N120" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="O120" s="5"/>
-      <c r="P120" s="5"/>
-      <c r="Q120" s="5"/>
-      <c r="R120" s="5"/>
-      <c r="S120" s="5"/>
-      <c r="T120" s="5"/>
-      <c r="U120" s="5"/>
-      <c r="V120" s="5"/>
-      <c r="W120" s="5"/>
-      <c r="X120" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="Y120" s="5"/>
-      <c r="Z120" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="AA120" s="5"/>
-      <c r="AB120" s="5"/>
-      <c r="AC120" s="5"/>
-    </row>
-    <row r="121" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A121" s="2"/>
-      <c r="B121" s="2"/>
-      <c r="C121" s="2"/>
-      <c r="D121" s="2"/>
-      <c r="E121" s="2"/>
-      <c r="F121" s="2"/>
-      <c r="G121" s="2"/>
-      <c r="H121" s="2"/>
-      <c r="I121" s="2"/>
-      <c r="J121" s="2"/>
-      <c r="K121" s="2"/>
-      <c r="L121" s="2"/>
-      <c r="M121" s="2"/>
-      <c r="N121" s="2"/>
-      <c r="O121" s="2"/>
-      <c r="P121" s="2"/>
-      <c r="Q121" s="2"/>
-      <c r="R121" s="2"/>
-      <c r="S121" s="2"/>
-      <c r="T121" s="2"/>
-      <c r="U121" s="2"/>
+      <c r="AA122" s="5"/>
+      <c r="AB122" s="5"/>
+      <c r="AC122" s="5"/>
+    </row>
+    <row r="123" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A123" s="2"/>
+      <c r="B123" s="2"/>
+      <c r="C123" s="2"/>
+      <c r="D123" s="2"/>
+      <c r="E123" s="2"/>
+      <c r="F123" s="2"/>
+      <c r="G123" s="2"/>
+      <c r="H123" s="2"/>
+      <c r="I123" s="2"/>
+      <c r="J123" s="2"/>
+      <c r="K123" s="2"/>
+      <c r="L123" s="2"/>
+      <c r="M123" s="2"/>
+      <c r="N123" s="2"/>
+      <c r="O123" s="2"/>
+      <c r="P123" s="2"/>
+      <c r="Q123" s="2"/>
+      <c r="R123" s="2"/>
+      <c r="S123" s="2"/>
+      <c r="T123" s="2"/>
+      <c r="U123" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="387">
+  <mergeCells count="393">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -5682,8 +5762,8 @@
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="G16:N16"/>
-    <mergeCell ref="O16:Q20"/>
-    <mergeCell ref="R16:U20"/>
+    <mergeCell ref="O16:Q22"/>
+    <mergeCell ref="R16:U22"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="G17:N17"/>
@@ -5696,57 +5776,59 @@
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="G20:N20"/>
-    <mergeCell ref="A21:U21"/>
-    <mergeCell ref="A22:U22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="G23:N23"/>
-    <mergeCell ref="O23:Q23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="G24:N24"/>
-    <mergeCell ref="O24:Q24"/>
-    <mergeCell ref="A25:U25"/>
-    <mergeCell ref="A26:U26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="G27:N27"/>
-    <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="G28:N28"/>
-    <mergeCell ref="O28:Q28"/>
-    <mergeCell ref="A29:U29"/>
-    <mergeCell ref="A30:U30"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="G21:N21"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="G22:N22"/>
+    <mergeCell ref="A23:U23"/>
+    <mergeCell ref="A24:U24"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="G25:N25"/>
+    <mergeCell ref="O25:Q25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:N26"/>
+    <mergeCell ref="O26:Q26"/>
+    <mergeCell ref="A27:U27"/>
+    <mergeCell ref="A28:U28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="G29:N29"/>
+    <mergeCell ref="O29:Q29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="G30:N30"/>
+    <mergeCell ref="O30:Q30"/>
     <mergeCell ref="A31:U31"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="H32:J32"/>
-    <mergeCell ref="K32:M32"/>
-    <mergeCell ref="N32:U32"/>
-    <mergeCell ref="A33:A37"/>
-    <mergeCell ref="B33:D37"/>
-    <mergeCell ref="E33:G44"/>
-    <mergeCell ref="H33:J33"/>
-    <mergeCell ref="K33:M33"/>
-    <mergeCell ref="N33:U37"/>
+    <mergeCell ref="A32:U32"/>
+    <mergeCell ref="A33:U33"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="E34:G34"/>
     <mergeCell ref="H34:J34"/>
     <mergeCell ref="K34:M34"/>
+    <mergeCell ref="N34:U34"/>
+    <mergeCell ref="A35:A39"/>
+    <mergeCell ref="B35:D39"/>
+    <mergeCell ref="E35:G46"/>
     <mergeCell ref="H35:J35"/>
     <mergeCell ref="K35:M35"/>
+    <mergeCell ref="N35:U39"/>
     <mergeCell ref="H36:J36"/>
     <mergeCell ref="K36:M36"/>
     <mergeCell ref="H37:J37"/>
     <mergeCell ref="K37:M37"/>
-    <mergeCell ref="A38:A44"/>
-    <mergeCell ref="B38:D44"/>
     <mergeCell ref="H38:J38"/>
     <mergeCell ref="K38:M38"/>
-    <mergeCell ref="N38:U44"/>
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="K39:M39"/>
+    <mergeCell ref="A40:A46"/>
+    <mergeCell ref="B40:D46"/>
     <mergeCell ref="H40:J40"/>
     <mergeCell ref="K40:M40"/>
+    <mergeCell ref="N40:U46"/>
     <mergeCell ref="H41:J41"/>
     <mergeCell ref="K41:M41"/>
     <mergeCell ref="H42:J42"/>
@@ -5755,28 +5837,28 @@
     <mergeCell ref="K43:M43"/>
     <mergeCell ref="H44:J44"/>
     <mergeCell ref="K44:M44"/>
-    <mergeCell ref="A45:A48"/>
-    <mergeCell ref="B45:D48"/>
-    <mergeCell ref="E45:G48"/>
     <mergeCell ref="H45:J45"/>
     <mergeCell ref="K45:M45"/>
-    <mergeCell ref="N45:U48"/>
     <mergeCell ref="H46:J46"/>
     <mergeCell ref="K46:M46"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="B47:D50"/>
+    <mergeCell ref="E47:G50"/>
     <mergeCell ref="H47:J47"/>
     <mergeCell ref="K47:M47"/>
+    <mergeCell ref="N47:U50"/>
     <mergeCell ref="H48:J48"/>
     <mergeCell ref="K48:M48"/>
-    <mergeCell ref="A49:A60"/>
-    <mergeCell ref="B49:D60"/>
-    <mergeCell ref="E49:G60"/>
     <mergeCell ref="H49:J49"/>
     <mergeCell ref="K49:M49"/>
-    <mergeCell ref="N49:U60"/>
     <mergeCell ref="H50:J50"/>
     <mergeCell ref="K50:M50"/>
+    <mergeCell ref="A51:A62"/>
+    <mergeCell ref="B51:D62"/>
+    <mergeCell ref="E51:G62"/>
     <mergeCell ref="H51:J51"/>
     <mergeCell ref="K51:M51"/>
+    <mergeCell ref="N51:U62"/>
     <mergeCell ref="H52:J52"/>
     <mergeCell ref="K52:M52"/>
     <mergeCell ref="H53:J53"/>
@@ -5795,48 +5877,38 @@
     <mergeCell ref="K59:M59"/>
     <mergeCell ref="H60:J60"/>
     <mergeCell ref="K60:M60"/>
-    <mergeCell ref="A61:U61"/>
-    <mergeCell ref="A62:AC62"/>
-    <mergeCell ref="A63:B63"/>
-    <mergeCell ref="E63:F63"/>
-    <mergeCell ref="G63:H63"/>
-    <mergeCell ref="I63:J63"/>
-    <mergeCell ref="L63:M63"/>
-    <mergeCell ref="P63:Q63"/>
-    <mergeCell ref="R63:S63"/>
-    <mergeCell ref="T63:U63"/>
-    <mergeCell ref="A64:B64"/>
-    <mergeCell ref="C64:C71"/>
-    <mergeCell ref="E64:F64"/>
-    <mergeCell ref="G64:H64"/>
-    <mergeCell ref="I64:J64"/>
-    <mergeCell ref="L64:M64"/>
-    <mergeCell ref="N64:N71"/>
-    <mergeCell ref="P64:Q65"/>
-    <mergeCell ref="R64:S65"/>
-    <mergeCell ref="T64:U65"/>
+    <mergeCell ref="H61:J61"/>
+    <mergeCell ref="K61:M61"/>
+    <mergeCell ref="H62:J62"/>
+    <mergeCell ref="K62:M62"/>
+    <mergeCell ref="A63:U63"/>
+    <mergeCell ref="A64:AC64"/>
+    <mergeCell ref="A65:B65"/>
     <mergeCell ref="E65:F65"/>
     <mergeCell ref="G65:H65"/>
     <mergeCell ref="I65:J65"/>
+    <mergeCell ref="L65:M65"/>
+    <mergeCell ref="P65:Q65"/>
+    <mergeCell ref="R65:S65"/>
+    <mergeCell ref="T65:U65"/>
     <mergeCell ref="A66:B66"/>
+    <mergeCell ref="C66:C73"/>
     <mergeCell ref="E66:F66"/>
     <mergeCell ref="G66:H66"/>
     <mergeCell ref="I66:J66"/>
     <mergeCell ref="L66:M66"/>
-    <mergeCell ref="P66:Q66"/>
-    <mergeCell ref="R66:S66"/>
-    <mergeCell ref="T66:U66"/>
-    <mergeCell ref="A67:B67"/>
+    <mergeCell ref="N66:N73"/>
+    <mergeCell ref="P66:Q67"/>
+    <mergeCell ref="R66:S67"/>
+    <mergeCell ref="T66:U67"/>
     <mergeCell ref="E67:F67"/>
     <mergeCell ref="G67:H67"/>
     <mergeCell ref="I67:J67"/>
-    <mergeCell ref="L67:M67"/>
-    <mergeCell ref="P67:Q67"/>
-    <mergeCell ref="R67:S67"/>
-    <mergeCell ref="T67:U67"/>
+    <mergeCell ref="A68:B68"/>
     <mergeCell ref="E68:F68"/>
     <mergeCell ref="G68:H68"/>
     <mergeCell ref="I68:J68"/>
+    <mergeCell ref="L68:M68"/>
     <mergeCell ref="P68:Q68"/>
     <mergeCell ref="R68:S68"/>
     <mergeCell ref="T68:U68"/>
@@ -5848,47 +5920,49 @@
     <mergeCell ref="P69:Q69"/>
     <mergeCell ref="R69:S69"/>
     <mergeCell ref="T69:U69"/>
-    <mergeCell ref="A70:B70"/>
     <mergeCell ref="E70:F70"/>
     <mergeCell ref="G70:H70"/>
     <mergeCell ref="I70:J70"/>
-    <mergeCell ref="L70:M70"/>
     <mergeCell ref="P70:Q70"/>
     <mergeCell ref="R70:S70"/>
     <mergeCell ref="T70:U70"/>
+    <mergeCell ref="A71:B71"/>
     <mergeCell ref="E71:F71"/>
     <mergeCell ref="G71:H71"/>
     <mergeCell ref="I71:J71"/>
+    <mergeCell ref="L71:M71"/>
     <mergeCell ref="P71:Q71"/>
     <mergeCell ref="R71:S71"/>
     <mergeCell ref="T71:U71"/>
     <mergeCell ref="A72:B72"/>
-    <mergeCell ref="C72:C79"/>
     <mergeCell ref="E72:F72"/>
     <mergeCell ref="G72:H72"/>
     <mergeCell ref="I72:J72"/>
     <mergeCell ref="L72:M72"/>
-    <mergeCell ref="N72:N79"/>
     <mergeCell ref="P72:Q72"/>
     <mergeCell ref="R72:S72"/>
     <mergeCell ref="T72:U72"/>
-    <mergeCell ref="A73:B73"/>
     <mergeCell ref="E73:F73"/>
     <mergeCell ref="G73:H73"/>
     <mergeCell ref="I73:J73"/>
-    <mergeCell ref="L73:M73"/>
     <mergeCell ref="P73:Q73"/>
     <mergeCell ref="R73:S73"/>
     <mergeCell ref="T73:U73"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="C74:C81"/>
     <mergeCell ref="E74:F74"/>
     <mergeCell ref="G74:H74"/>
     <mergeCell ref="I74:J74"/>
+    <mergeCell ref="L74:M74"/>
+    <mergeCell ref="N74:N81"/>
     <mergeCell ref="P74:Q74"/>
     <mergeCell ref="R74:S74"/>
     <mergeCell ref="T74:U74"/>
+    <mergeCell ref="A75:B75"/>
     <mergeCell ref="E75:F75"/>
     <mergeCell ref="G75:H75"/>
     <mergeCell ref="I75:J75"/>
+    <mergeCell ref="L75:M75"/>
     <mergeCell ref="P75:Q75"/>
     <mergeCell ref="R75:S75"/>
     <mergeCell ref="T75:U75"/>
@@ -5916,42 +5990,48 @@
     <mergeCell ref="P79:Q79"/>
     <mergeCell ref="R79:S79"/>
     <mergeCell ref="T79:U79"/>
-    <mergeCell ref="A81:B81"/>
+    <mergeCell ref="E80:F80"/>
+    <mergeCell ref="G80:H80"/>
+    <mergeCell ref="I80:J80"/>
+    <mergeCell ref="P80:Q80"/>
+    <mergeCell ref="R80:S80"/>
+    <mergeCell ref="T80:U80"/>
     <mergeCell ref="E81:F81"/>
     <mergeCell ref="G81:H81"/>
     <mergeCell ref="I81:J81"/>
-    <mergeCell ref="L81:M81"/>
-    <mergeCell ref="O81:P81"/>
-    <mergeCell ref="A82:B82"/>
-    <mergeCell ref="C82:C89"/>
-    <mergeCell ref="E82:F85"/>
-    <mergeCell ref="G82:H85"/>
-    <mergeCell ref="I82:J85"/>
+    <mergeCell ref="P81:Q81"/>
+    <mergeCell ref="R81:S81"/>
+    <mergeCell ref="T81:U81"/>
+    <mergeCell ref="A83:B83"/>
+    <mergeCell ref="E83:F83"/>
+    <mergeCell ref="G83:H83"/>
+    <mergeCell ref="I83:J83"/>
+    <mergeCell ref="L83:M83"/>
+    <mergeCell ref="O83:P83"/>
     <mergeCell ref="A84:B84"/>
-    <mergeCell ref="A85:B85"/>
-    <mergeCell ref="E86:F87"/>
-    <mergeCell ref="G86:H87"/>
-    <mergeCell ref="I86:J87"/>
+    <mergeCell ref="C84:C91"/>
+    <mergeCell ref="E84:F87"/>
+    <mergeCell ref="G84:H87"/>
+    <mergeCell ref="I84:J87"/>
+    <mergeCell ref="A86:B86"/>
     <mergeCell ref="A87:B87"/>
-    <mergeCell ref="A88:B88"/>
-    <mergeCell ref="E88:F88"/>
-    <mergeCell ref="G88:H88"/>
-    <mergeCell ref="I88:J88"/>
-    <mergeCell ref="E89:F89"/>
-    <mergeCell ref="G89:H89"/>
-    <mergeCell ref="I89:J89"/>
+    <mergeCell ref="E88:F89"/>
+    <mergeCell ref="G88:H89"/>
+    <mergeCell ref="I88:J89"/>
+    <mergeCell ref="A89:B89"/>
     <mergeCell ref="A90:B90"/>
-    <mergeCell ref="C90:C97"/>
     <mergeCell ref="E90:F90"/>
     <mergeCell ref="G90:H90"/>
     <mergeCell ref="I90:J90"/>
-    <mergeCell ref="A91:B91"/>
     <mergeCell ref="E91:F91"/>
     <mergeCell ref="G91:H91"/>
     <mergeCell ref="I91:J91"/>
+    <mergeCell ref="A92:B92"/>
+    <mergeCell ref="C92:C99"/>
     <mergeCell ref="E92:F92"/>
     <mergeCell ref="G92:H92"/>
     <mergeCell ref="I92:J92"/>
+    <mergeCell ref="A93:B93"/>
     <mergeCell ref="E93:F93"/>
     <mergeCell ref="G93:H93"/>
     <mergeCell ref="I93:J93"/>
@@ -5967,62 +6047,68 @@
     <mergeCell ref="E97:F97"/>
     <mergeCell ref="G97:H97"/>
     <mergeCell ref="I97:J97"/>
-    <mergeCell ref="A98:U98"/>
-    <mergeCell ref="A99:U99"/>
-    <mergeCell ref="D100:F100"/>
-    <mergeCell ref="H100:O100"/>
-    <mergeCell ref="D101:F101"/>
+    <mergeCell ref="E98:F98"/>
+    <mergeCell ref="G98:H98"/>
+    <mergeCell ref="I98:J98"/>
+    <mergeCell ref="E99:F99"/>
+    <mergeCell ref="G99:H99"/>
+    <mergeCell ref="I99:J99"/>
+    <mergeCell ref="A100:U100"/>
+    <mergeCell ref="A101:U101"/>
     <mergeCell ref="D102:F102"/>
+    <mergeCell ref="H102:O102"/>
     <mergeCell ref="D103:F103"/>
     <mergeCell ref="D104:F104"/>
     <mergeCell ref="D105:F105"/>
     <mergeCell ref="D106:F106"/>
     <mergeCell ref="D107:F107"/>
     <mergeCell ref="D108:F108"/>
-    <mergeCell ref="A109:U109"/>
-    <mergeCell ref="A110:U110"/>
+    <mergeCell ref="D109:F109"/>
+    <mergeCell ref="D110:F110"/>
     <mergeCell ref="A111:U111"/>
-    <mergeCell ref="B112:D112"/>
-    <mergeCell ref="E112:G112"/>
-    <mergeCell ref="H112:J112"/>
-    <mergeCell ref="K112:M112"/>
-    <mergeCell ref="N112:U112"/>
-    <mergeCell ref="A113:A115"/>
-    <mergeCell ref="B113:D115"/>
-    <mergeCell ref="E113:G115"/>
-    <mergeCell ref="H113:J113"/>
-    <mergeCell ref="K113:M113"/>
-    <mergeCell ref="N113:U115"/>
+    <mergeCell ref="A112:U112"/>
+    <mergeCell ref="A113:U113"/>
+    <mergeCell ref="B114:D114"/>
+    <mergeCell ref="E114:G114"/>
     <mergeCell ref="H114:J114"/>
     <mergeCell ref="K114:M114"/>
+    <mergeCell ref="N114:U114"/>
+    <mergeCell ref="A115:A117"/>
+    <mergeCell ref="B115:D117"/>
+    <mergeCell ref="E115:G117"/>
     <mergeCell ref="H115:J115"/>
     <mergeCell ref="K115:M115"/>
-    <mergeCell ref="A116:U116"/>
-    <mergeCell ref="A117:AC117"/>
-    <mergeCell ref="A118:A119"/>
-    <mergeCell ref="B118:D119"/>
-    <mergeCell ref="E118:G119"/>
-    <mergeCell ref="H118:J119"/>
-    <mergeCell ref="K118:M119"/>
-    <mergeCell ref="N118:O118"/>
-    <mergeCell ref="P118:AA118"/>
-    <mergeCell ref="AB118:AC118"/>
-    <mergeCell ref="N119:O119"/>
-    <mergeCell ref="P119:Q119"/>
-    <mergeCell ref="R119:S119"/>
-    <mergeCell ref="T119:U119"/>
-    <mergeCell ref="V119:W119"/>
-    <mergeCell ref="X119:Y119"/>
-    <mergeCell ref="Z119:AA119"/>
-    <mergeCell ref="AB119:AC119"/>
-    <mergeCell ref="B120:D120"/>
-    <mergeCell ref="E120:G120"/>
-    <mergeCell ref="H120:J120"/>
-    <mergeCell ref="K120:M120"/>
-    <mergeCell ref="N120:W120"/>
-    <mergeCell ref="X120:Y120"/>
-    <mergeCell ref="Z120:AC120"/>
-    <mergeCell ref="A121:U121"/>
+    <mergeCell ref="N115:U117"/>
+    <mergeCell ref="H116:J116"/>
+    <mergeCell ref="K116:M116"/>
+    <mergeCell ref="H117:J117"/>
+    <mergeCell ref="K117:M117"/>
+    <mergeCell ref="A118:U118"/>
+    <mergeCell ref="A119:AC119"/>
+    <mergeCell ref="A120:A121"/>
+    <mergeCell ref="B120:D121"/>
+    <mergeCell ref="E120:G121"/>
+    <mergeCell ref="H120:J121"/>
+    <mergeCell ref="K120:M121"/>
+    <mergeCell ref="N120:O120"/>
+    <mergeCell ref="P120:AA120"/>
+    <mergeCell ref="AB120:AC120"/>
+    <mergeCell ref="N121:O121"/>
+    <mergeCell ref="P121:Q121"/>
+    <mergeCell ref="R121:S121"/>
+    <mergeCell ref="T121:U121"/>
+    <mergeCell ref="V121:W121"/>
+    <mergeCell ref="X121:Y121"/>
+    <mergeCell ref="Z121:AA121"/>
+    <mergeCell ref="AB121:AC121"/>
+    <mergeCell ref="B122:D122"/>
+    <mergeCell ref="E122:G122"/>
+    <mergeCell ref="H122:J122"/>
+    <mergeCell ref="K122:M122"/>
+    <mergeCell ref="N122:W122"/>
+    <mergeCell ref="X122:Y122"/>
+    <mergeCell ref="Z122:AC122"/>
+    <mergeCell ref="A123:U123"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -6302,7 +6388,7 @@
       <c r="C11" s="36"/>
       <c r="D11" s="32"/>
       <c r="E11" s="37" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="F11" s="37"/>
       <c r="G11" s="32"/>
@@ -6378,13 +6464,13 @@
       <c r="B14" s="32"/>
       <c r="C14" s="36"/>
       <c r="D14" s="41" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="E14" s="42" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F14" s="43" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="G14" s="32"/>
       <c r="H14" s="32"/>
@@ -6410,10 +6496,10 @@
       <c r="C15" s="36"/>
       <c r="D15" s="41"/>
       <c r="E15" s="44" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F15" s="45" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="G15" s="32"/>
       <c r="H15" s="32"/>
@@ -6439,10 +6525,10 @@
       <c r="C16" s="36"/>
       <c r="D16" s="41"/>
       <c r="E16" s="46" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F16" s="47" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="G16" s="32"/>
       <c r="H16" s="32"/>
@@ -6456,7 +6542,7 @@
       <c r="P16" s="32"/>
       <c r="Q16" s="32"/>
       <c r="R16" s="48" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="S16" s="48"/>
       <c r="T16" s="48"/>
@@ -6469,10 +6555,10 @@
       <c r="C17" s="36"/>
       <c r="D17" s="41"/>
       <c r="E17" s="49" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F17" s="50" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="G17" s="32"/>
       <c r="H17" s="32"/>
@@ -6520,13 +6606,13 @@
       <c r="B19" s="32"/>
       <c r="C19" s="36"/>
       <c r="D19" s="41" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="E19" s="49" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F19" s="50" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="G19" s="32"/>
       <c r="H19" s="32"/>
@@ -6550,10 +6636,10 @@
       <c r="C20" s="51"/>
       <c r="D20" s="41"/>
       <c r="E20" s="46" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F20" s="47" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="W20" s="52"/>
     </row>
@@ -6562,10 +6648,10 @@
       <c r="C21" s="36"/>
       <c r="D21" s="41"/>
       <c r="E21" s="44" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F21" s="45" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="G21" s="32"/>
       <c r="H21" s="32"/>
@@ -6591,10 +6677,10 @@
       <c r="C22" s="36"/>
       <c r="D22" s="41"/>
       <c r="E22" s="42" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F22" s="43" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="G22" s="55"/>
       <c r="H22" s="55"/>
@@ -6618,7 +6704,7 @@
     <row r="23" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C23" s="36"/>
       <c r="L23" s="57" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="U23" s="32"/>
       <c r="V23" s="32"/>
@@ -6648,7 +6734,7 @@
       <c r="J25" s="32"/>
       <c r="K25" s="32"/>
       <c r="L25" s="61" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="M25" s="62"/>
       <c r="N25" s="62"/>
@@ -6688,7 +6774,7 @@
       <c r="H27" s="32"/>
       <c r="I27" s="32"/>
       <c r="L27" s="68" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="M27" s="68"/>
       <c r="N27" s="68"/>
@@ -6699,7 +6785,7 @@
     <row r="28" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="36"/>
       <c r="G28" s="68" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="H28" s="68"/>
       <c r="I28" s="68"/>
@@ -6720,12 +6806,12 @@
       <c r="G29" s="72"/>
       <c r="H29" s="73"/>
       <c r="I29" s="74" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="L29" s="75"/>
       <c r="M29" s="76"/>
       <c r="N29" s="77" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="V29" s="32"/>
       <c r="W29" s="52"/>
@@ -6737,12 +6823,12 @@
       <c r="H30" s="79"/>
       <c r="I30" s="80"/>
       <c r="L30" s="68" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="M30" s="68"/>
       <c r="N30" s="68"/>
       <c r="R30" s="48" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="S30" s="48"/>
       <c r="T30" s="48"/>
@@ -6753,15 +6839,15 @@
     <row r="31" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C31" s="36"/>
       <c r="D31" s="41" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="E31" s="81"/>
       <c r="G31" s="78" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="H31" s="79"/>
       <c r="I31" s="80" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="L31" s="69" t="s">
         <v>49</v>
@@ -6777,16 +6863,16 @@
       <c r="D32" s="41"/>
       <c r="E32" s="82"/>
       <c r="G32" s="78" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="H32" s="79"/>
       <c r="I32" s="80" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="L32" s="75"/>
       <c r="M32" s="76"/>
       <c r="N32" s="77" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="V32" s="32"/>
       <c r="W32" s="52"/>
@@ -6802,7 +6888,7 @@
         <v>49</v>
       </c>
       <c r="L33" s="68" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="M33" s="68"/>
       <c r="N33" s="68"/>
@@ -6810,7 +6896,7 @@
       <c r="T33" s="84"/>
       <c r="U33" s="40"/>
       <c r="V33" s="85" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="W33" s="52"/>
       <c r="X33" s="32"/>
@@ -6818,19 +6904,19 @@
     <row r="34" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="36"/>
       <c r="G34" s="86" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="H34" s="87"/>
       <c r="I34" s="88"/>
       <c r="L34" s="69"/>
       <c r="M34" s="71" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="S34" s="83"/>
       <c r="T34" s="84"/>
       <c r="U34" s="40"/>
       <c r="V34" s="85" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="W34" s="52"/>
       <c r="X34" s="32"/>
@@ -6843,7 +6929,7 @@
       <c r="T35" s="84"/>
       <c r="U35" s="40"/>
       <c r="V35" s="85" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="W35" s="52"/>
       <c r="X35" s="32"/>
@@ -6862,7 +6948,7 @@
       <c r="T36" s="84"/>
       <c r="U36" s="40"/>
       <c r="V36" s="85" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="W36" s="52"/>
       <c r="X36" s="32"/>
@@ -6870,11 +6956,11 @@
     <row r="37" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C37" s="51"/>
       <c r="E37" s="37" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F37" s="37"/>
       <c r="P37" s="37" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="Q37" s="37"/>
       <c r="V37" s="32"/>

</xml_diff>

<commit_message>
[ Version 0.0.32.1 ] - roulette driver was resoldered. New TODOs were added.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="252">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -757,9 +757,6 @@
   </si>
   <si>
     <t xml:space="preserve">IN2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CD4001BE (NOR)</t>
   </si>
   <si>
     <t xml:space="preserve">BOT 2</t>
@@ -6159,35 +6156,37 @@
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="32"/>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="32"/>
-      <c r="S2" s="32"/>
-      <c r="T2" s="32"/>
-      <c r="U2" s="32"/>
-      <c r="V2" s="32"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
+      <c r="L2" s="34"/>
+      <c r="M2" s="34"/>
+      <c r="N2" s="34"/>
+      <c r="O2" s="34"/>
+      <c r="P2" s="34"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
+      <c r="T2" s="34"/>
+      <c r="U2" s="34"/>
+      <c r="V2" s="35"/>
       <c r="W2" s="32"/>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="32"/>
-      <c r="B3" s="32"/>
+      <c r="B3" s="36"/>
       <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
+      <c r="D3" s="37" t="s">
+        <v>227</v>
+      </c>
+      <c r="E3" s="37"/>
       <c r="F3" s="32"/>
       <c r="G3" s="32"/>
       <c r="H3" s="32"/>
@@ -6204,15 +6203,15 @@
       <c r="S3" s="32"/>
       <c r="T3" s="32"/>
       <c r="U3" s="32"/>
-      <c r="V3" s="32"/>
+      <c r="V3" s="38"/>
       <c r="W3" s="32"/>
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="32"/>
-      <c r="B4" s="32"/>
+      <c r="B4" s="36"/>
       <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="40"/>
       <c r="F4" s="32"/>
       <c r="G4" s="32"/>
       <c r="H4" s="32"/>
@@ -6229,12 +6228,12 @@
       <c r="S4" s="32"/>
       <c r="T4" s="32"/>
       <c r="U4" s="32"/>
-      <c r="V4" s="32"/>
+      <c r="V4" s="38"/>
       <c r="W4" s="32"/>
     </row>
     <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32"/>
-      <c r="B5" s="32"/>
+      <c r="B5" s="36"/>
       <c r="C5" s="32"/>
       <c r="D5" s="32"/>
       <c r="E5" s="32"/>
@@ -6254,15 +6253,21 @@
       <c r="S5" s="32"/>
       <c r="T5" s="32"/>
       <c r="U5" s="32"/>
-      <c r="V5" s="32"/>
+      <c r="V5" s="38"/>
       <c r="W5" s="32"/>
     </row>
     <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32"/>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="41" t="s">
+        <v>228</v>
+      </c>
+      <c r="D6" s="42" t="s">
+        <v>229</v>
+      </c>
+      <c r="E6" s="43" t="s">
+        <v>229</v>
+      </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
       <c r="H6" s="32"/>
@@ -6279,15 +6284,19 @@
       <c r="S6" s="32"/>
       <c r="T6" s="32"/>
       <c r="U6" s="32"/>
-      <c r="V6" s="32"/>
+      <c r="V6" s="38"/>
       <c r="W6" s="32"/>
     </row>
     <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32"/>
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="44" t="s">
+        <v>229</v>
+      </c>
+      <c r="E7" s="45" t="s">
+        <v>229</v>
+      </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
       <c r="H7" s="32"/>
@@ -6304,15 +6313,19 @@
       <c r="S7" s="32"/>
       <c r="T7" s="32"/>
       <c r="U7" s="32"/>
-      <c r="V7" s="32"/>
+      <c r="V7" s="38"/>
       <c r="W7" s="32"/>
     </row>
     <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32"/>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="46" t="s">
+        <v>229</v>
+      </c>
+      <c r="E8" s="47" t="s">
+        <v>229</v>
+      </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
       <c r="H8" s="32"/>
@@ -6324,20 +6337,26 @@
       <c r="N8" s="32"/>
       <c r="O8" s="32"/>
       <c r="P8" s="32"/>
-      <c r="Q8" s="32"/>
-      <c r="R8" s="32"/>
-      <c r="S8" s="32"/>
-      <c r="T8" s="32"/>
+      <c r="Q8" s="48" t="s">
+        <v>230</v>
+      </c>
+      <c r="R8" s="48"/>
+      <c r="S8" s="48"/>
+      <c r="T8" s="48"/>
       <c r="U8" s="32"/>
-      <c r="V8" s="32"/>
+      <c r="V8" s="38"/>
       <c r="W8" s="32"/>
     </row>
     <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32"/>
-      <c r="B9" s="32"/>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="49" t="s">
+        <v>229</v>
+      </c>
+      <c r="E9" s="50" t="s">
+        <v>229</v>
+      </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
       <c r="H9" s="32"/>
@@ -6354,43 +6373,47 @@
       <c r="S9" s="32"/>
       <c r="T9" s="32"/>
       <c r="U9" s="32"/>
-      <c r="V9" s="32"/>
+      <c r="V9" s="38"/>
       <c r="W9" s="32"/>
     </row>
     <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
-      <c r="M10" s="34"/>
-      <c r="N10" s="34"/>
-      <c r="O10" s="34"/>
-      <c r="P10" s="34"/>
-      <c r="Q10" s="34"/>
-      <c r="R10" s="34"/>
-      <c r="S10" s="34"/>
-      <c r="T10" s="34"/>
-      <c r="U10" s="34"/>
-      <c r="V10" s="34"/>
-      <c r="W10" s="35"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="32"/>
+      <c r="K10" s="32"/>
+      <c r="L10" s="32"/>
+      <c r="M10" s="32"/>
+      <c r="N10" s="32"/>
+      <c r="O10" s="32"/>
+      <c r="P10" s="32"/>
+      <c r="Q10" s="32"/>
+      <c r="R10" s="32"/>
+      <c r="S10" s="32"/>
+      <c r="T10" s="32"/>
+      <c r="U10" s="32"/>
+      <c r="V10" s="38"/>
+      <c r="W10" s="0"/>
     </row>
     <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32"/>
-      <c r="B11" s="32"/>
-      <c r="C11" s="36"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="37" t="s">
-        <v>227</v>
-      </c>
-      <c r="F11" s="37"/>
+      <c r="B11" s="36"/>
+      <c r="C11" s="41" t="s">
+        <v>231</v>
+      </c>
+      <c r="D11" s="49" t="s">
+        <v>229</v>
+      </c>
+      <c r="E11" s="50" t="s">
+        <v>229</v>
+      </c>
+      <c r="F11" s="32"/>
       <c r="G11" s="32"/>
       <c r="H11" s="32"/>
       <c r="I11" s="32"/>
@@ -6406,40 +6429,32 @@
       <c r="S11" s="32"/>
       <c r="T11" s="32"/>
       <c r="U11" s="32"/>
-      <c r="V11" s="32"/>
-      <c r="W11" s="38"/>
+      <c r="V11" s="38"/>
+      <c r="W11" s="0"/>
     </row>
     <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32"/>
-      <c r="B12" s="32"/>
-      <c r="C12" s="36"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32"/>
-      <c r="K12" s="32"/>
-      <c r="L12" s="32"/>
-      <c r="M12" s="32"/>
-      <c r="N12" s="32"/>
-      <c r="O12" s="32"/>
-      <c r="P12" s="32"/>
-      <c r="Q12" s="32"/>
-      <c r="R12" s="32"/>
-      <c r="S12" s="32"/>
-      <c r="T12" s="32"/>
-      <c r="U12" s="32"/>
-      <c r="V12" s="32"/>
-      <c r="W12" s="38"/>
+      <c r="B12" s="51"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="46" t="s">
+        <v>229</v>
+      </c>
+      <c r="E12" s="47" t="s">
+        <v>229</v>
+      </c>
+      <c r="V12" s="52"/>
+      <c r="W12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32"/>
-      <c r="B13" s="32"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="44" t="s">
+        <v>229</v>
+      </c>
+      <c r="E13" s="45" t="s">
+        <v>229</v>
+      </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
       <c r="H13" s="32"/>
@@ -6453,542 +6468,534 @@
       <c r="P13" s="32"/>
       <c r="Q13" s="32"/>
       <c r="R13" s="32"/>
-      <c r="S13" s="32"/>
-      <c r="T13" s="32"/>
-      <c r="U13" s="32"/>
-      <c r="V13" s="32"/>
-      <c r="W13" s="38"/>
+      <c r="T13" s="53"/>
+      <c r="U13" s="54" t="s">
+        <v>47</v>
+      </c>
+      <c r="V13" s="52"/>
+      <c r="W13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32"/>
-      <c r="B14" s="32"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="41" t="s">
-        <v>228</v>
-      </c>
-      <c r="E14" s="42" t="s">
+      <c r="B14" s="36"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="42" t="s">
         <v>229</v>
       </c>
-      <c r="F14" s="43" t="s">
+      <c r="E14" s="43" t="s">
         <v>229</v>
       </c>
-      <c r="G14" s="32"/>
-      <c r="H14" s="32"/>
-      <c r="I14" s="32"/>
-      <c r="J14" s="32"/>
-      <c r="K14" s="32"/>
-      <c r="L14" s="32"/>
-      <c r="M14" s="32"/>
-      <c r="N14" s="32"/>
-      <c r="O14" s="32"/>
-      <c r="P14" s="32"/>
-      <c r="Q14" s="32"/>
-      <c r="R14" s="32"/>
-      <c r="S14" s="32"/>
-      <c r="T14" s="32"/>
-      <c r="U14" s="32"/>
-      <c r="V14" s="32"/>
-      <c r="W14" s="38"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
+      <c r="J14" s="55"/>
+      <c r="K14" s="55"/>
+      <c r="L14" s="55"/>
+      <c r="M14" s="55"/>
+      <c r="N14" s="55"/>
+      <c r="O14" s="55"/>
+      <c r="P14" s="55"/>
+      <c r="Q14" s="55"/>
+      <c r="R14" s="55"/>
+      <c r="S14" s="55"/>
+      <c r="T14" s="56"/>
+      <c r="U14" s="54"/>
+      <c r="V14" s="52"/>
+      <c r="W14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32"/>
-      <c r="B15" s="32"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="44" t="s">
-        <v>229</v>
-      </c>
-      <c r="F15" s="45" t="s">
-        <v>229</v>
-      </c>
-      <c r="G15" s="32"/>
-      <c r="H15" s="32"/>
-      <c r="I15" s="32"/>
-      <c r="J15" s="32"/>
-      <c r="K15" s="32"/>
-      <c r="L15" s="32"/>
-      <c r="M15" s="32"/>
-      <c r="N15" s="32"/>
-      <c r="O15" s="32"/>
-      <c r="P15" s="32"/>
-      <c r="Q15" s="32"/>
-      <c r="R15" s="32"/>
-      <c r="S15" s="32"/>
+      <c r="B15" s="36"/>
+      <c r="K15" s="57" t="s">
+        <v>232</v>
+      </c>
       <c r="T15" s="32"/>
       <c r="U15" s="32"/>
-      <c r="V15" s="32"/>
-      <c r="W15" s="38"/>
+      <c r="V15" s="52"/>
+      <c r="W15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32"/>
-      <c r="B16" s="32"/>
-      <c r="C16" s="36"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="46" t="s">
-        <v>229</v>
-      </c>
-      <c r="F16" s="47" t="s">
-        <v>229</v>
-      </c>
-      <c r="G16" s="32"/>
+      <c r="B16" s="36"/>
       <c r="H16" s="32"/>
       <c r="I16" s="32"/>
       <c r="J16" s="32"/>
-      <c r="K16" s="32"/>
-      <c r="L16" s="32"/>
-      <c r="M16" s="32"/>
-      <c r="N16" s="32"/>
-      <c r="O16" s="32"/>
-      <c r="P16" s="32"/>
-      <c r="Q16" s="32"/>
-      <c r="R16" s="48" t="s">
-        <v>230</v>
-      </c>
-      <c r="S16" s="48"/>
-      <c r="T16" s="48"/>
-      <c r="U16" s="48"/>
-      <c r="V16" s="32"/>
-      <c r="W16" s="38"/>
+      <c r="K16" s="58" t="s">
+        <v>44</v>
+      </c>
+      <c r="L16" s="59"/>
+      <c r="M16" s="59"/>
+      <c r="N16" s="59"/>
+      <c r="O16" s="59"/>
+      <c r="P16" s="60"/>
+      <c r="U16" s="32"/>
+      <c r="V16" s="52"/>
+      <c r="W16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="32"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="41"/>
-      <c r="E17" s="49" t="s">
-        <v>229</v>
-      </c>
-      <c r="F17" s="50" t="s">
-        <v>229</v>
-      </c>
-      <c r="G17" s="32"/>
+      <c r="B17" s="36"/>
       <c r="H17" s="32"/>
       <c r="I17" s="32"/>
       <c r="J17" s="32"/>
-      <c r="K17" s="32"/>
-      <c r="L17" s="32"/>
-      <c r="M17" s="32"/>
-      <c r="N17" s="32"/>
-      <c r="O17" s="32"/>
-      <c r="P17" s="32"/>
-      <c r="Q17" s="32"/>
+      <c r="K17" s="61" t="s">
+        <v>233</v>
+      </c>
+      <c r="L17" s="62"/>
+      <c r="M17" s="62"/>
+      <c r="N17" s="62"/>
+      <c r="O17" s="62"/>
+      <c r="P17" s="63"/>
       <c r="R17" s="32"/>
-      <c r="S17" s="32"/>
-      <c r="T17" s="32"/>
-      <c r="U17" s="32"/>
-      <c r="V17" s="32"/>
-      <c r="W17" s="38"/>
+      <c r="T17" s="53"/>
+      <c r="U17" s="54" t="s">
+        <v>44</v>
+      </c>
+      <c r="V17" s="52"/>
+      <c r="W17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="32"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
+      <c r="B18" s="36"/>
       <c r="H18" s="32"/>
       <c r="I18" s="32"/>
       <c r="J18" s="32"/>
-      <c r="K18" s="32"/>
-      <c r="L18" s="32"/>
-      <c r="M18" s="32"/>
-      <c r="N18" s="32"/>
-      <c r="O18" s="32"/>
-      <c r="P18" s="32"/>
-      <c r="Q18" s="32"/>
+      <c r="K18" s="64"/>
+      <c r="L18" s="65"/>
+      <c r="M18" s="65"/>
+      <c r="N18" s="65"/>
+      <c r="O18" s="65"/>
+      <c r="P18" s="66" t="s">
+        <v>49</v>
+      </c>
       <c r="R18" s="32"/>
-      <c r="S18" s="32"/>
-      <c r="T18" s="32"/>
-      <c r="U18" s="32"/>
-      <c r="V18" s="32"/>
-      <c r="W18" s="38"/>
+      <c r="T18" s="67"/>
+      <c r="U18" s="54"/>
+      <c r="V18" s="52"/>
+      <c r="W18" s="0"/>
     </row>
     <row r="19" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="32"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="41" t="s">
-        <v>231</v>
-      </c>
-      <c r="E19" s="49" t="s">
-        <v>229</v>
-      </c>
-      <c r="F19" s="50" t="s">
-        <v>229</v>
-      </c>
+      <c r="B19" s="36"/>
+      <c r="F19" s="32"/>
       <c r="G19" s="32"/>
       <c r="H19" s="32"/>
-      <c r="I19" s="32"/>
-      <c r="J19" s="32"/>
-      <c r="K19" s="32"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="32"/>
-      <c r="N19" s="32"/>
-      <c r="O19" s="32"/>
-      <c r="P19" s="32"/>
-      <c r="Q19" s="32"/>
-      <c r="R19" s="32"/>
-      <c r="S19" s="32"/>
-      <c r="T19" s="32"/>
+      <c r="K19" s="68" t="s">
+        <v>234</v>
+      </c>
+      <c r="L19" s="68"/>
+      <c r="M19" s="68"/>
       <c r="U19" s="32"/>
-      <c r="V19" s="32"/>
-      <c r="W19" s="38"/>
+      <c r="V19" s="52"/>
+      <c r="W19" s="0"/>
     </row>
     <row r="20" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C20" s="51"/>
-      <c r="D20" s="41"/>
-      <c r="E20" s="46" t="s">
-        <v>229</v>
-      </c>
-      <c r="F20" s="47" t="s">
-        <v>229</v>
-      </c>
-      <c r="W20" s="52"/>
+      <c r="B20" s="36"/>
+      <c r="F20" s="68" t="s">
+        <v>235</v>
+      </c>
+      <c r="G20" s="68"/>
+      <c r="H20" s="68"/>
+      <c r="K20" s="69" t="s">
+        <v>49</v>
+      </c>
+      <c r="L20" s="70"/>
+      <c r="M20" s="71"/>
+      <c r="U20" s="32"/>
+      <c r="V20" s="52"/>
+      <c r="W20" s="0"/>
     </row>
     <row r="21" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="32"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="44" t="s">
-        <v>229</v>
-      </c>
-      <c r="F21" s="45" t="s">
-        <v>229</v>
-      </c>
-      <c r="G21" s="32"/>
-      <c r="H21" s="32"/>
-      <c r="I21" s="32"/>
-      <c r="J21" s="32"/>
-      <c r="K21" s="32"/>
-      <c r="L21" s="32"/>
-      <c r="M21" s="32"/>
-      <c r="N21" s="32"/>
-      <c r="O21" s="32"/>
-      <c r="P21" s="32"/>
-      <c r="Q21" s="32"/>
-      <c r="R21" s="32"/>
-      <c r="S21" s="32"/>
-      <c r="U21" s="53"/>
-      <c r="V21" s="54" t="s">
-        <v>47</v>
-      </c>
-      <c r="W21" s="52"/>
+      <c r="B21" s="36"/>
+      <c r="F21" s="72"/>
+      <c r="G21" s="73"/>
+      <c r="H21" s="74" t="s">
+        <v>236</v>
+      </c>
+      <c r="K21" s="75"/>
+      <c r="L21" s="76"/>
+      <c r="M21" s="77" t="s">
+        <v>237</v>
+      </c>
+      <c r="U21" s="32"/>
+      <c r="V21" s="52"/>
+      <c r="W21" s="0"/>
       <c r="X21" s="32"/>
     </row>
     <row r="22" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="36"/>
-      <c r="D22" s="41"/>
-      <c r="E22" s="42" t="s">
-        <v>229</v>
-      </c>
-      <c r="F22" s="43" t="s">
-        <v>229</v>
-      </c>
-      <c r="G22" s="55"/>
-      <c r="H22" s="55"/>
-      <c r="I22" s="55"/>
-      <c r="J22" s="55"/>
-      <c r="K22" s="55"/>
-      <c r="L22" s="55"/>
-      <c r="M22" s="55"/>
-      <c r="N22" s="55"/>
-      <c r="O22" s="55"/>
-      <c r="P22" s="55"/>
-      <c r="Q22" s="55"/>
-      <c r="R22" s="55"/>
-      <c r="S22" s="55"/>
-      <c r="T22" s="55"/>
-      <c r="U22" s="56"/>
-      <c r="V22" s="54"/>
-      <c r="W22" s="52"/>
+      <c r="B22" s="36"/>
+      <c r="F22" s="78"/>
+      <c r="G22" s="79"/>
+      <c r="H22" s="80"/>
+      <c r="K22" s="68" t="s">
+        <v>238</v>
+      </c>
+      <c r="L22" s="68"/>
+      <c r="M22" s="68"/>
+      <c r="Q22" s="48" t="s">
+        <v>239</v>
+      </c>
+      <c r="R22" s="48"/>
+      <c r="S22" s="48"/>
+      <c r="U22" s="32"/>
+      <c r="V22" s="52"/>
+      <c r="W22" s="0"/>
       <c r="X22" s="32"/>
     </row>
     <row r="23" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C23" s="36"/>
-      <c r="L23" s="57" t="s">
-        <v>232</v>
-      </c>
+      <c r="B23" s="36"/>
+      <c r="C23" s="41" t="s">
+        <v>240</v>
+      </c>
+      <c r="D23" s="81"/>
+      <c r="F23" s="78" t="s">
+        <v>241</v>
+      </c>
+      <c r="G23" s="79"/>
+      <c r="H23" s="80" t="s">
+        <v>242</v>
+      </c>
+      <c r="K23" s="69" t="s">
+        <v>49</v>
+      </c>
+      <c r="L23" s="70"/>
+      <c r="M23" s="71"/>
       <c r="U23" s="32"/>
-      <c r="V23" s="32"/>
-      <c r="W23" s="52"/>
+      <c r="V23" s="52"/>
+      <c r="W23" s="0"/>
       <c r="X23" s="32"/>
     </row>
     <row r="24" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C24" s="36"/>
-      <c r="I24" s="32"/>
-      <c r="J24" s="32"/>
-      <c r="K24" s="32"/>
-      <c r="L24" s="58" t="s">
-        <v>44</v>
-      </c>
-      <c r="M24" s="59"/>
-      <c r="N24" s="59"/>
-      <c r="O24" s="59"/>
-      <c r="P24" s="59"/>
-      <c r="Q24" s="60"/>
-      <c r="V24" s="32"/>
-      <c r="W24" s="52"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="82"/>
+      <c r="F24" s="78" t="s">
+        <v>243</v>
+      </c>
+      <c r="G24" s="79"/>
+      <c r="H24" s="80" t="s">
+        <v>244</v>
+      </c>
+      <c r="K24" s="75"/>
+      <c r="L24" s="76"/>
+      <c r="M24" s="77" t="s">
+        <v>237</v>
+      </c>
+      <c r="U24" s="32"/>
+      <c r="V24" s="52"/>
+      <c r="W24" s="0"/>
       <c r="X24" s="32"/>
     </row>
     <row r="25" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C25" s="36"/>
-      <c r="I25" s="32"/>
-      <c r="J25" s="32"/>
-      <c r="K25" s="32"/>
-      <c r="L25" s="61" t="s">
-        <v>233</v>
-      </c>
-      <c r="M25" s="62"/>
-      <c r="N25" s="62"/>
-      <c r="O25" s="62"/>
-      <c r="P25" s="62"/>
-      <c r="Q25" s="63"/>
-      <c r="S25" s="32"/>
-      <c r="U25" s="53"/>
-      <c r="V25" s="54" t="s">
-        <v>44</v>
-      </c>
-      <c r="W25" s="52"/>
+      <c r="B25" s="36"/>
+      <c r="F25" s="78" t="s">
+        <v>49</v>
+      </c>
+      <c r="G25" s="79"/>
+      <c r="H25" s="80" t="s">
+        <v>49</v>
+      </c>
+      <c r="K25" s="68" t="s">
+        <v>234</v>
+      </c>
+      <c r="L25" s="68"/>
+      <c r="M25" s="68"/>
+      <c r="R25" s="83"/>
+      <c r="S25" s="84"/>
+      <c r="T25" s="40"/>
+      <c r="U25" s="85" t="s">
+        <v>245</v>
+      </c>
+      <c r="V25" s="52"/>
+      <c r="W25" s="0"/>
       <c r="X25" s="32"/>
     </row>
     <row r="26" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C26" s="36"/>
-      <c r="I26" s="32"/>
-      <c r="J26" s="32"/>
-      <c r="K26" s="32"/>
-      <c r="L26" s="64"/>
-      <c r="M26" s="65"/>
-      <c r="N26" s="65"/>
-      <c r="O26" s="65"/>
-      <c r="P26" s="65"/>
-      <c r="Q26" s="66" t="s">
+      <c r="B26" s="36"/>
+      <c r="F26" s="86" t="s">
+        <v>246</v>
+      </c>
+      <c r="G26" s="87"/>
+      <c r="H26" s="88"/>
+      <c r="K26" s="69"/>
+      <c r="L26" s="71" t="s">
+        <v>237</v>
+      </c>
+      <c r="R26" s="83"/>
+      <c r="S26" s="84"/>
+      <c r="T26" s="40"/>
+      <c r="U26" s="85" t="s">
+        <v>247</v>
+      </c>
+      <c r="V26" s="52"/>
+      <c r="W26" s="0"/>
+      <c r="X26" s="32"/>
+    </row>
+    <row r="27" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="36"/>
+      <c r="K27" s="89"/>
+      <c r="L27" s="90"/>
+      <c r="R27" s="83"/>
+      <c r="S27" s="84"/>
+      <c r="T27" s="40"/>
+      <c r="U27" s="85" t="s">
+        <v>248</v>
+      </c>
+      <c r="V27" s="52"/>
+      <c r="W27" s="0"/>
+      <c r="X27" s="32"/>
+    </row>
+    <row r="28" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="36"/>
+      <c r="D28" s="39"/>
+      <c r="E28" s="40"/>
+      <c r="K28" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="S26" s="32"/>
-      <c r="U26" s="67"/>
-      <c r="V26" s="54"/>
-      <c r="W26" s="52"/>
-      <c r="X26" s="32"/>
-    </row>
-    <row r="27" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="36"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="32"/>
-      <c r="I27" s="32"/>
-      <c r="L27" s="68" t="s">
-        <v>234</v>
-      </c>
-      <c r="M27" s="68"/>
-      <c r="N27" s="68"/>
-      <c r="V27" s="32"/>
-      <c r="W27" s="52"/>
-      <c r="X27" s="32"/>
-    </row>
-    <row r="28" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="36"/>
-      <c r="G28" s="68" t="s">
-        <v>235</v>
-      </c>
-      <c r="H28" s="68"/>
-      <c r="I28" s="68"/>
-      <c r="L28" s="69" t="s">
-        <v>49</v>
-      </c>
-      <c r="M28" s="70"/>
-      <c r="N28" s="71"/>
-      <c r="V28" s="32"/>
-      <c r="W28" s="52"/>
+      <c r="L28" s="77"/>
+      <c r="O28" s="39"/>
+      <c r="P28" s="40"/>
+      <c r="R28" s="83"/>
+      <c r="S28" s="84"/>
+      <c r="T28" s="40"/>
+      <c r="U28" s="85" t="s">
+        <v>249</v>
+      </c>
+      <c r="V28" s="52"/>
+      <c r="W28" s="0"/>
       <c r="X28" s="32"/>
       <c r="AF28" s="32"/>
       <c r="AG28" s="32"/>
       <c r="AH28" s="32"/>
     </row>
     <row r="29" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C29" s="36"/>
-      <c r="G29" s="72"/>
-      <c r="H29" s="73"/>
-      <c r="I29" s="74" t="s">
-        <v>236</v>
-      </c>
-      <c r="L29" s="75"/>
-      <c r="M29" s="76"/>
-      <c r="N29" s="77" t="s">
-        <v>237</v>
-      </c>
-      <c r="V29" s="32"/>
-      <c r="W29" s="52"/>
+      <c r="B29" s="51"/>
+      <c r="D29" s="37" t="s">
+        <v>250</v>
+      </c>
+      <c r="E29" s="37"/>
+      <c r="O29" s="37" t="s">
+        <v>251</v>
+      </c>
+      <c r="P29" s="37"/>
+      <c r="U29" s="32"/>
+      <c r="V29" s="52"/>
+      <c r="W29" s="0"/>
       <c r="X29" s="32"/>
     </row>
     <row r="30" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C30" s="36"/>
-      <c r="G30" s="78"/>
-      <c r="H30" s="79"/>
-      <c r="I30" s="80"/>
-      <c r="L30" s="68" t="s">
-        <v>238</v>
-      </c>
-      <c r="M30" s="68"/>
-      <c r="N30" s="68"/>
-      <c r="R30" s="48" t="s">
-        <v>239</v>
-      </c>
-      <c r="S30" s="48"/>
-      <c r="T30" s="48"/>
-      <c r="V30" s="32"/>
-      <c r="W30" s="52"/>
+      <c r="B30" s="91"/>
+      <c r="C30" s="92"/>
+      <c r="D30" s="92"/>
+      <c r="E30" s="92"/>
+      <c r="F30" s="92"/>
+      <c r="G30" s="92"/>
+      <c r="H30" s="92"/>
+      <c r="I30" s="92"/>
+      <c r="J30" s="92"/>
+      <c r="K30" s="92"/>
+      <c r="L30" s="92"/>
+      <c r="M30" s="92"/>
+      <c r="N30" s="92"/>
+      <c r="O30" s="92"/>
+      <c r="P30" s="92"/>
+      <c r="Q30" s="92"/>
+      <c r="R30" s="92"/>
+      <c r="S30" s="92"/>
+      <c r="T30" s="92"/>
+      <c r="U30" s="92"/>
+      <c r="V30" s="93"/>
+      <c r="W30" s="0"/>
       <c r="X30" s="32"/>
     </row>
     <row r="31" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="36"/>
-      <c r="D31" s="41" t="s">
-        <v>240</v>
-      </c>
-      <c r="E31" s="81"/>
-      <c r="G31" s="78" t="s">
-        <v>241</v>
-      </c>
-      <c r="H31" s="79"/>
-      <c r="I31" s="80" t="s">
-        <v>242</v>
-      </c>
-      <c r="L31" s="69" t="s">
-        <v>49</v>
-      </c>
-      <c r="M31" s="70"/>
-      <c r="N31" s="71"/>
-      <c r="V31" s="32"/>
-      <c r="W31" s="52"/>
+      <c r="C31" s="0"/>
+      <c r="D31" s="0"/>
+      <c r="E31" s="0"/>
+      <c r="F31" s="0"/>
+      <c r="G31" s="0"/>
+      <c r="H31" s="0"/>
+      <c r="I31" s="0"/>
+      <c r="J31" s="0"/>
+      <c r="K31" s="0"/>
+      <c r="L31" s="0"/>
+      <c r="M31" s="0"/>
+      <c r="N31" s="0"/>
+      <c r="O31" s="0"/>
+      <c r="P31" s="0"/>
+      <c r="Q31" s="0"/>
+      <c r="R31" s="0"/>
+      <c r="S31" s="0"/>
+      <c r="T31" s="0"/>
+      <c r="U31" s="0"/>
+      <c r="V31" s="0"/>
+      <c r="W31" s="0"/>
       <c r="X31" s="32"/>
     </row>
     <row r="32" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="36"/>
-      <c r="D32" s="41"/>
-      <c r="E32" s="82"/>
-      <c r="G32" s="78" t="s">
-        <v>243</v>
-      </c>
-      <c r="H32" s="79"/>
-      <c r="I32" s="80" t="s">
-        <v>244</v>
-      </c>
-      <c r="L32" s="75"/>
-      <c r="M32" s="76"/>
-      <c r="N32" s="77" t="s">
-        <v>237</v>
-      </c>
-      <c r="V32" s="32"/>
-      <c r="W32" s="52"/>
+      <c r="C32" s="0"/>
+      <c r="D32" s="0"/>
+      <c r="E32" s="0"/>
+      <c r="F32" s="0"/>
+      <c r="G32" s="0"/>
+      <c r="H32" s="0"/>
+      <c r="I32" s="0"/>
+      <c r="J32" s="0"/>
+      <c r="K32" s="0"/>
+      <c r="L32" s="0"/>
+      <c r="M32" s="0"/>
+      <c r="N32" s="0"/>
+      <c r="O32" s="0"/>
+      <c r="P32" s="0"/>
+      <c r="Q32" s="0"/>
+      <c r="R32" s="0"/>
+      <c r="S32" s="0"/>
+      <c r="T32" s="0"/>
+      <c r="U32" s="0"/>
+      <c r="V32" s="0"/>
+      <c r="W32" s="0"/>
       <c r="X32" s="32"/>
     </row>
     <row r="33" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="36"/>
-      <c r="G33" s="78" t="s">
-        <v>49</v>
-      </c>
-      <c r="H33" s="79"/>
-      <c r="I33" s="80" t="s">
-        <v>49</v>
-      </c>
-      <c r="L33" s="68" t="s">
-        <v>245</v>
-      </c>
-      <c r="M33" s="68"/>
-      <c r="N33" s="68"/>
-      <c r="S33" s="83"/>
-      <c r="T33" s="84"/>
-      <c r="U33" s="40"/>
-      <c r="V33" s="85" t="s">
-        <v>246</v>
-      </c>
-      <c r="W33" s="52"/>
+      <c r="C33" s="0"/>
+      <c r="D33" s="0"/>
+      <c r="E33" s="0"/>
+      <c r="F33" s="0"/>
+      <c r="G33" s="0"/>
+      <c r="H33" s="0"/>
+      <c r="I33" s="0"/>
+      <c r="J33" s="0"/>
+      <c r="K33" s="0"/>
+      <c r="L33" s="0"/>
+      <c r="M33" s="0"/>
+      <c r="N33" s="0"/>
+      <c r="O33" s="0"/>
+      <c r="P33" s="0"/>
+      <c r="Q33" s="0"/>
+      <c r="R33" s="0"/>
+      <c r="S33" s="0"/>
+      <c r="T33" s="0"/>
+      <c r="U33" s="0"/>
+      <c r="V33" s="0"/>
+      <c r="W33" s="0"/>
       <c r="X33" s="32"/>
     </row>
     <row r="34" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="36"/>
-      <c r="G34" s="86" t="s">
-        <v>247</v>
-      </c>
-      <c r="H34" s="87"/>
-      <c r="I34" s="88"/>
-      <c r="L34" s="69"/>
-      <c r="M34" s="71" t="s">
-        <v>237</v>
-      </c>
-      <c r="S34" s="83"/>
-      <c r="T34" s="84"/>
-      <c r="U34" s="40"/>
-      <c r="V34" s="85" t="s">
-        <v>248</v>
-      </c>
-      <c r="W34" s="52"/>
+      <c r="C34" s="0"/>
+      <c r="D34" s="0"/>
+      <c r="E34" s="0"/>
+      <c r="F34" s="0"/>
+      <c r="G34" s="0"/>
+      <c r="H34" s="0"/>
+      <c r="I34" s="0"/>
+      <c r="J34" s="0"/>
+      <c r="K34" s="0"/>
+      <c r="L34" s="0"/>
+      <c r="M34" s="0"/>
+      <c r="N34" s="0"/>
+      <c r="O34" s="0"/>
+      <c r="P34" s="0"/>
+      <c r="Q34" s="0"/>
+      <c r="R34" s="0"/>
+      <c r="S34" s="0"/>
+      <c r="T34" s="0"/>
+      <c r="U34" s="0"/>
+      <c r="V34" s="0"/>
+      <c r="W34" s="0"/>
       <c r="X34" s="32"/>
     </row>
     <row r="35" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C35" s="36"/>
-      <c r="L35" s="89"/>
-      <c r="M35" s="90"/>
-      <c r="S35" s="83"/>
-      <c r="T35" s="84"/>
-      <c r="U35" s="40"/>
-      <c r="V35" s="85" t="s">
-        <v>249</v>
-      </c>
-      <c r="W35" s="52"/>
+      <c r="C35" s="0"/>
+      <c r="D35" s="0"/>
+      <c r="E35" s="0"/>
+      <c r="F35" s="0"/>
+      <c r="G35" s="0"/>
+      <c r="H35" s="0"/>
+      <c r="I35" s="0"/>
+      <c r="J35" s="0"/>
+      <c r="K35" s="0"/>
+      <c r="L35" s="0"/>
+      <c r="M35" s="0"/>
+      <c r="N35" s="0"/>
+      <c r="O35" s="0"/>
+      <c r="P35" s="0"/>
+      <c r="Q35" s="0"/>
+      <c r="R35" s="0"/>
+      <c r="S35" s="0"/>
+      <c r="T35" s="0"/>
+      <c r="U35" s="0"/>
+      <c r="V35" s="0"/>
+      <c r="W35" s="0"/>
       <c r="X35" s="32"/>
     </row>
     <row r="36" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C36" s="36"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="40"/>
-      <c r="L36" s="75" t="s">
-        <v>49</v>
-      </c>
-      <c r="M36" s="77"/>
-      <c r="P36" s="39"/>
-      <c r="Q36" s="40"/>
-      <c r="S36" s="83"/>
-      <c r="T36" s="84"/>
-      <c r="U36" s="40"/>
-      <c r="V36" s="85" t="s">
-        <v>250</v>
-      </c>
-      <c r="W36" s="52"/>
+      <c r="C36" s="0"/>
+      <c r="D36" s="0"/>
+      <c r="E36" s="0"/>
+      <c r="F36" s="0"/>
+      <c r="G36" s="0"/>
+      <c r="H36" s="0"/>
+      <c r="I36" s="0"/>
+      <c r="J36" s="0"/>
+      <c r="K36" s="0"/>
+      <c r="L36" s="0"/>
+      <c r="M36" s="0"/>
+      <c r="N36" s="0"/>
+      <c r="O36" s="0"/>
+      <c r="P36" s="0"/>
+      <c r="Q36" s="0"/>
+      <c r="R36" s="0"/>
+      <c r="S36" s="0"/>
+      <c r="T36" s="0"/>
+      <c r="U36" s="0"/>
+      <c r="V36" s="0"/>
+      <c r="W36" s="0"/>
       <c r="X36" s="32"/>
     </row>
     <row r="37" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C37" s="51"/>
-      <c r="E37" s="37" t="s">
-        <v>251</v>
-      </c>
-      <c r="F37" s="37"/>
-      <c r="P37" s="37" t="s">
-        <v>252</v>
-      </c>
-      <c r="Q37" s="37"/>
-      <c r="V37" s="32"/>
-      <c r="W37" s="52"/>
+      <c r="C37" s="0"/>
+      <c r="D37" s="0"/>
+      <c r="E37" s="0"/>
+      <c r="F37" s="0"/>
+      <c r="G37" s="0"/>
+      <c r="H37" s="0"/>
+      <c r="I37" s="0"/>
+      <c r="J37" s="0"/>
+      <c r="K37" s="0"/>
+      <c r="L37" s="0"/>
+      <c r="M37" s="0"/>
+      <c r="N37" s="0"/>
+      <c r="O37" s="0"/>
+      <c r="P37" s="0"/>
+      <c r="Q37" s="0"/>
+      <c r="R37" s="0"/>
+      <c r="S37" s="0"/>
+      <c r="T37" s="0"/>
+      <c r="U37" s="0"/>
+      <c r="V37" s="0"/>
+      <c r="W37" s="0"/>
       <c r="X37" s="32"/>
     </row>
     <row r="38" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C38" s="91"/>
-      <c r="D38" s="92"/>
-      <c r="E38" s="92"/>
-      <c r="F38" s="92"/>
-      <c r="G38" s="92"/>
-      <c r="H38" s="92"/>
-      <c r="I38" s="92"/>
-      <c r="J38" s="92"/>
-      <c r="K38" s="92"/>
-      <c r="L38" s="92"/>
-      <c r="M38" s="92"/>
-      <c r="N38" s="92"/>
-      <c r="O38" s="92"/>
-      <c r="P38" s="92"/>
-      <c r="Q38" s="92"/>
-      <c r="R38" s="92"/>
-      <c r="S38" s="92"/>
-      <c r="T38" s="92"/>
-      <c r="U38" s="92"/>
-      <c r="V38" s="92"/>
-      <c r="W38" s="93"/>
+      <c r="C38" s="0"/>
+      <c r="D38" s="0"/>
+      <c r="E38" s="0"/>
+      <c r="F38" s="0"/>
+      <c r="G38" s="0"/>
+      <c r="H38" s="0"/>
+      <c r="I38" s="0"/>
+      <c r="J38" s="0"/>
+      <c r="K38" s="0"/>
+      <c r="L38" s="0"/>
+      <c r="M38" s="0"/>
+      <c r="N38" s="0"/>
+      <c r="O38" s="0"/>
+      <c r="P38" s="0"/>
+      <c r="Q38" s="0"/>
+      <c r="R38" s="0"/>
+      <c r="S38" s="0"/>
+      <c r="T38" s="0"/>
+      <c r="U38" s="0"/>
+      <c r="V38" s="0"/>
+      <c r="W38" s="0"/>
       <c r="X38" s="32"/>
     </row>
     <row r="39" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6996,20 +7003,20 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="R16:U16"/>
-    <mergeCell ref="D19:D22"/>
-    <mergeCell ref="V21:V22"/>
-    <mergeCell ref="V25:V26"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="R30:T30"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="P37:Q37"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="Q8:T8"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="U13:U14"/>
+    <mergeCell ref="U17:U18"/>
+    <mergeCell ref="K19:M19"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="K22:M22"/>
+    <mergeCell ref="Q22:S22"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="K25:M25"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="O29:P29"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
[ Version 0.0.32.2 ] - roulette driver code was rewrite as FSM. Everything were tested.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="250">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -675,34 +675,28 @@
     <t xml:space="preserve">roulette_dataset_t</t>
   </si>
   <si>
-    <t xml:space="preserve">esp_timer_handle_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">power_cut_off_timer</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dataset structure which store roulette runtime properties.</t>
   </si>
   <si>
-    <t xml:space="preserve">event_start_tick</t>
-  </si>
-  <si>
-    <t xml:space="preserve">control_flags</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIZE [bytes]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BYTE NUMBER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LSB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROULETTE R1 ENABLE </t>
+    <t xml:space="preserve">r1_opn_ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r1_cls_ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROULETTE 1 ENABLED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACKNOWLEDGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DUPONT connector – TOP view</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIGNAL</t>
   </si>
   <si>
     <t xml:space="preserve">6V</t>
@@ -787,7 +781,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -860,8 +854,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b val="true"/>
-      <i val="true"/>
+      <u val="single"/>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -869,7 +868,7 @@
     </font>
     <font>
       <b val="true"/>
-      <u val="single"/>
+      <i val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -997,14 +996,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF000000"/>
-        <bgColor rgb="FF003300"/>
+        <fgColor rgb="FFF44336"/>
+        <bgColor rgb="FF993366"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF44336"/>
-        <bgColor rgb="FF993366"/>
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF003300"/>
       </patternFill>
     </fill>
     <fill>
@@ -1050,14 +1049,14 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
+      <left/>
       <right/>
       <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left/>
+      <left style="thin"/>
       <right/>
       <top style="thin"/>
       <bottom/>
@@ -1152,7 +1151,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="99">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1277,7 +1276,35 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="15" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="14" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="14" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1285,14 +1312,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1309,39 +1336,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="180" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="15" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1349,11 +1376,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1362,10 +1389,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1377,19 +1400,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1421,7 +1440,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1429,11 +1448,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1441,14 +1460,14 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1477,11 +1496,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1489,11 +1508,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2396,7 +2415,7 @@
     <tabColor rgb="FFFDD835"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AC123"/>
+  <dimension ref="A1:AC163"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5383,7 +5402,7 @@
       <c r="F115" s="5"/>
       <c r="G115" s="5"/>
       <c r="H115" s="5" t="s">
-        <v>217</v>
+        <v>138</v>
       </c>
       <c r="I115" s="5" t="s">
         <v>109</v>
@@ -5392,16 +5411,12 @@
         <v>109</v>
       </c>
       <c r="K115" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="L115" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="M115" s="5" t="s">
-        <v>109</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="L115" s="5"/>
+      <c r="M115" s="5"/>
       <c r="N115" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="O115" s="5"/>
       <c r="P115" s="5"/>
@@ -5420,23 +5435,15 @@
       <c r="F116" s="5"/>
       <c r="G116" s="5"/>
       <c r="H116" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="I116" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="J116" s="5" t="s">
-        <v>109</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="I116" s="5"/>
+      <c r="J116" s="5"/>
       <c r="K116" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="L116" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="M116" s="5" t="s">
-        <v>109</v>
-      </c>
+        <v>218</v>
+      </c>
+      <c r="L116" s="5"/>
+      <c r="M116" s="5"/>
       <c r="N116" s="5"/>
       <c r="O116" s="5"/>
       <c r="P116" s="5"/>
@@ -5455,23 +5462,15 @@
       <c r="F117" s="5"/>
       <c r="G117" s="5"/>
       <c r="H117" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="I117" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="J117" s="5" t="s">
-        <v>109</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="I117" s="5"/>
+      <c r="J117" s="5"/>
       <c r="K117" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="L117" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="M117" s="5" t="s">
-        <v>109</v>
-      </c>
+        <v>219</v>
+      </c>
+      <c r="L117" s="5"/>
+      <c r="M117" s="5"/>
       <c r="N117" s="5"/>
       <c r="O117" s="5"/>
       <c r="P117" s="5"/>
@@ -5481,238 +5480,1080 @@
       <c r="T117" s="5"/>
       <c r="U117" s="5"/>
     </row>
-    <row r="118" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="2"/>
-      <c r="B118" s="2"/>
-      <c r="C118" s="2"/>
-      <c r="D118" s="2"/>
-      <c r="E118" s="2"/>
-      <c r="F118" s="2"/>
-      <c r="G118" s="2"/>
-      <c r="H118" s="2"/>
-      <c r="I118" s="2"/>
-      <c r="J118" s="2"/>
-      <c r="K118" s="2"/>
-      <c r="L118" s="2"/>
-      <c r="M118" s="2"/>
-      <c r="N118" s="2"/>
-      <c r="O118" s="2"/>
-      <c r="P118" s="2"/>
-      <c r="Q118" s="2"/>
-      <c r="R118" s="2"/>
-      <c r="S118" s="2"/>
-      <c r="T118" s="2"/>
-      <c r="U118" s="2"/>
-    </row>
-    <row r="119" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A119" s="6" t="s">
+    <row r="118" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A118" s="9"/>
+      <c r="B118" s="5"/>
+      <c r="C118" s="5"/>
+      <c r="D118" s="5"/>
+      <c r="E118" s="5"/>
+      <c r="F118" s="5"/>
+      <c r="G118" s="5"/>
+      <c r="H118" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="I118" s="5"/>
+      <c r="J118" s="5"/>
+      <c r="K118" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="L118" s="5"/>
+      <c r="M118" s="5"/>
+      <c r="N118" s="5"/>
+      <c r="O118" s="5"/>
+      <c r="P118" s="5"/>
+      <c r="Q118" s="5"/>
+      <c r="R118" s="5"/>
+      <c r="S118" s="5"/>
+      <c r="T118" s="5"/>
+      <c r="U118" s="5"/>
+    </row>
+    <row r="119" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A119" s="9"/>
+      <c r="B119" s="5"/>
+      <c r="C119" s="5"/>
+      <c r="D119" s="5"/>
+      <c r="E119" s="5"/>
+      <c r="F119" s="5"/>
+      <c r="G119" s="5"/>
+      <c r="H119" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="I119" s="5"/>
+      <c r="J119" s="5"/>
+      <c r="K119" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="L119" s="5"/>
+      <c r="M119" s="5"/>
+      <c r="N119" s="5"/>
+      <c r="O119" s="5"/>
+      <c r="P119" s="5"/>
+      <c r="Q119" s="5"/>
+      <c r="R119" s="5"/>
+      <c r="S119" s="5"/>
+      <c r="T119" s="5"/>
+      <c r="U119" s="5"/>
+    </row>
+    <row r="120" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A120" s="9"/>
+      <c r="B120" s="5"/>
+      <c r="C120" s="5"/>
+      <c r="D120" s="5"/>
+      <c r="E120" s="5"/>
+      <c r="F120" s="5"/>
+      <c r="G120" s="5"/>
+      <c r="H120" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="I120" s="5"/>
+      <c r="J120" s="5"/>
+      <c r="K120" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="L120" s="5"/>
+      <c r="M120" s="5"/>
+      <c r="N120" s="5"/>
+      <c r="O120" s="5"/>
+      <c r="P120" s="5"/>
+      <c r="Q120" s="5"/>
+      <c r="R120" s="5"/>
+      <c r="S120" s="5"/>
+      <c r="T120" s="5"/>
+      <c r="U120" s="5"/>
+    </row>
+    <row r="121" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A121" s="2"/>
+      <c r="B121" s="2"/>
+      <c r="C121" s="2"/>
+      <c r="D121" s="2"/>
+      <c r="E121" s="2"/>
+      <c r="F121" s="2"/>
+      <c r="G121" s="2"/>
+      <c r="H121" s="2"/>
+      <c r="I121" s="2"/>
+      <c r="J121" s="2"/>
+      <c r="K121" s="2"/>
+      <c r="L121" s="2"/>
+      <c r="M121" s="2"/>
+      <c r="N121" s="2"/>
+      <c r="O121" s="2"/>
+      <c r="P121" s="2"/>
+      <c r="Q121" s="2"/>
+      <c r="R121" s="2"/>
+      <c r="S121" s="2"/>
+      <c r="T121" s="2"/>
+      <c r="U121" s="2"/>
+    </row>
+    <row r="122" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A122" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="B119" s="6"/>
-      <c r="C119" s="6"/>
-      <c r="D119" s="6"/>
-      <c r="E119" s="6"/>
-      <c r="F119" s="6"/>
-      <c r="G119" s="6"/>
-      <c r="H119" s="6"/>
-      <c r="I119" s="6"/>
-      <c r="J119" s="6"/>
-      <c r="K119" s="6"/>
-      <c r="L119" s="6"/>
-      <c r="M119" s="6"/>
-      <c r="N119" s="6"/>
-      <c r="O119" s="6"/>
-      <c r="P119" s="6"/>
-      <c r="Q119" s="6"/>
-      <c r="R119" s="6"/>
-      <c r="S119" s="6"/>
-      <c r="T119" s="6"/>
-      <c r="U119" s="6"/>
-      <c r="V119" s="6"/>
-      <c r="W119" s="6"/>
-      <c r="X119" s="6"/>
-      <c r="Y119" s="6"/>
-      <c r="Z119" s="6"/>
-      <c r="AA119" s="6"/>
-      <c r="AB119" s="6"/>
-      <c r="AC119" s="6"/>
-    </row>
-    <row r="120" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A120" s="4" t="s">
+      <c r="B122" s="6"/>
+      <c r="C122" s="6"/>
+      <c r="D122" s="6"/>
+      <c r="E122" s="6"/>
+      <c r="F122" s="6"/>
+      <c r="G122" s="6"/>
+      <c r="H122" s="6"/>
+      <c r="I122" s="6"/>
+      <c r="J122" s="6"/>
+      <c r="K122" s="6"/>
+      <c r="L122" s="6"/>
+      <c r="M122" s="6"/>
+      <c r="N122" s="6"/>
+      <c r="O122" s="6"/>
+      <c r="P122" s="6"/>
+      <c r="Q122" s="6"/>
+      <c r="R122" s="6"/>
+      <c r="S122" s="6"/>
+      <c r="T122" s="6"/>
+      <c r="U122" s="6"/>
+      <c r="V122" s="6"/>
+      <c r="W122" s="6"/>
+      <c r="X122" s="6"/>
+      <c r="Y122" s="6"/>
+      <c r="Z122" s="6"/>
+      <c r="AA122" s="6"/>
+      <c r="AB122" s="6"/>
+      <c r="AC122" s="6"/>
+    </row>
+    <row r="123" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A123" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B120" s="4" t="s">
+      <c r="B123" s="4"/>
+      <c r="C123" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D123" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="E123" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="F123" s="4"/>
+      <c r="G123" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H123" s="4"/>
+      <c r="I123" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="J123" s="4"/>
+      <c r="L123" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="M123" s="4"/>
+      <c r="N123" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="O123" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="P123" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q123" s="4"/>
+      <c r="R123" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="S123" s="4"/>
+      <c r="T123" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="U123" s="4"/>
+    </row>
+    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B124" s="9"/>
+      <c r="C124" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E124" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F124" s="9"/>
+      <c r="G124" s="9"/>
+      <c r="H124" s="9"/>
+      <c r="I124" s="9"/>
+      <c r="J124" s="9"/>
+      <c r="L124" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="M124" s="9"/>
+      <c r="N124" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O124" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="P124" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q124" s="5"/>
+      <c r="R124" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="S124" s="5"/>
+      <c r="T124" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="U124" s="5"/>
+    </row>
+    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C125" s="9"/>
+      <c r="D125" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E125" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F125" s="9"/>
+      <c r="G125" s="9"/>
+      <c r="H125" s="9"/>
+      <c r="I125" s="9"/>
+      <c r="J125" s="9"/>
+      <c r="N125" s="9"/>
+      <c r="O125" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="P125" s="5"/>
+      <c r="Q125" s="5"/>
+      <c r="R125" s="5"/>
+      <c r="S125" s="5"/>
+      <c r="T125" s="5"/>
+      <c r="U125" s="5"/>
+    </row>
+    <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="C120" s="4"/>
-      <c r="D120" s="4"/>
-      <c r="E120" s="4" t="s">
+      <c r="B126" s="4"/>
+      <c r="C126" s="9"/>
+      <c r="D126" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="E126" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F126" s="9"/>
+      <c r="G126" s="9"/>
+      <c r="H126" s="9"/>
+      <c r="I126" s="9"/>
+      <c r="J126" s="9"/>
+      <c r="L126" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="M126" s="4"/>
+      <c r="N126" s="9"/>
+      <c r="O126" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="P126" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q126" s="9"/>
+      <c r="R126" s="9"/>
+      <c r="S126" s="9"/>
+      <c r="T126" s="9"/>
+      <c r="U126" s="9"/>
+    </row>
+    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="31" t="s">
+        <v>216</v>
+      </c>
+      <c r="B127" s="31"/>
+      <c r="C127" s="9"/>
+      <c r="D127" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E127" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F127" s="9"/>
+      <c r="G127" s="9"/>
+      <c r="H127" s="9"/>
+      <c r="I127" s="9"/>
+      <c r="J127" s="9"/>
+      <c r="L127" s="31" t="s">
+        <v>216</v>
+      </c>
+      <c r="M127" s="31"/>
+      <c r="N127" s="9"/>
+      <c r="O127" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="P127" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q127" s="9"/>
+      <c r="R127" s="9"/>
+      <c r="S127" s="9"/>
+      <c r="T127" s="9"/>
+      <c r="U127" s="9"/>
+    </row>
+    <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C128" s="9"/>
+      <c r="D128" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E128" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F128" s="9"/>
+      <c r="G128" s="9"/>
+      <c r="H128" s="9"/>
+      <c r="I128" s="9"/>
+      <c r="J128" s="9"/>
+      <c r="N128" s="9"/>
+      <c r="O128" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="P128" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="Q128" s="9"/>
+      <c r="R128" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="S128" s="9"/>
+      <c r="T128" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="U128" s="9"/>
+    </row>
+    <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="F120" s="4"/>
-      <c r="G120" s="4"/>
-      <c r="H120" s="4" t="s">
+      <c r="B129" s="4"/>
+      <c r="C129" s="9"/>
+      <c r="D129" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="E129" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F129" s="9"/>
+      <c r="G129" s="9"/>
+      <c r="H129" s="9"/>
+      <c r="I129" s="9"/>
+      <c r="J129" s="9"/>
+      <c r="L129" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="M129" s="4"/>
+      <c r="N129" s="9"/>
+      <c r="O129" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="P129" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q129" s="9"/>
+      <c r="R129" s="9"/>
+      <c r="S129" s="9"/>
+      <c r="T129" s="9"/>
+      <c r="U129" s="9"/>
+    </row>
+    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B130" s="5"/>
+      <c r="C130" s="9"/>
+      <c r="D130" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="E130" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F130" s="9"/>
+      <c r="G130" s="9"/>
+      <c r="H130" s="9"/>
+      <c r="I130" s="9"/>
+      <c r="J130" s="9"/>
+      <c r="L130" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="M130" s="5"/>
+      <c r="N130" s="9"/>
+      <c r="O130" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="P130" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q130" s="9"/>
+      <c r="R130" s="9"/>
+      <c r="S130" s="9"/>
+      <c r="T130" s="9"/>
+      <c r="U130" s="9"/>
+    </row>
+    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C131" s="9"/>
+      <c r="D131" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="E131" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F131" s="9"/>
+      <c r="G131" s="9"/>
+      <c r="H131" s="9"/>
+      <c r="I131" s="9"/>
+      <c r="J131" s="9"/>
+      <c r="N131" s="9"/>
+      <c r="O131" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="P131" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q131" s="9"/>
+      <c r="R131" s="9"/>
+      <c r="S131" s="9"/>
+      <c r="T131" s="9"/>
+      <c r="U131" s="9"/>
+    </row>
+    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B132" s="4"/>
+      <c r="C132" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D132" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="E132" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F132" s="9"/>
+      <c r="G132" s="9"/>
+      <c r="H132" s="9"/>
+      <c r="I132" s="9"/>
+      <c r="J132" s="9"/>
+      <c r="L132" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="M132" s="4"/>
+      <c r="N132" s="9"/>
+      <c r="O132" s="4"/>
+      <c r="P132" s="9"/>
+      <c r="Q132" s="9"/>
+      <c r="R132" s="9"/>
+      <c r="S132" s="9"/>
+      <c r="T132" s="9"/>
+      <c r="U132" s="9"/>
+    </row>
+    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B133" s="5"/>
+      <c r="C133" s="9"/>
+      <c r="D133" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="E133" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F133" s="9"/>
+      <c r="G133" s="9"/>
+      <c r="H133" s="9"/>
+      <c r="I133" s="9"/>
+      <c r="J133" s="9"/>
+      <c r="L133" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="M133" s="5"/>
+      <c r="N133" s="9"/>
+      <c r="O133" s="4"/>
+      <c r="P133" s="9"/>
+      <c r="Q133" s="9"/>
+      <c r="R133" s="9"/>
+      <c r="S133" s="9"/>
+      <c r="T133" s="9"/>
+      <c r="U133" s="9"/>
+    </row>
+    <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C134" s="9"/>
+      <c r="D134" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="E134" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F134" s="9"/>
+      <c r="G134" s="9"/>
+      <c r="H134" s="9"/>
+      <c r="I134" s="9"/>
+      <c r="J134" s="9"/>
+      <c r="N134" s="9"/>
+      <c r="O134" s="4"/>
+      <c r="P134" s="9"/>
+      <c r="Q134" s="9"/>
+      <c r="R134" s="9"/>
+      <c r="S134" s="9"/>
+      <c r="T134" s="9"/>
+      <c r="U134" s="9"/>
+    </row>
+    <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C135" s="9"/>
+      <c r="D135" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E135" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F135" s="9"/>
+      <c r="G135" s="9"/>
+      <c r="H135" s="9"/>
+      <c r="I135" s="9"/>
+      <c r="J135" s="9"/>
+      <c r="N135" s="9"/>
+      <c r="O135" s="4"/>
+      <c r="P135" s="9"/>
+      <c r="Q135" s="9"/>
+      <c r="R135" s="9"/>
+      <c r="S135" s="9"/>
+      <c r="T135" s="9"/>
+      <c r="U135" s="9"/>
+    </row>
+    <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C136" s="9"/>
+      <c r="D136" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="E136" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F136" s="9"/>
+      <c r="G136" s="9"/>
+      <c r="H136" s="9"/>
+      <c r="I136" s="9"/>
+      <c r="J136" s="9"/>
+      <c r="N136" s="9"/>
+      <c r="O136" s="4"/>
+      <c r="P136" s="9"/>
+      <c r="Q136" s="9"/>
+      <c r="R136" s="9"/>
+      <c r="S136" s="9"/>
+      <c r="T136" s="9"/>
+      <c r="U136" s="9"/>
+    </row>
+    <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C137" s="9"/>
+      <c r="D137" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E137" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F137" s="9"/>
+      <c r="G137" s="9"/>
+      <c r="H137" s="9"/>
+      <c r="I137" s="9"/>
+      <c r="J137" s="9"/>
+      <c r="N137" s="9"/>
+      <c r="O137" s="4"/>
+      <c r="P137" s="9"/>
+      <c r="Q137" s="9"/>
+      <c r="R137" s="9"/>
+      <c r="S137" s="9"/>
+      <c r="T137" s="9"/>
+      <c r="U137" s="9"/>
+    </row>
+    <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C138" s="9"/>
+      <c r="D138" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E138" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F138" s="9"/>
+      <c r="G138" s="9"/>
+      <c r="H138" s="9"/>
+      <c r="I138" s="9"/>
+      <c r="J138" s="9"/>
+      <c r="N138" s="9"/>
+      <c r="O138" s="4"/>
+      <c r="P138" s="9"/>
+      <c r="Q138" s="9"/>
+      <c r="R138" s="9"/>
+      <c r="S138" s="9"/>
+      <c r="T138" s="9"/>
+      <c r="U138" s="9"/>
+    </row>
+    <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C139" s="9"/>
+      <c r="D139" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="E139" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F139" s="9"/>
+      <c r="G139" s="9"/>
+      <c r="H139" s="9"/>
+      <c r="I139" s="9"/>
+      <c r="J139" s="9"/>
+      <c r="N139" s="9"/>
+      <c r="O139" s="4"/>
+      <c r="P139" s="9"/>
+      <c r="Q139" s="9"/>
+      <c r="R139" s="9"/>
+      <c r="S139" s="9"/>
+      <c r="T139" s="9"/>
+      <c r="U139" s="9"/>
+    </row>
+    <row r="141" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A141" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B141" s="4"/>
+      <c r="C141" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D141" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="E141" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="F141" s="4"/>
+      <c r="G141" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H141" s="4"/>
+      <c r="I141" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="J141" s="4"/>
+      <c r="L141" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="M141" s="4"/>
+      <c r="N141" s="4"/>
+      <c r="P141" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q141" s="4"/>
+    </row>
+    <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B142" s="9"/>
+      <c r="C142" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E142" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="F142" s="5"/>
+      <c r="G142" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="H142" s="5"/>
+      <c r="I142" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="J142" s="5"/>
+      <c r="L142" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M142" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="N142" s="9"/>
+      <c r="P142" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q142" s="9" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C143" s="9"/>
+      <c r="D143" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E143" s="5"/>
+      <c r="F143" s="5"/>
+      <c r="G143" s="5"/>
+      <c r="H143" s="5"/>
+      <c r="I143" s="5"/>
+      <c r="J143" s="5"/>
+      <c r="L143" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M143" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="N143" s="9"/>
+      <c r="P143" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q143" s="9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B144" s="4"/>
+      <c r="C144" s="9"/>
+      <c r="D144" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="E144" s="5"/>
+      <c r="F144" s="5"/>
+      <c r="G144" s="5"/>
+      <c r="H144" s="5"/>
+      <c r="I144" s="5"/>
+      <c r="J144" s="5"/>
+      <c r="L144" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="M144" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="N144" s="9"/>
+      <c r="P144" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q144" s="9" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="31" t="s">
+        <v>216</v>
+      </c>
+      <c r="B145" s="31"/>
+      <c r="C145" s="9"/>
+      <c r="D145" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E145" s="5"/>
+      <c r="F145" s="5"/>
+      <c r="G145" s="5"/>
+      <c r="H145" s="5"/>
+      <c r="I145" s="5"/>
+      <c r="J145" s="5"/>
+      <c r="L145" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="M145" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="N145" s="9"/>
+      <c r="P145" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q145" s="9" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C146" s="9"/>
+      <c r="D146" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E146" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="F146" s="5"/>
+      <c r="G146" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="H146" s="5"/>
+      <c r="I146" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="J146" s="5"/>
+      <c r="L146" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M146" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="N146" s="9"/>
+    </row>
+    <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B147" s="4"/>
+      <c r="C147" s="9"/>
+      <c r="D147" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="E147" s="5"/>
+      <c r="F147" s="5"/>
+      <c r="G147" s="5"/>
+      <c r="H147" s="5"/>
+      <c r="I147" s="5"/>
+      <c r="J147" s="5"/>
+      <c r="L147" s="32"/>
+      <c r="M147" s="32"/>
+    </row>
+    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B148" s="5"/>
+      <c r="C148" s="9"/>
+      <c r="D148" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="E148" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F148" s="9"/>
+      <c r="G148" s="9"/>
+      <c r="H148" s="9"/>
+      <c r="I148" s="9"/>
+      <c r="J148" s="9"/>
+    </row>
+    <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C149" s="9"/>
+      <c r="D149" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="E149" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F149" s="9"/>
+      <c r="G149" s="9"/>
+      <c r="H149" s="9"/>
+      <c r="I149" s="9"/>
+      <c r="J149" s="9"/>
+    </row>
+    <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B150" s="4"/>
+      <c r="C150" s="9"/>
+      <c r="D150" s="4"/>
+      <c r="E150" s="9"/>
+      <c r="F150" s="9"/>
+      <c r="G150" s="9"/>
+      <c r="H150" s="9"/>
+      <c r="I150" s="9"/>
+      <c r="J150" s="9"/>
+    </row>
+    <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="B151" s="5"/>
+      <c r="C151" s="9"/>
+      <c r="D151" s="4"/>
+      <c r="E151" s="9"/>
+      <c r="F151" s="9"/>
+      <c r="G151" s="9"/>
+      <c r="H151" s="9"/>
+      <c r="I151" s="9"/>
+      <c r="J151" s="9"/>
+    </row>
+    <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C152" s="9"/>
+      <c r="D152" s="4"/>
+      <c r="E152" s="9"/>
+      <c r="F152" s="9"/>
+      <c r="G152" s="9"/>
+      <c r="H152" s="9"/>
+      <c r="I152" s="9"/>
+      <c r="J152" s="9"/>
+    </row>
+    <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C153" s="9"/>
+      <c r="D153" s="4"/>
+      <c r="E153" s="9"/>
+      <c r="F153" s="9"/>
+      <c r="G153" s="9"/>
+      <c r="H153" s="9"/>
+      <c r="I153" s="9"/>
+      <c r="J153" s="9"/>
+    </row>
+    <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C154" s="9"/>
+      <c r="D154" s="4"/>
+      <c r="E154" s="9"/>
+      <c r="F154" s="9"/>
+      <c r="G154" s="9"/>
+      <c r="H154" s="9"/>
+      <c r="I154" s="9"/>
+      <c r="J154" s="9"/>
+    </row>
+    <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C155" s="9"/>
+      <c r="D155" s="4"/>
+      <c r="E155" s="9"/>
+      <c r="F155" s="9"/>
+      <c r="G155" s="9"/>
+      <c r="H155" s="9"/>
+      <c r="I155" s="9"/>
+      <c r="J155" s="9"/>
+    </row>
+    <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C156" s="9"/>
+      <c r="D156" s="4"/>
+      <c r="E156" s="9"/>
+      <c r="F156" s="9"/>
+      <c r="G156" s="9"/>
+      <c r="H156" s="9"/>
+      <c r="I156" s="9"/>
+      <c r="J156" s="9"/>
+    </row>
+    <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C157" s="9"/>
+      <c r="D157" s="4"/>
+      <c r="E157" s="9"/>
+      <c r="F157" s="9"/>
+      <c r="G157" s="9"/>
+      <c r="H157" s="9"/>
+      <c r="I157" s="9"/>
+      <c r="J157" s="9"/>
+    </row>
+    <row r="158" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A158" s="2"/>
+      <c r="B158" s="2"/>
+      <c r="C158" s="2"/>
+      <c r="D158" s="2"/>
+      <c r="E158" s="2"/>
+      <c r="F158" s="2"/>
+      <c r="G158" s="2"/>
+      <c r="H158" s="2"/>
+      <c r="I158" s="2"/>
+      <c r="J158" s="2"/>
+      <c r="K158" s="2"/>
+      <c r="L158" s="2"/>
+      <c r="M158" s="2"/>
+      <c r="N158" s="2"/>
+      <c r="O158" s="2"/>
+      <c r="P158" s="2"/>
+      <c r="Q158" s="2"/>
+      <c r="R158" s="2"/>
+      <c r="S158" s="2"/>
+      <c r="T158" s="2"/>
+      <c r="U158" s="2"/>
+    </row>
+    <row r="159" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A159" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="B159" s="6"/>
+      <c r="C159" s="6"/>
+      <c r="D159" s="6"/>
+      <c r="E159" s="6"/>
+      <c r="F159" s="6"/>
+      <c r="G159" s="6"/>
+      <c r="H159" s="6"/>
+      <c r="I159" s="6"/>
+      <c r="J159" s="6"/>
+      <c r="K159" s="6"/>
+      <c r="L159" s="6"/>
+      <c r="M159" s="6"/>
+      <c r="N159" s="6"/>
+      <c r="O159" s="6"/>
+      <c r="P159" s="6"/>
+      <c r="Q159" s="6"/>
+      <c r="R159" s="6"/>
+      <c r="S159" s="6"/>
+      <c r="T159" s="6"/>
+      <c r="U159" s="6"/>
+    </row>
+    <row r="160" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A160" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B160" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="I120" s="4"/>
-      <c r="J120" s="4"/>
-      <c r="K120" s="4" t="s">
+      <c r="C160" s="4"/>
+      <c r="D160" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E160" s="4"/>
+      <c r="F160" s="4"/>
+      <c r="H160" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="L120" s="4"/>
-      <c r="M120" s="4"/>
-      <c r="N120" s="4" t="s">
+      <c r="I160" s="4"/>
+      <c r="J160" s="4"/>
+      <c r="K160" s="4"/>
+      <c r="L160" s="4"/>
+      <c r="M160" s="4"/>
+    </row>
+    <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B161" s="33"/>
+      <c r="C161" s="33"/>
+      <c r="D161" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="E161" s="5"/>
+      <c r="F161" s="5"/>
+      <c r="H161" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="O120" s="4"/>
-      <c r="P120" s="4"/>
-      <c r="Q120" s="4"/>
-      <c r="R120" s="4"/>
-      <c r="S120" s="4"/>
-      <c r="T120" s="4"/>
-      <c r="U120" s="4"/>
-      <c r="V120" s="4"/>
-      <c r="W120" s="4"/>
-      <c r="X120" s="4"/>
-      <c r="Y120" s="4"/>
-      <c r="Z120" s="4"/>
-      <c r="AA120" s="4"/>
-      <c r="AB120" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="AC120" s="4"/>
-    </row>
-    <row r="121" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A121" s="4"/>
-      <c r="B121" s="4"/>
-      <c r="C121" s="4"/>
-      <c r="D121" s="4"/>
-      <c r="E121" s="4"/>
-      <c r="F121" s="4"/>
-      <c r="G121" s="4"/>
-      <c r="H121" s="4"/>
-      <c r="I121" s="4"/>
-      <c r="J121" s="4"/>
-      <c r="K121" s="4"/>
-      <c r="L121" s="4"/>
-      <c r="M121" s="4"/>
-      <c r="N121" s="31" t="s">
-        <v>179</v>
-      </c>
-      <c r="O121" s="31"/>
-      <c r="P121" s="31" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q121" s="31"/>
-      <c r="R121" s="31" t="s">
-        <v>174</v>
-      </c>
-      <c r="S121" s="31"/>
-      <c r="T121" s="31" t="s">
-        <v>169</v>
-      </c>
-      <c r="U121" s="31"/>
-      <c r="V121" s="31" t="s">
-        <v>168</v>
-      </c>
-      <c r="W121" s="31"/>
-      <c r="X121" s="31" t="s">
-        <v>167</v>
-      </c>
-      <c r="Y121" s="31"/>
-      <c r="Z121" s="31" t="s">
-        <v>165</v>
-      </c>
-      <c r="AA121" s="31"/>
-      <c r="AB121" s="31" t="s">
-        <v>160</v>
-      </c>
-      <c r="AC121" s="31"/>
-    </row>
-    <row r="122" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A122" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B122" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="C122" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="D122" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="E122" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="F122" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="G122" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="H122" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I122" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="J122" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="K122" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L122" s="5"/>
-      <c r="M122" s="5"/>
-      <c r="N122" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="O122" s="5"/>
-      <c r="P122" s="5"/>
-      <c r="Q122" s="5"/>
-      <c r="R122" s="5"/>
-      <c r="S122" s="5"/>
-      <c r="T122" s="5"/>
-      <c r="U122" s="5"/>
-      <c r="V122" s="5"/>
-      <c r="W122" s="5"/>
-      <c r="X122" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="Y122" s="5"/>
-      <c r="Z122" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="AA122" s="5"/>
-      <c r="AB122" s="5"/>
-      <c r="AC122" s="5"/>
-    </row>
-    <row r="123" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A123" s="2"/>
-      <c r="B123" s="2"/>
-      <c r="C123" s="2"/>
-      <c r="D123" s="2"/>
-      <c r="E123" s="2"/>
-      <c r="F123" s="2"/>
-      <c r="G123" s="2"/>
-      <c r="H123" s="2"/>
-      <c r="I123" s="2"/>
-      <c r="J123" s="2"/>
-      <c r="K123" s="2"/>
-      <c r="L123" s="2"/>
-      <c r="M123" s="2"/>
-      <c r="N123" s="2"/>
-      <c r="O123" s="2"/>
-      <c r="P123" s="2"/>
-      <c r="Q123" s="2"/>
-      <c r="R123" s="2"/>
-      <c r="S123" s="2"/>
-      <c r="T123" s="2"/>
-      <c r="U123" s="2"/>
+      <c r="I161" s="23"/>
+      <c r="J161" s="34" t="s">
+        <v>49</v>
+      </c>
+      <c r="K161" s="35"/>
+      <c r="L161" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="M161" s="37"/>
+    </row>
+    <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B162" s="38"/>
+      <c r="C162" s="38"/>
+      <c r="D162" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E162" s="5"/>
+      <c r="F162" s="5"/>
+      <c r="M162" s="26" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B163" s="29"/>
+      <c r="C163" s="29"/>
+      <c r="D163" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="E163" s="5"/>
+      <c r="F163" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="393">
+  <mergeCells count="558">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -6070,42 +6911,207 @@
     <mergeCell ref="H114:J114"/>
     <mergeCell ref="K114:M114"/>
     <mergeCell ref="N114:U114"/>
-    <mergeCell ref="A115:A117"/>
-    <mergeCell ref="B115:D117"/>
-    <mergeCell ref="E115:G117"/>
+    <mergeCell ref="A115:A120"/>
+    <mergeCell ref="B115:D120"/>
+    <mergeCell ref="E115:G120"/>
     <mergeCell ref="H115:J115"/>
     <mergeCell ref="K115:M115"/>
-    <mergeCell ref="N115:U117"/>
+    <mergeCell ref="N115:U120"/>
     <mergeCell ref="H116:J116"/>
     <mergeCell ref="K116:M116"/>
     <mergeCell ref="H117:J117"/>
     <mergeCell ref="K117:M117"/>
-    <mergeCell ref="A118:U118"/>
-    <mergeCell ref="A119:AC119"/>
-    <mergeCell ref="A120:A121"/>
-    <mergeCell ref="B120:D121"/>
-    <mergeCell ref="E120:G121"/>
-    <mergeCell ref="H120:J121"/>
-    <mergeCell ref="K120:M121"/>
-    <mergeCell ref="N120:O120"/>
-    <mergeCell ref="P120:AA120"/>
-    <mergeCell ref="AB120:AC120"/>
-    <mergeCell ref="N121:O121"/>
-    <mergeCell ref="P121:Q121"/>
-    <mergeCell ref="R121:S121"/>
-    <mergeCell ref="T121:U121"/>
-    <mergeCell ref="V121:W121"/>
-    <mergeCell ref="X121:Y121"/>
-    <mergeCell ref="Z121:AA121"/>
-    <mergeCell ref="AB121:AC121"/>
-    <mergeCell ref="B122:D122"/>
-    <mergeCell ref="E122:G122"/>
-    <mergeCell ref="H122:J122"/>
-    <mergeCell ref="K122:M122"/>
-    <mergeCell ref="N122:W122"/>
-    <mergeCell ref="X122:Y122"/>
-    <mergeCell ref="Z122:AC122"/>
-    <mergeCell ref="A123:U123"/>
+    <mergeCell ref="H118:J118"/>
+    <mergeCell ref="K118:M118"/>
+    <mergeCell ref="H119:J119"/>
+    <mergeCell ref="K119:M119"/>
+    <mergeCell ref="H120:J120"/>
+    <mergeCell ref="K120:M120"/>
+    <mergeCell ref="A121:U121"/>
+    <mergeCell ref="A122:AC122"/>
+    <mergeCell ref="A123:B123"/>
+    <mergeCell ref="E123:F123"/>
+    <mergeCell ref="G123:H123"/>
+    <mergeCell ref="I123:J123"/>
+    <mergeCell ref="L123:M123"/>
+    <mergeCell ref="P123:Q123"/>
+    <mergeCell ref="R123:S123"/>
+    <mergeCell ref="T123:U123"/>
+    <mergeCell ref="A124:B124"/>
+    <mergeCell ref="C124:C131"/>
+    <mergeCell ref="E124:F124"/>
+    <mergeCell ref="G124:H124"/>
+    <mergeCell ref="I124:J124"/>
+    <mergeCell ref="L124:M124"/>
+    <mergeCell ref="N124:N131"/>
+    <mergeCell ref="P124:Q125"/>
+    <mergeCell ref="R124:S125"/>
+    <mergeCell ref="T124:U125"/>
+    <mergeCell ref="E125:F125"/>
+    <mergeCell ref="G125:H125"/>
+    <mergeCell ref="I125:J125"/>
+    <mergeCell ref="A126:B126"/>
+    <mergeCell ref="E126:F126"/>
+    <mergeCell ref="G126:H126"/>
+    <mergeCell ref="I126:J126"/>
+    <mergeCell ref="L126:M126"/>
+    <mergeCell ref="P126:Q126"/>
+    <mergeCell ref="R126:S126"/>
+    <mergeCell ref="T126:U126"/>
+    <mergeCell ref="A127:B127"/>
+    <mergeCell ref="E127:F127"/>
+    <mergeCell ref="G127:H127"/>
+    <mergeCell ref="I127:J127"/>
+    <mergeCell ref="L127:M127"/>
+    <mergeCell ref="P127:Q127"/>
+    <mergeCell ref="R127:S127"/>
+    <mergeCell ref="T127:U127"/>
+    <mergeCell ref="E128:F128"/>
+    <mergeCell ref="G128:H128"/>
+    <mergeCell ref="I128:J128"/>
+    <mergeCell ref="P128:Q128"/>
+    <mergeCell ref="R128:S128"/>
+    <mergeCell ref="T128:U128"/>
+    <mergeCell ref="A129:B129"/>
+    <mergeCell ref="E129:F129"/>
+    <mergeCell ref="G129:H129"/>
+    <mergeCell ref="I129:J129"/>
+    <mergeCell ref="L129:M129"/>
+    <mergeCell ref="P129:Q129"/>
+    <mergeCell ref="R129:S129"/>
+    <mergeCell ref="T129:U129"/>
+    <mergeCell ref="A130:B130"/>
+    <mergeCell ref="E130:F130"/>
+    <mergeCell ref="G130:H130"/>
+    <mergeCell ref="I130:J130"/>
+    <mergeCell ref="L130:M130"/>
+    <mergeCell ref="P130:Q130"/>
+    <mergeCell ref="R130:S130"/>
+    <mergeCell ref="T130:U130"/>
+    <mergeCell ref="E131:F131"/>
+    <mergeCell ref="G131:H131"/>
+    <mergeCell ref="I131:J131"/>
+    <mergeCell ref="P131:Q131"/>
+    <mergeCell ref="R131:S131"/>
+    <mergeCell ref="T131:U131"/>
+    <mergeCell ref="A132:B132"/>
+    <mergeCell ref="C132:C139"/>
+    <mergeCell ref="E132:F132"/>
+    <mergeCell ref="G132:H132"/>
+    <mergeCell ref="I132:J132"/>
+    <mergeCell ref="L132:M132"/>
+    <mergeCell ref="N132:N139"/>
+    <mergeCell ref="P132:Q132"/>
+    <mergeCell ref="R132:S132"/>
+    <mergeCell ref="T132:U132"/>
+    <mergeCell ref="A133:B133"/>
+    <mergeCell ref="E133:F133"/>
+    <mergeCell ref="G133:H133"/>
+    <mergeCell ref="I133:J133"/>
+    <mergeCell ref="L133:M133"/>
+    <mergeCell ref="P133:Q133"/>
+    <mergeCell ref="R133:S133"/>
+    <mergeCell ref="T133:U133"/>
+    <mergeCell ref="E134:F134"/>
+    <mergeCell ref="G134:H134"/>
+    <mergeCell ref="I134:J134"/>
+    <mergeCell ref="P134:Q134"/>
+    <mergeCell ref="R134:S134"/>
+    <mergeCell ref="T134:U134"/>
+    <mergeCell ref="E135:F135"/>
+    <mergeCell ref="G135:H135"/>
+    <mergeCell ref="I135:J135"/>
+    <mergeCell ref="P135:Q135"/>
+    <mergeCell ref="R135:S135"/>
+    <mergeCell ref="T135:U135"/>
+    <mergeCell ref="E136:F136"/>
+    <mergeCell ref="G136:H136"/>
+    <mergeCell ref="I136:J136"/>
+    <mergeCell ref="P136:Q136"/>
+    <mergeCell ref="R136:S136"/>
+    <mergeCell ref="T136:U136"/>
+    <mergeCell ref="E137:F137"/>
+    <mergeCell ref="G137:H137"/>
+    <mergeCell ref="I137:J137"/>
+    <mergeCell ref="P137:Q137"/>
+    <mergeCell ref="R137:S137"/>
+    <mergeCell ref="T137:U137"/>
+    <mergeCell ref="E138:F138"/>
+    <mergeCell ref="G138:H138"/>
+    <mergeCell ref="I138:J138"/>
+    <mergeCell ref="P138:Q138"/>
+    <mergeCell ref="R138:S138"/>
+    <mergeCell ref="T138:U138"/>
+    <mergeCell ref="E139:F139"/>
+    <mergeCell ref="G139:H139"/>
+    <mergeCell ref="I139:J139"/>
+    <mergeCell ref="P139:Q139"/>
+    <mergeCell ref="R139:S139"/>
+    <mergeCell ref="T139:U139"/>
+    <mergeCell ref="A141:B141"/>
+    <mergeCell ref="E141:F141"/>
+    <mergeCell ref="G141:H141"/>
+    <mergeCell ref="I141:J141"/>
+    <mergeCell ref="L141:N141"/>
+    <mergeCell ref="P141:Q141"/>
+    <mergeCell ref="A142:B142"/>
+    <mergeCell ref="C142:C149"/>
+    <mergeCell ref="E142:F145"/>
+    <mergeCell ref="G142:H145"/>
+    <mergeCell ref="I142:J145"/>
+    <mergeCell ref="M142:N142"/>
+    <mergeCell ref="M143:N143"/>
+    <mergeCell ref="A144:B144"/>
+    <mergeCell ref="M144:N144"/>
+    <mergeCell ref="A145:B145"/>
+    <mergeCell ref="M145:N145"/>
+    <mergeCell ref="E146:F147"/>
+    <mergeCell ref="G146:H147"/>
+    <mergeCell ref="I146:J147"/>
+    <mergeCell ref="M146:N146"/>
+    <mergeCell ref="A147:B147"/>
+    <mergeCell ref="A148:B148"/>
+    <mergeCell ref="E148:F148"/>
+    <mergeCell ref="G148:H148"/>
+    <mergeCell ref="I148:J148"/>
+    <mergeCell ref="E149:F149"/>
+    <mergeCell ref="G149:H149"/>
+    <mergeCell ref="I149:J149"/>
+    <mergeCell ref="A150:B150"/>
+    <mergeCell ref="C150:C157"/>
+    <mergeCell ref="E150:F150"/>
+    <mergeCell ref="G150:H150"/>
+    <mergeCell ref="I150:J150"/>
+    <mergeCell ref="A151:B151"/>
+    <mergeCell ref="E151:F151"/>
+    <mergeCell ref="G151:H151"/>
+    <mergeCell ref="I151:J151"/>
+    <mergeCell ref="E152:F152"/>
+    <mergeCell ref="G152:H152"/>
+    <mergeCell ref="I152:J152"/>
+    <mergeCell ref="E153:F153"/>
+    <mergeCell ref="G153:H153"/>
+    <mergeCell ref="I153:J153"/>
+    <mergeCell ref="E154:F154"/>
+    <mergeCell ref="G154:H154"/>
+    <mergeCell ref="I154:J154"/>
+    <mergeCell ref="E155:F155"/>
+    <mergeCell ref="G155:H155"/>
+    <mergeCell ref="I155:J155"/>
+    <mergeCell ref="E156:F156"/>
+    <mergeCell ref="G156:H156"/>
+    <mergeCell ref="I156:J156"/>
+    <mergeCell ref="E157:F157"/>
+    <mergeCell ref="G157:H157"/>
+    <mergeCell ref="I157:J157"/>
+    <mergeCell ref="A158:U158"/>
+    <mergeCell ref="A159:U159"/>
+    <mergeCell ref="B160:C160"/>
+    <mergeCell ref="D160:F160"/>
+    <mergeCell ref="H160:M160"/>
+    <mergeCell ref="D161:F161"/>
+    <mergeCell ref="D162:F162"/>
+    <mergeCell ref="D163:F163"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -6130,876 +7136,876 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="32"/>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32"/>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="32"/>
-      <c r="R1" s="32"/>
-      <c r="S1" s="32"/>
-      <c r="T1" s="32"/>
-      <c r="U1" s="32"/>
-      <c r="V1" s="32"/>
-      <c r="W1" s="32"/>
+      <c r="A1" s="39"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39"/>
+      <c r="R1" s="39"/>
+      <c r="S1" s="39"/>
+      <c r="T1" s="39"/>
+      <c r="U1" s="39"/>
+      <c r="V1" s="39"/>
+      <c r="W1" s="39"/>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="32"/>
-      <c r="B2" s="33"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="34"/>
-      <c r="O2" s="34"/>
-      <c r="P2" s="34"/>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
-      <c r="T2" s="34"/>
-      <c r="U2" s="34"/>
-      <c r="V2" s="35"/>
-      <c r="W2" s="32"/>
+      <c r="A2" s="39"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
+      <c r="Q2" s="41"/>
+      <c r="R2" s="41"/>
+      <c r="S2" s="41"/>
+      <c r="T2" s="41"/>
+      <c r="U2" s="41"/>
+      <c r="V2" s="42"/>
+      <c r="W2" s="39"/>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="32"/>
-      <c r="B3" s="36"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="37" t="s">
+      <c r="A3" s="39"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="44" t="s">
+        <v>225</v>
+      </c>
+      <c r="E3" s="44"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="39"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="39"/>
+      <c r="T3" s="39"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="45"/>
+      <c r="W3" s="39"/>
+    </row>
+    <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="39"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
+      <c r="L4" s="39"/>
+      <c r="M4" s="39"/>
+      <c r="N4" s="39"/>
+      <c r="O4" s="39"/>
+      <c r="P4" s="39"/>
+      <c r="Q4" s="39"/>
+      <c r="R4" s="39"/>
+      <c r="S4" s="39"/>
+      <c r="T4" s="39"/>
+      <c r="U4" s="39"/>
+      <c r="V4" s="45"/>
+      <c r="W4" s="39"/>
+    </row>
+    <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="39"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="39"/>
+      <c r="I5" s="39"/>
+      <c r="J5" s="39"/>
+      <c r="K5" s="39"/>
+      <c r="L5" s="39"/>
+      <c r="M5" s="39"/>
+      <c r="N5" s="39"/>
+      <c r="O5" s="39"/>
+      <c r="P5" s="39"/>
+      <c r="Q5" s="39"/>
+      <c r="R5" s="39"/>
+      <c r="S5" s="39"/>
+      <c r="T5" s="39"/>
+      <c r="U5" s="39"/>
+      <c r="V5" s="45"/>
+      <c r="W5" s="39"/>
+    </row>
+    <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="39"/>
+      <c r="B6" s="43"/>
+      <c r="C6" s="48" t="s">
+        <v>226</v>
+      </c>
+      <c r="D6" s="49" t="s">
         <v>227</v>
       </c>
-      <c r="E3" s="37"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32"/>
-      <c r="M3" s="32"/>
-      <c r="N3" s="32"/>
-      <c r="O3" s="32"/>
-      <c r="P3" s="32"/>
-      <c r="Q3" s="32"/>
-      <c r="R3" s="32"/>
-      <c r="S3" s="32"/>
-      <c r="T3" s="32"/>
-      <c r="U3" s="32"/>
-      <c r="V3" s="38"/>
-      <c r="W3" s="32"/>
-    </row>
-    <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="32"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="32"/>
-      <c r="M4" s="32"/>
-      <c r="N4" s="32"/>
-      <c r="O4" s="32"/>
-      <c r="P4" s="32"/>
-      <c r="Q4" s="32"/>
-      <c r="R4" s="32"/>
-      <c r="S4" s="32"/>
-      <c r="T4" s="32"/>
-      <c r="U4" s="32"/>
-      <c r="V4" s="38"/>
-      <c r="W4" s="32"/>
-    </row>
-    <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="32"/>
-      <c r="B5" s="36"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
-      <c r="K5" s="32"/>
-      <c r="L5" s="32"/>
-      <c r="M5" s="32"/>
-      <c r="N5" s="32"/>
-      <c r="O5" s="32"/>
-      <c r="P5" s="32"/>
-      <c r="Q5" s="32"/>
-      <c r="R5" s="32"/>
-      <c r="S5" s="32"/>
-      <c r="T5" s="32"/>
-      <c r="U5" s="32"/>
-      <c r="V5" s="38"/>
-      <c r="W5" s="32"/>
-    </row>
-    <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="32"/>
-      <c r="B6" s="36"/>
-      <c r="C6" s="41" t="s">
+      <c r="E6" s="50" t="s">
+        <v>227</v>
+      </c>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="39"/>
+      <c r="J6" s="39"/>
+      <c r="K6" s="39"/>
+      <c r="L6" s="39"/>
+      <c r="M6" s="39"/>
+      <c r="N6" s="39"/>
+      <c r="O6" s="39"/>
+      <c r="P6" s="39"/>
+      <c r="Q6" s="39"/>
+      <c r="R6" s="39"/>
+      <c r="S6" s="39"/>
+      <c r="T6" s="39"/>
+      <c r="U6" s="39"/>
+      <c r="V6" s="45"/>
+      <c r="W6" s="39"/>
+    </row>
+    <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="39"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="51" t="s">
+        <v>227</v>
+      </c>
+      <c r="E7" s="52" t="s">
+        <v>227</v>
+      </c>
+      <c r="F7" s="39"/>
+      <c r="G7" s="39"/>
+      <c r="H7" s="39"/>
+      <c r="I7" s="39"/>
+      <c r="J7" s="39"/>
+      <c r="K7" s="39"/>
+      <c r="L7" s="39"/>
+      <c r="M7" s="39"/>
+      <c r="N7" s="39"/>
+      <c r="O7" s="39"/>
+      <c r="P7" s="39"/>
+      <c r="Q7" s="39"/>
+      <c r="R7" s="39"/>
+      <c r="S7" s="39"/>
+      <c r="T7" s="39"/>
+      <c r="U7" s="39"/>
+      <c r="V7" s="45"/>
+      <c r="W7" s="39"/>
+    </row>
+    <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="39"/>
+      <c r="B8" s="43"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="53" t="s">
+        <v>227</v>
+      </c>
+      <c r="E8" s="54" t="s">
+        <v>227</v>
+      </c>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="39"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="39"/>
+      <c r="M8" s="39"/>
+      <c r="N8" s="39"/>
+      <c r="O8" s="39"/>
+      <c r="P8" s="39"/>
+      <c r="Q8" s="55" t="s">
         <v>228</v>
       </c>
-      <c r="D6" s="42" t="s">
+      <c r="R8" s="55"/>
+      <c r="S8" s="55"/>
+      <c r="T8" s="55"/>
+      <c r="U8" s="39"/>
+      <c r="V8" s="45"/>
+      <c r="W8" s="39"/>
+    </row>
+    <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="39"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="56" t="s">
+        <v>227</v>
+      </c>
+      <c r="E9" s="57" t="s">
+        <v>227</v>
+      </c>
+      <c r="F9" s="39"/>
+      <c r="G9" s="39"/>
+      <c r="H9" s="39"/>
+      <c r="I9" s="39"/>
+      <c r="J9" s="39"/>
+      <c r="K9" s="39"/>
+      <c r="L9" s="39"/>
+      <c r="M9" s="39"/>
+      <c r="N9" s="39"/>
+      <c r="O9" s="39"/>
+      <c r="P9" s="39"/>
+      <c r="Q9" s="39"/>
+      <c r="R9" s="39"/>
+      <c r="S9" s="39"/>
+      <c r="T9" s="39"/>
+      <c r="U9" s="39"/>
+      <c r="V9" s="45"/>
+      <c r="W9" s="39"/>
+    </row>
+    <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="39"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
+      <c r="G10" s="39"/>
+      <c r="H10" s="39"/>
+      <c r="I10" s="39"/>
+      <c r="J10" s="39"/>
+      <c r="K10" s="39"/>
+      <c r="L10" s="39"/>
+      <c r="M10" s="39"/>
+      <c r="N10" s="39"/>
+      <c r="O10" s="39"/>
+      <c r="P10" s="39"/>
+      <c r="Q10" s="39"/>
+      <c r="R10" s="39"/>
+      <c r="S10" s="39"/>
+      <c r="T10" s="39"/>
+      <c r="U10" s="39"/>
+      <c r="V10" s="45"/>
+      <c r="W10" s="39"/>
+    </row>
+    <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="39"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="48" t="s">
         <v>229</v>
       </c>
-      <c r="E6" s="43" t="s">
-        <v>229</v>
-      </c>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
-      <c r="J6" s="32"/>
-      <c r="K6" s="32"/>
-      <c r="L6" s="32"/>
-      <c r="M6" s="32"/>
-      <c r="N6" s="32"/>
-      <c r="O6" s="32"/>
-      <c r="P6" s="32"/>
-      <c r="Q6" s="32"/>
-      <c r="R6" s="32"/>
-      <c r="S6" s="32"/>
-      <c r="T6" s="32"/>
-      <c r="U6" s="32"/>
-      <c r="V6" s="38"/>
-      <c r="W6" s="32"/>
-    </row>
-    <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="32"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="44" t="s">
-        <v>229</v>
-      </c>
-      <c r="E7" s="45" t="s">
-        <v>229</v>
-      </c>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
-      <c r="J7" s="32"/>
-      <c r="K7" s="32"/>
-      <c r="L7" s="32"/>
-      <c r="M7" s="32"/>
-      <c r="N7" s="32"/>
-      <c r="O7" s="32"/>
-      <c r="P7" s="32"/>
-      <c r="Q7" s="32"/>
-      <c r="R7" s="32"/>
-      <c r="S7" s="32"/>
-      <c r="T7" s="32"/>
-      <c r="U7" s="32"/>
-      <c r="V7" s="38"/>
-      <c r="W7" s="32"/>
-    </row>
-    <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="32"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="46" t="s">
-        <v>229</v>
-      </c>
-      <c r="E8" s="47" t="s">
-        <v>229</v>
-      </c>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="32"/>
-      <c r="K8" s="32"/>
-      <c r="L8" s="32"/>
-      <c r="M8" s="32"/>
-      <c r="N8" s="32"/>
-      <c r="O8" s="32"/>
-      <c r="P8" s="32"/>
-      <c r="Q8" s="48" t="s">
+      <c r="D11" s="56" t="s">
+        <v>227</v>
+      </c>
+      <c r="E11" s="57" t="s">
+        <v>227</v>
+      </c>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="39"/>
+      <c r="I11" s="39"/>
+      <c r="J11" s="39"/>
+      <c r="K11" s="39"/>
+      <c r="L11" s="39"/>
+      <c r="M11" s="39"/>
+      <c r="N11" s="39"/>
+      <c r="O11" s="39"/>
+      <c r="P11" s="39"/>
+      <c r="Q11" s="39"/>
+      <c r="R11" s="39"/>
+      <c r="S11" s="39"/>
+      <c r="T11" s="39"/>
+      <c r="U11" s="39"/>
+      <c r="V11" s="45"/>
+      <c r="W11" s="39"/>
+    </row>
+    <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="39"/>
+      <c r="B12" s="58"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="53" t="s">
+        <v>227</v>
+      </c>
+      <c r="E12" s="54" t="s">
+        <v>227</v>
+      </c>
+      <c r="V12" s="59"/>
+      <c r="W12" s="39"/>
+    </row>
+    <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="39"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="51" t="s">
+        <v>227</v>
+      </c>
+      <c r="E13" s="52" t="s">
+        <v>227</v>
+      </c>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="39"/>
+      <c r="I13" s="39"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
+      <c r="L13" s="39"/>
+      <c r="M13" s="39"/>
+      <c r="N13" s="39"/>
+      <c r="O13" s="39"/>
+      <c r="P13" s="39"/>
+      <c r="Q13" s="39"/>
+      <c r="R13" s="39"/>
+      <c r="T13" s="33"/>
+      <c r="U13" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="V13" s="59"/>
+      <c r="W13" s="39"/>
+    </row>
+    <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="39"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="49" t="s">
+        <v>227</v>
+      </c>
+      <c r="E14" s="50" t="s">
+        <v>227</v>
+      </c>
+      <c r="F14" s="61"/>
+      <c r="G14" s="61"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="61"/>
+      <c r="L14" s="61"/>
+      <c r="M14" s="61"/>
+      <c r="N14" s="61"/>
+      <c r="O14" s="61"/>
+      <c r="P14" s="61"/>
+      <c r="Q14" s="61"/>
+      <c r="R14" s="61"/>
+      <c r="S14" s="61"/>
+      <c r="T14" s="38"/>
+      <c r="U14" s="60"/>
+      <c r="V14" s="59"/>
+      <c r="W14" s="39"/>
+    </row>
+    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="39"/>
+      <c r="B15" s="43"/>
+      <c r="K15" s="62" t="s">
         <v>230</v>
       </c>
-      <c r="R8" s="48"/>
-      <c r="S8" s="48"/>
-      <c r="T8" s="48"/>
-      <c r="U8" s="32"/>
-      <c r="V8" s="38"/>
-      <c r="W8" s="32"/>
-    </row>
-    <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="32"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="41"/>
-      <c r="D9" s="49" t="s">
-        <v>229</v>
-      </c>
-      <c r="E9" s="50" t="s">
-        <v>229</v>
-      </c>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="32"/>
-      <c r="I9" s="32"/>
-      <c r="J9" s="32"/>
-      <c r="K9" s="32"/>
-      <c r="L9" s="32"/>
-      <c r="M9" s="32"/>
-      <c r="N9" s="32"/>
-      <c r="O9" s="32"/>
-      <c r="P9" s="32"/>
-      <c r="Q9" s="32"/>
-      <c r="R9" s="32"/>
-      <c r="S9" s="32"/>
-      <c r="T9" s="32"/>
-      <c r="U9" s="32"/>
-      <c r="V9" s="38"/>
-      <c r="W9" s="32"/>
-    </row>
-    <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="32"/>
-      <c r="B10" s="36"/>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="32"/>
-      <c r="H10" s="32"/>
-      <c r="I10" s="32"/>
-      <c r="J10" s="32"/>
-      <c r="K10" s="32"/>
-      <c r="L10" s="32"/>
-      <c r="M10" s="32"/>
-      <c r="N10" s="32"/>
-      <c r="O10" s="32"/>
-      <c r="P10" s="32"/>
-      <c r="Q10" s="32"/>
-      <c r="R10" s="32"/>
-      <c r="S10" s="32"/>
-      <c r="T10" s="32"/>
-      <c r="U10" s="32"/>
-      <c r="V10" s="38"/>
-      <c r="W10" s="0"/>
-    </row>
-    <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="32"/>
-      <c r="B11" s="36"/>
-      <c r="C11" s="41" t="s">
+      <c r="T15" s="39"/>
+      <c r="U15" s="39"/>
+      <c r="V15" s="59"/>
+      <c r="W15" s="39"/>
+    </row>
+    <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="39"/>
+      <c r="B16" s="43"/>
+      <c r="H16" s="39"/>
+      <c r="I16" s="39"/>
+      <c r="J16" s="39"/>
+      <c r="K16" s="63" t="s">
+        <v>44</v>
+      </c>
+      <c r="L16" s="64"/>
+      <c r="M16" s="64"/>
+      <c r="N16" s="64"/>
+      <c r="O16" s="64"/>
+      <c r="P16" s="65"/>
+      <c r="U16" s="39"/>
+      <c r="V16" s="59"/>
+      <c r="W16" s="39"/>
+    </row>
+    <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="43"/>
+      <c r="H17" s="39"/>
+      <c r="I17" s="39"/>
+      <c r="J17" s="39"/>
+      <c r="K17" s="66" t="s">
         <v>231</v>
       </c>
-      <c r="D11" s="49" t="s">
-        <v>229</v>
-      </c>
-      <c r="E11" s="50" t="s">
-        <v>229</v>
-      </c>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="32"/>
-      <c r="J11" s="32"/>
-      <c r="K11" s="32"/>
-      <c r="L11" s="32"/>
-      <c r="M11" s="32"/>
-      <c r="N11" s="32"/>
-      <c r="O11" s="32"/>
-      <c r="P11" s="32"/>
-      <c r="Q11" s="32"/>
-      <c r="R11" s="32"/>
-      <c r="S11" s="32"/>
-      <c r="T11" s="32"/>
-      <c r="U11" s="32"/>
-      <c r="V11" s="38"/>
-      <c r="W11" s="0"/>
-    </row>
-    <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="32"/>
-      <c r="B12" s="51"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="46" t="s">
-        <v>229</v>
-      </c>
-      <c r="E12" s="47" t="s">
-        <v>229</v>
-      </c>
-      <c r="V12" s="52"/>
-      <c r="W12" s="0"/>
-    </row>
-    <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="32"/>
-      <c r="B13" s="36"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="44" t="s">
-        <v>229</v>
-      </c>
-      <c r="E13" s="45" t="s">
-        <v>229</v>
-      </c>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="32"/>
-      <c r="J13" s="32"/>
-      <c r="K13" s="32"/>
-      <c r="L13" s="32"/>
-      <c r="M13" s="32"/>
-      <c r="N13" s="32"/>
-      <c r="O13" s="32"/>
-      <c r="P13" s="32"/>
-      <c r="Q13" s="32"/>
-      <c r="R13" s="32"/>
-      <c r="T13" s="53"/>
-      <c r="U13" s="54" t="s">
-        <v>47</v>
-      </c>
-      <c r="V13" s="52"/>
-      <c r="W13" s="0"/>
-    </row>
-    <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="32"/>
-      <c r="B14" s="36"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="42" t="s">
-        <v>229</v>
-      </c>
-      <c r="E14" s="43" t="s">
-        <v>229</v>
-      </c>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
-      <c r="J14" s="55"/>
-      <c r="K14" s="55"/>
-      <c r="L14" s="55"/>
-      <c r="M14" s="55"/>
-      <c r="N14" s="55"/>
-      <c r="O14" s="55"/>
-      <c r="P14" s="55"/>
-      <c r="Q14" s="55"/>
-      <c r="R14" s="55"/>
-      <c r="S14" s="55"/>
-      <c r="T14" s="56"/>
-      <c r="U14" s="54"/>
-      <c r="V14" s="52"/>
-      <c r="W14" s="0"/>
-    </row>
-    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="32"/>
-      <c r="B15" s="36"/>
-      <c r="K15" s="57" t="s">
+      <c r="L17" s="67"/>
+      <c r="M17" s="67"/>
+      <c r="N17" s="67"/>
+      <c r="O17" s="67"/>
+      <c r="P17" s="68"/>
+      <c r="R17" s="39"/>
+      <c r="T17" s="33"/>
+      <c r="U17" s="60" t="s">
+        <v>44</v>
+      </c>
+      <c r="V17" s="59"/>
+      <c r="W17" s="39"/>
+    </row>
+    <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="43"/>
+      <c r="H18" s="39"/>
+      <c r="I18" s="39"/>
+      <c r="J18" s="39"/>
+      <c r="K18" s="69"/>
+      <c r="L18" s="70"/>
+      <c r="M18" s="70"/>
+      <c r="N18" s="70"/>
+      <c r="O18" s="70"/>
+      <c r="P18" s="71" t="s">
+        <v>49</v>
+      </c>
+      <c r="R18" s="39"/>
+      <c r="T18" s="72"/>
+      <c r="U18" s="60"/>
+      <c r="V18" s="59"/>
+      <c r="W18" s="39"/>
+    </row>
+    <row r="19" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="43"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="39"/>
+      <c r="H19" s="39"/>
+      <c r="K19" s="73" t="s">
         <v>232</v>
       </c>
-      <c r="T15" s="32"/>
-      <c r="U15" s="32"/>
-      <c r="V15" s="52"/>
-      <c r="W15" s="0"/>
-    </row>
-    <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="32"/>
-      <c r="B16" s="36"/>
-      <c r="H16" s="32"/>
-      <c r="I16" s="32"/>
-      <c r="J16" s="32"/>
-      <c r="K16" s="58" t="s">
-        <v>44</v>
-      </c>
-      <c r="L16" s="59"/>
-      <c r="M16" s="59"/>
-      <c r="N16" s="59"/>
-      <c r="O16" s="59"/>
-      <c r="P16" s="60"/>
-      <c r="U16" s="32"/>
-      <c r="V16" s="52"/>
-      <c r="W16" s="0"/>
-    </row>
-    <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="36"/>
-      <c r="H17" s="32"/>
-      <c r="I17" s="32"/>
-      <c r="J17" s="32"/>
-      <c r="K17" s="61" t="s">
+      <c r="L19" s="73"/>
+      <c r="M19" s="73"/>
+      <c r="U19" s="39"/>
+      <c r="V19" s="59"/>
+      <c r="W19" s="39"/>
+    </row>
+    <row r="20" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="43"/>
+      <c r="F20" s="73" t="s">
         <v>233</v>
       </c>
-      <c r="L17" s="62"/>
-      <c r="M17" s="62"/>
-      <c r="N17" s="62"/>
-      <c r="O17" s="62"/>
-      <c r="P17" s="63"/>
-      <c r="R17" s="32"/>
-      <c r="T17" s="53"/>
-      <c r="U17" s="54" t="s">
-        <v>44</v>
-      </c>
-      <c r="V17" s="52"/>
-      <c r="W17" s="0"/>
-    </row>
-    <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="36"/>
-      <c r="H18" s="32"/>
-      <c r="I18" s="32"/>
-      <c r="J18" s="32"/>
-      <c r="K18" s="64"/>
-      <c r="L18" s="65"/>
-      <c r="M18" s="65"/>
-      <c r="N18" s="65"/>
-      <c r="O18" s="65"/>
-      <c r="P18" s="66" t="s">
+      <c r="G20" s="73"/>
+      <c r="H20" s="73"/>
+      <c r="K20" s="74" t="s">
         <v>49</v>
       </c>
-      <c r="R18" s="32"/>
-      <c r="T18" s="67"/>
-      <c r="U18" s="54"/>
-      <c r="V18" s="52"/>
-      <c r="W18" s="0"/>
-    </row>
-    <row r="19" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="36"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="32"/>
-      <c r="K19" s="68" t="s">
+      <c r="L20" s="75"/>
+      <c r="M20" s="76"/>
+      <c r="U20" s="39"/>
+      <c r="V20" s="59"/>
+      <c r="W20" s="39"/>
+    </row>
+    <row r="21" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="43"/>
+      <c r="F21" s="77"/>
+      <c r="G21" s="78"/>
+      <c r="H21" s="79" t="s">
         <v>234</v>
       </c>
-      <c r="L19" s="68"/>
-      <c r="M19" s="68"/>
-      <c r="U19" s="32"/>
-      <c r="V19" s="52"/>
-      <c r="W19" s="0"/>
-    </row>
-    <row r="20" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="36"/>
-      <c r="F20" s="68" t="s">
+      <c r="K21" s="80"/>
+      <c r="L21" s="81"/>
+      <c r="M21" s="82" t="s">
         <v>235</v>
       </c>
-      <c r="G20" s="68"/>
-      <c r="H20" s="68"/>
-      <c r="K20" s="69" t="s">
+      <c r="U21" s="39"/>
+      <c r="V21" s="59"/>
+      <c r="W21" s="39"/>
+      <c r="X21" s="39"/>
+    </row>
+    <row r="22" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="43"/>
+      <c r="F22" s="83"/>
+      <c r="G22" s="84"/>
+      <c r="H22" s="85"/>
+      <c r="K22" s="73" t="s">
+        <v>236</v>
+      </c>
+      <c r="L22" s="73"/>
+      <c r="M22" s="73"/>
+      <c r="Q22" s="55" t="s">
+        <v>237</v>
+      </c>
+      <c r="R22" s="55"/>
+      <c r="S22" s="55"/>
+      <c r="U22" s="39"/>
+      <c r="V22" s="59"/>
+      <c r="W22" s="39"/>
+      <c r="X22" s="39"/>
+    </row>
+    <row r="23" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="43"/>
+      <c r="C23" s="48" t="s">
+        <v>238</v>
+      </c>
+      <c r="D23" s="86"/>
+      <c r="F23" s="83" t="s">
+        <v>239</v>
+      </c>
+      <c r="G23" s="84"/>
+      <c r="H23" s="85" t="s">
+        <v>240</v>
+      </c>
+      <c r="K23" s="74" t="s">
         <v>49</v>
       </c>
-      <c r="L20" s="70"/>
-      <c r="M20" s="71"/>
-      <c r="U20" s="32"/>
-      <c r="V20" s="52"/>
-      <c r="W20" s="0"/>
-    </row>
-    <row r="21" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="36"/>
-      <c r="F21" s="72"/>
-      <c r="G21" s="73"/>
-      <c r="H21" s="74" t="s">
-        <v>236</v>
-      </c>
-      <c r="K21" s="75"/>
-      <c r="L21" s="76"/>
-      <c r="M21" s="77" t="s">
-        <v>237</v>
-      </c>
-      <c r="U21" s="32"/>
-      <c r="V21" s="52"/>
-      <c r="W21" s="0"/>
-      <c r="X21" s="32"/>
-    </row>
-    <row r="22" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="36"/>
-      <c r="F22" s="78"/>
-      <c r="G22" s="79"/>
-      <c r="H22" s="80"/>
-      <c r="K22" s="68" t="s">
-        <v>238</v>
-      </c>
-      <c r="L22" s="68"/>
-      <c r="M22" s="68"/>
-      <c r="Q22" s="48" t="s">
-        <v>239</v>
-      </c>
-      <c r="R22" s="48"/>
-      <c r="S22" s="48"/>
-      <c r="U22" s="32"/>
-      <c r="V22" s="52"/>
-      <c r="W22" s="0"/>
-      <c r="X22" s="32"/>
-    </row>
-    <row r="23" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="36"/>
-      <c r="C23" s="41" t="s">
-        <v>240</v>
-      </c>
-      <c r="D23" s="81"/>
-      <c r="F23" s="78" t="s">
+      <c r="L23" s="75"/>
+      <c r="M23" s="76"/>
+      <c r="U23" s="39"/>
+      <c r="V23" s="59"/>
+      <c r="W23" s="39"/>
+      <c r="X23" s="39"/>
+    </row>
+    <row r="24" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="43"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="87"/>
+      <c r="F24" s="83" t="s">
         <v>241</v>
       </c>
-      <c r="G23" s="79"/>
-      <c r="H23" s="80" t="s">
+      <c r="G24" s="84"/>
+      <c r="H24" s="85" t="s">
         <v>242</v>
       </c>
-      <c r="K23" s="69" t="s">
+      <c r="K24" s="80"/>
+      <c r="L24" s="81"/>
+      <c r="M24" s="82" t="s">
+        <v>235</v>
+      </c>
+      <c r="U24" s="39"/>
+      <c r="V24" s="59"/>
+      <c r="W24" s="39"/>
+      <c r="X24" s="39"/>
+    </row>
+    <row r="25" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="43"/>
+      <c r="F25" s="83" t="s">
         <v>49</v>
       </c>
-      <c r="L23" s="70"/>
-      <c r="M23" s="71"/>
-      <c r="U23" s="32"/>
-      <c r="V23" s="52"/>
-      <c r="W23" s="0"/>
-      <c r="X23" s="32"/>
-    </row>
-    <row r="24" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="36"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="82"/>
-      <c r="F24" s="78" t="s">
+      <c r="G25" s="84"/>
+      <c r="H25" s="85" t="s">
+        <v>49</v>
+      </c>
+      <c r="K25" s="73" t="s">
+        <v>232</v>
+      </c>
+      <c r="L25" s="73"/>
+      <c r="M25" s="73"/>
+      <c r="R25" s="88"/>
+      <c r="S25" s="89"/>
+      <c r="T25" s="47"/>
+      <c r="U25" s="90" t="s">
         <v>243</v>
       </c>
-      <c r="G24" s="79"/>
-      <c r="H24" s="80" t="s">
+      <c r="V25" s="59"/>
+      <c r="W25" s="39"/>
+      <c r="X25" s="39"/>
+    </row>
+    <row r="26" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="43"/>
+      <c r="F26" s="91" t="s">
         <v>244</v>
       </c>
-      <c r="K24" s="75"/>
-      <c r="L24" s="76"/>
-      <c r="M24" s="77" t="s">
-        <v>237</v>
-      </c>
-      <c r="U24" s="32"/>
-      <c r="V24" s="52"/>
-      <c r="W24" s="0"/>
-      <c r="X24" s="32"/>
-    </row>
-    <row r="25" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="36"/>
-      <c r="F25" s="78" t="s">
+      <c r="G26" s="92"/>
+      <c r="H26" s="93"/>
+      <c r="K26" s="74"/>
+      <c r="L26" s="76" t="s">
+        <v>235</v>
+      </c>
+      <c r="R26" s="88"/>
+      <c r="S26" s="89"/>
+      <c r="T26" s="47"/>
+      <c r="U26" s="90" t="s">
+        <v>245</v>
+      </c>
+      <c r="V26" s="59"/>
+      <c r="W26" s="39"/>
+      <c r="X26" s="39"/>
+    </row>
+    <row r="27" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="43"/>
+      <c r="K27" s="94"/>
+      <c r="L27" s="95"/>
+      <c r="R27" s="88"/>
+      <c r="S27" s="89"/>
+      <c r="T27" s="47"/>
+      <c r="U27" s="90" t="s">
+        <v>246</v>
+      </c>
+      <c r="V27" s="59"/>
+      <c r="W27" s="39"/>
+      <c r="X27" s="39"/>
+    </row>
+    <row r="28" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="43"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="47"/>
+      <c r="K28" s="80" t="s">
         <v>49</v>
       </c>
-      <c r="G25" s="79"/>
-      <c r="H25" s="80" t="s">
-        <v>49</v>
-      </c>
-      <c r="K25" s="68" t="s">
-        <v>234</v>
-      </c>
-      <c r="L25" s="68"/>
-      <c r="M25" s="68"/>
-      <c r="R25" s="83"/>
-      <c r="S25" s="84"/>
-      <c r="T25" s="40"/>
-      <c r="U25" s="85" t="s">
-        <v>245</v>
-      </c>
-      <c r="V25" s="52"/>
-      <c r="W25" s="0"/>
-      <c r="X25" s="32"/>
-    </row>
-    <row r="26" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="36"/>
-      <c r="F26" s="86" t="s">
-        <v>246</v>
-      </c>
-      <c r="G26" s="87"/>
-      <c r="H26" s="88"/>
-      <c r="K26" s="69"/>
-      <c r="L26" s="71" t="s">
-        <v>237</v>
-      </c>
-      <c r="R26" s="83"/>
-      <c r="S26" s="84"/>
-      <c r="T26" s="40"/>
-      <c r="U26" s="85" t="s">
+      <c r="L28" s="82"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="47"/>
+      <c r="R28" s="88"/>
+      <c r="S28" s="89"/>
+      <c r="T28" s="47"/>
+      <c r="U28" s="90" t="s">
         <v>247</v>
       </c>
-      <c r="V26" s="52"/>
-      <c r="W26" s="0"/>
-      <c r="X26" s="32"/>
-    </row>
-    <row r="27" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="36"/>
-      <c r="K27" s="89"/>
-      <c r="L27" s="90"/>
-      <c r="R27" s="83"/>
-      <c r="S27" s="84"/>
-      <c r="T27" s="40"/>
-      <c r="U27" s="85" t="s">
+      <c r="V28" s="59"/>
+      <c r="W28" s="39"/>
+      <c r="X28" s="39"/>
+      <c r="AF28" s="39"/>
+      <c r="AG28" s="39"/>
+      <c r="AH28" s="39"/>
+    </row>
+    <row r="29" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="58"/>
+      <c r="D29" s="44" t="s">
         <v>248</v>
       </c>
-      <c r="V27" s="52"/>
-      <c r="W27" s="0"/>
-      <c r="X27" s="32"/>
-    </row>
-    <row r="28" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="36"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="40"/>
-      <c r="K28" s="75" t="s">
-        <v>49</v>
-      </c>
-      <c r="L28" s="77"/>
-      <c r="O28" s="39"/>
-      <c r="P28" s="40"/>
-      <c r="R28" s="83"/>
-      <c r="S28" s="84"/>
-      <c r="T28" s="40"/>
-      <c r="U28" s="85" t="s">
+      <c r="E29" s="44"/>
+      <c r="O29" s="44" t="s">
         <v>249</v>
       </c>
-      <c r="V28" s="52"/>
-      <c r="W28" s="0"/>
-      <c r="X28" s="32"/>
-      <c r="AF28" s="32"/>
-      <c r="AG28" s="32"/>
-      <c r="AH28" s="32"/>
-    </row>
-    <row r="29" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="51"/>
-      <c r="D29" s="37" t="s">
-        <v>250</v>
-      </c>
-      <c r="E29" s="37"/>
-      <c r="O29" s="37" t="s">
-        <v>251</v>
-      </c>
-      <c r="P29" s="37"/>
-      <c r="U29" s="32"/>
-      <c r="V29" s="52"/>
-      <c r="W29" s="0"/>
-      <c r="X29" s="32"/>
+      <c r="P29" s="44"/>
+      <c r="U29" s="39"/>
+      <c r="V29" s="59"/>
+      <c r="W29" s="39"/>
+      <c r="X29" s="39"/>
     </row>
     <row r="30" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="91"/>
-      <c r="C30" s="92"/>
-      <c r="D30" s="92"/>
-      <c r="E30" s="92"/>
-      <c r="F30" s="92"/>
-      <c r="G30" s="92"/>
-      <c r="H30" s="92"/>
-      <c r="I30" s="92"/>
-      <c r="J30" s="92"/>
-      <c r="K30" s="92"/>
-      <c r="L30" s="92"/>
-      <c r="M30" s="92"/>
-      <c r="N30" s="92"/>
-      <c r="O30" s="92"/>
-      <c r="P30" s="92"/>
-      <c r="Q30" s="92"/>
-      <c r="R30" s="92"/>
-      <c r="S30" s="92"/>
-      <c r="T30" s="92"/>
-      <c r="U30" s="92"/>
-      <c r="V30" s="93"/>
-      <c r="W30" s="0"/>
-      <c r="X30" s="32"/>
+      <c r="B30" s="96"/>
+      <c r="C30" s="97"/>
+      <c r="D30" s="97"/>
+      <c r="E30" s="97"/>
+      <c r="F30" s="97"/>
+      <c r="G30" s="97"/>
+      <c r="H30" s="97"/>
+      <c r="I30" s="97"/>
+      <c r="J30" s="97"/>
+      <c r="K30" s="97"/>
+      <c r="L30" s="97"/>
+      <c r="M30" s="97"/>
+      <c r="N30" s="97"/>
+      <c r="O30" s="97"/>
+      <c r="P30" s="97"/>
+      <c r="Q30" s="97"/>
+      <c r="R30" s="97"/>
+      <c r="S30" s="97"/>
+      <c r="T30" s="97"/>
+      <c r="U30" s="97"/>
+      <c r="V30" s="98"/>
+      <c r="W30" s="39"/>
+      <c r="X30" s="39"/>
     </row>
     <row r="31" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="0"/>
-      <c r="D31" s="0"/>
-      <c r="E31" s="0"/>
-      <c r="F31" s="0"/>
-      <c r="G31" s="0"/>
-      <c r="H31" s="0"/>
-      <c r="I31" s="0"/>
-      <c r="J31" s="0"/>
-      <c r="K31" s="0"/>
-      <c r="L31" s="0"/>
-      <c r="M31" s="0"/>
-      <c r="N31" s="0"/>
-      <c r="O31" s="0"/>
-      <c r="P31" s="0"/>
-      <c r="Q31" s="0"/>
-      <c r="R31" s="0"/>
-      <c r="S31" s="0"/>
-      <c r="T31" s="0"/>
-      <c r="U31" s="0"/>
-      <c r="V31" s="0"/>
-      <c r="W31" s="0"/>
-      <c r="X31" s="32"/>
+      <c r="C31" s="39"/>
+      <c r="D31" s="39"/>
+      <c r="E31" s="39"/>
+      <c r="F31" s="39"/>
+      <c r="G31" s="39"/>
+      <c r="H31" s="39"/>
+      <c r="I31" s="39"/>
+      <c r="J31" s="39"/>
+      <c r="K31" s="39"/>
+      <c r="L31" s="39"/>
+      <c r="M31" s="39"/>
+      <c r="N31" s="39"/>
+      <c r="O31" s="39"/>
+      <c r="P31" s="39"/>
+      <c r="Q31" s="39"/>
+      <c r="R31" s="39"/>
+      <c r="S31" s="39"/>
+      <c r="T31" s="39"/>
+      <c r="U31" s="39"/>
+      <c r="V31" s="39"/>
+      <c r="W31" s="39"/>
+      <c r="X31" s="39"/>
     </row>
     <row r="32" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="0"/>
-      <c r="D32" s="0"/>
-      <c r="E32" s="0"/>
-      <c r="F32" s="0"/>
-      <c r="G32" s="0"/>
-      <c r="H32" s="0"/>
-      <c r="I32" s="0"/>
-      <c r="J32" s="0"/>
-      <c r="K32" s="0"/>
-      <c r="L32" s="0"/>
-      <c r="M32" s="0"/>
-      <c r="N32" s="0"/>
-      <c r="O32" s="0"/>
-      <c r="P32" s="0"/>
-      <c r="Q32" s="0"/>
-      <c r="R32" s="0"/>
-      <c r="S32" s="0"/>
-      <c r="T32" s="0"/>
-      <c r="U32" s="0"/>
-      <c r="V32" s="0"/>
-      <c r="W32" s="0"/>
-      <c r="X32" s="32"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="39"/>
+      <c r="E32" s="39"/>
+      <c r="F32" s="39"/>
+      <c r="G32" s="39"/>
+      <c r="H32" s="39"/>
+      <c r="I32" s="39"/>
+      <c r="J32" s="39"/>
+      <c r="K32" s="39"/>
+      <c r="L32" s="39"/>
+      <c r="M32" s="39"/>
+      <c r="N32" s="39"/>
+      <c r="O32" s="39"/>
+      <c r="P32" s="39"/>
+      <c r="Q32" s="39"/>
+      <c r="R32" s="39"/>
+      <c r="S32" s="39"/>
+      <c r="T32" s="39"/>
+      <c r="U32" s="39"/>
+      <c r="V32" s="39"/>
+      <c r="W32" s="39"/>
+      <c r="X32" s="39"/>
     </row>
     <row r="33" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="0"/>
-      <c r="D33" s="0"/>
-      <c r="E33" s="0"/>
-      <c r="F33" s="0"/>
-      <c r="G33" s="0"/>
-      <c r="H33" s="0"/>
-      <c r="I33" s="0"/>
-      <c r="J33" s="0"/>
-      <c r="K33" s="0"/>
-      <c r="L33" s="0"/>
-      <c r="M33" s="0"/>
-      <c r="N33" s="0"/>
-      <c r="O33" s="0"/>
-      <c r="P33" s="0"/>
-      <c r="Q33" s="0"/>
-      <c r="R33" s="0"/>
-      <c r="S33" s="0"/>
-      <c r="T33" s="0"/>
-      <c r="U33" s="0"/>
-      <c r="V33" s="0"/>
-      <c r="W33" s="0"/>
-      <c r="X33" s="32"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="39"/>
+      <c r="E33" s="39"/>
+      <c r="F33" s="39"/>
+      <c r="G33" s="39"/>
+      <c r="H33" s="39"/>
+      <c r="I33" s="39"/>
+      <c r="J33" s="39"/>
+      <c r="K33" s="39"/>
+      <c r="L33" s="39"/>
+      <c r="M33" s="39"/>
+      <c r="N33" s="39"/>
+      <c r="O33" s="39"/>
+      <c r="P33" s="39"/>
+      <c r="Q33" s="39"/>
+      <c r="R33" s="39"/>
+      <c r="S33" s="39"/>
+      <c r="T33" s="39"/>
+      <c r="U33" s="39"/>
+      <c r="V33" s="39"/>
+      <c r="W33" s="39"/>
+      <c r="X33" s="39"/>
     </row>
     <row r="34" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="0"/>
-      <c r="D34" s="0"/>
-      <c r="E34" s="0"/>
-      <c r="F34" s="0"/>
-      <c r="G34" s="0"/>
-      <c r="H34" s="0"/>
-      <c r="I34" s="0"/>
-      <c r="J34" s="0"/>
-      <c r="K34" s="0"/>
-      <c r="L34" s="0"/>
-      <c r="M34" s="0"/>
-      <c r="N34" s="0"/>
-      <c r="O34" s="0"/>
-      <c r="P34" s="0"/>
-      <c r="Q34" s="0"/>
-      <c r="R34" s="0"/>
-      <c r="S34" s="0"/>
-      <c r="T34" s="0"/>
-      <c r="U34" s="0"/>
-      <c r="V34" s="0"/>
-      <c r="W34" s="0"/>
-      <c r="X34" s="32"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="39"/>
+      <c r="E34" s="39"/>
+      <c r="F34" s="39"/>
+      <c r="G34" s="39"/>
+      <c r="H34" s="39"/>
+      <c r="I34" s="39"/>
+      <c r="J34" s="39"/>
+      <c r="K34" s="39"/>
+      <c r="L34" s="39"/>
+      <c r="M34" s="39"/>
+      <c r="N34" s="39"/>
+      <c r="O34" s="39"/>
+      <c r="P34" s="39"/>
+      <c r="Q34" s="39"/>
+      <c r="R34" s="39"/>
+      <c r="S34" s="39"/>
+      <c r="T34" s="39"/>
+      <c r="U34" s="39"/>
+      <c r="V34" s="39"/>
+      <c r="W34" s="39"/>
+      <c r="X34" s="39"/>
     </row>
     <row r="35" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C35" s="0"/>
-      <c r="D35" s="0"/>
-      <c r="E35" s="0"/>
-      <c r="F35" s="0"/>
-      <c r="G35" s="0"/>
-      <c r="H35" s="0"/>
-      <c r="I35" s="0"/>
-      <c r="J35" s="0"/>
-      <c r="K35" s="0"/>
-      <c r="L35" s="0"/>
-      <c r="M35" s="0"/>
-      <c r="N35" s="0"/>
-      <c r="O35" s="0"/>
-      <c r="P35" s="0"/>
-      <c r="Q35" s="0"/>
-      <c r="R35" s="0"/>
-      <c r="S35" s="0"/>
-      <c r="T35" s="0"/>
-      <c r="U35" s="0"/>
-      <c r="V35" s="0"/>
-      <c r="W35" s="0"/>
-      <c r="X35" s="32"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="39"/>
+      <c r="E35" s="39"/>
+      <c r="F35" s="39"/>
+      <c r="G35" s="39"/>
+      <c r="H35" s="39"/>
+      <c r="I35" s="39"/>
+      <c r="J35" s="39"/>
+      <c r="K35" s="39"/>
+      <c r="L35" s="39"/>
+      <c r="M35" s="39"/>
+      <c r="N35" s="39"/>
+      <c r="O35" s="39"/>
+      <c r="P35" s="39"/>
+      <c r="Q35" s="39"/>
+      <c r="R35" s="39"/>
+      <c r="S35" s="39"/>
+      <c r="T35" s="39"/>
+      <c r="U35" s="39"/>
+      <c r="V35" s="39"/>
+      <c r="W35" s="39"/>
+      <c r="X35" s="39"/>
     </row>
     <row r="36" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C36" s="0"/>
-      <c r="D36" s="0"/>
-      <c r="E36" s="0"/>
-      <c r="F36" s="0"/>
-      <c r="G36" s="0"/>
-      <c r="H36" s="0"/>
-      <c r="I36" s="0"/>
-      <c r="J36" s="0"/>
-      <c r="K36" s="0"/>
-      <c r="L36" s="0"/>
-      <c r="M36" s="0"/>
-      <c r="N36" s="0"/>
-      <c r="O36" s="0"/>
-      <c r="P36" s="0"/>
-      <c r="Q36" s="0"/>
-      <c r="R36" s="0"/>
-      <c r="S36" s="0"/>
-      <c r="T36" s="0"/>
-      <c r="U36" s="0"/>
-      <c r="V36" s="0"/>
-      <c r="W36" s="0"/>
-      <c r="X36" s="32"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="39"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="39"/>
+      <c r="G36" s="39"/>
+      <c r="H36" s="39"/>
+      <c r="I36" s="39"/>
+      <c r="J36" s="39"/>
+      <c r="K36" s="39"/>
+      <c r="L36" s="39"/>
+      <c r="M36" s="39"/>
+      <c r="N36" s="39"/>
+      <c r="O36" s="39"/>
+      <c r="P36" s="39"/>
+      <c r="Q36" s="39"/>
+      <c r="R36" s="39"/>
+      <c r="S36" s="39"/>
+      <c r="T36" s="39"/>
+      <c r="U36" s="39"/>
+      <c r="V36" s="39"/>
+      <c r="W36" s="39"/>
+      <c r="X36" s="39"/>
     </row>
     <row r="37" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C37" s="0"/>
-      <c r="D37" s="0"/>
-      <c r="E37" s="0"/>
-      <c r="F37" s="0"/>
-      <c r="G37" s="0"/>
-      <c r="H37" s="0"/>
-      <c r="I37" s="0"/>
-      <c r="J37" s="0"/>
-      <c r="K37" s="0"/>
-      <c r="L37" s="0"/>
-      <c r="M37" s="0"/>
-      <c r="N37" s="0"/>
-      <c r="O37" s="0"/>
-      <c r="P37" s="0"/>
-      <c r="Q37" s="0"/>
-      <c r="R37" s="0"/>
-      <c r="S37" s="0"/>
-      <c r="T37" s="0"/>
-      <c r="U37" s="0"/>
-      <c r="V37" s="0"/>
-      <c r="W37" s="0"/>
-      <c r="X37" s="32"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="39"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="39"/>
+      <c r="I37" s="39"/>
+      <c r="J37" s="39"/>
+      <c r="K37" s="39"/>
+      <c r="L37" s="39"/>
+      <c r="M37" s="39"/>
+      <c r="N37" s="39"/>
+      <c r="O37" s="39"/>
+      <c r="P37" s="39"/>
+      <c r="Q37" s="39"/>
+      <c r="R37" s="39"/>
+      <c r="S37" s="39"/>
+      <c r="T37" s="39"/>
+      <c r="U37" s="39"/>
+      <c r="V37" s="39"/>
+      <c r="W37" s="39"/>
+      <c r="X37" s="39"/>
     </row>
     <row r="38" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C38" s="0"/>
-      <c r="D38" s="0"/>
-      <c r="E38" s="0"/>
-      <c r="F38" s="0"/>
-      <c r="G38" s="0"/>
-      <c r="H38" s="0"/>
-      <c r="I38" s="0"/>
-      <c r="J38" s="0"/>
-      <c r="K38" s="0"/>
-      <c r="L38" s="0"/>
-      <c r="M38" s="0"/>
-      <c r="N38" s="0"/>
-      <c r="O38" s="0"/>
-      <c r="P38" s="0"/>
-      <c r="Q38" s="0"/>
-      <c r="R38" s="0"/>
-      <c r="S38" s="0"/>
-      <c r="T38" s="0"/>
-      <c r="U38" s="0"/>
-      <c r="V38" s="0"/>
-      <c r="W38" s="0"/>
-      <c r="X38" s="32"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="39"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
+      <c r="H38" s="39"/>
+      <c r="I38" s="39"/>
+      <c r="J38" s="39"/>
+      <c r="K38" s="39"/>
+      <c r="L38" s="39"/>
+      <c r="M38" s="39"/>
+      <c r="N38" s="39"/>
+      <c r="O38" s="39"/>
+      <c r="P38" s="39"/>
+      <c r="Q38" s="39"/>
+      <c r="R38" s="39"/>
+      <c r="S38" s="39"/>
+      <c r="T38" s="39"/>
+      <c r="U38" s="39"/>
+      <c r="V38" s="39"/>
+      <c r="W38" s="39"/>
+      <c r="X38" s="39"/>
     </row>
     <row r="39" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="X39" s="32"/>
+      <c r="X39" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>

<commit_message>
[ Version 0.0.32.4 ] - SPARE pins wires were soldered.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -162,592 +162,592 @@
     <t xml:space="preserve">Power 5V.</t>
   </si>
   <si>
-    <t xml:space="preserve">3V</t>
+    <t xml:space="preserve">GND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GND.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP32 sleep/enable pin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serial communication transmit pin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMMUNICATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serial communication receive pin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_DRAIN_VENT_PWM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PWM output for drainage vent servos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRAINAGE_VENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_DRAIN_VENT_SPM1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for drainage vent power mosfet V1 – servo power mosfet 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_DRAIN_VENT_SPM2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for drainage vent power mosfet V2 - servo power mosfet 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_DRAIN_VENT_ESO1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI (only) for drainage vent V1 open position end switch - end switch open 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_DRAIN_VENT_ESO2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI (only) for drainage vent V2 open position end switch - end switch open 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_DRAIN_VENT_ESC1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI (only) for drainage vent V1 close position end switch - end switch close 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_DRAIN_VENT_ESC2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI (only) for drainage vent V2 close position end switch - end switch close 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_ROULETTE_EN1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R1 motor driver enable pin – enable 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROULETTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_ROULETTE_DIR1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R1 motor driver direction bit 1 – direction 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_ROULETTE_DIR2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R1 motor driver direction bit 2 – direction 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_TOP1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI for roulette R1 open position hall sensors – top 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_TOP2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI for roulette R1 open position hall sensors – top 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_BOT1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI for roulette R1 close position hall sensors – bottom 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_BOT2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI for roulette R1 close position hall sensors – bottom 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPARE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spare pin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP-IDF TIMERS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SYS_DRAIN_VENT_PWM_TIME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LEDC_TIMER_0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drainage vent servo PWM timer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP-IDF CHANNELS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SYS_DRAIN_VENT_PWM_CHNL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LEDC_CHANNEL_0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drainage vent servo PWM channel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRAINAGE VENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STRUCTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FILE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATRIBUTE TYPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATRIBUTE NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_timer_config_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vsrp_dataset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc.h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_mode_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">speed_mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration structure for LEDC TIMER.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_timer_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timer_num</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_timer_bit_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">duty_resolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uint32_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">freq_hz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_clk_cfg_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">clk_cfg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_channel_config_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration structure for LEDC CHANNEL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_channel_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">channel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timer_sel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_intr_type_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">intr_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">int</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gpio_num</t>
+  </si>
+  <si>
+    <t xml:space="preserve">duty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hpoint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pwm_generator_config_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration structure for PWM GENERATOR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">out_pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drainage_vent_dataset_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TickType_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">action_start_tick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dataset structure which store drainage vent runtime properties.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v1_opn_ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v1_cls_ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v2_opn_ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v2_cls_ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v1_opn_duty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v1_cls_duty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v2_opn_duty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v2_cls_duty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uint16_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">err_word</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uint8_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">io_byte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ctrl_byte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIT STRUCTURES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BYTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">READ BIN MASK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">READ HEX MASK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROCESS CODE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0b0000 0011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STRUCTURE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VENT 1 ENABLED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0b0001 0000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATRIBUTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VENT 2 ENABLED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0b0010 0000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATA TYPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FSM STATES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FSM STATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0b0000 1111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x0F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">START 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOVING 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLOSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">START 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMP PROCESS CODE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0b0011 0000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOVING 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FINISH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DUPONT &amp; UTP CABLE CONNECTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CABLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLOR 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLOR 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DUPONT terminal – TOP view</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+10V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+6V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PWM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARROW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roulette_dataset_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dataset structure which store roulette runtime properties.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r1_opn_ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r1_cls_ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROULETTE 1 ENABLED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACKNOWLEDGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DUPONT connector – TOP view</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIGNAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VENT 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRAINAGE VENT DRIVER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VENT 2</t>
   </si>
   <si>
     <t xml:space="preserve">3.3V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Power 3.3V.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GND.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serial communication transmit pin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COMMUNICATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serial communication receive pin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_DRAIN_VENT_PWM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PWM output for drainage vent servos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRAINAGE_VENT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_DRAIN_VENT_SPM1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO for drainage vent power mosfet V1 – servo power mosfet 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_DRAIN_VENT_SPM2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO for drainage vent power mosfet V2 - servo power mosfet 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_DRAIN_VENT_ESO1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI (only) for drainage vent V1 open position end switch - end switch open 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_DRAIN_VENT_ESO2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO39</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI (only) for drainage vent V2 open position end switch - end switch open 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_DRAIN_VENT_ESC1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI (only) for drainage vent V1 close position end switch - end switch close 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_DRAIN_VENT_ESC2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI (only) for drainage vent V2 close position end switch - end switch close 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_ROULETTE_EN1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO for roulette R1 motor driver enable pin – enable 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROULETTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_ROULETTE_DIR1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO for roulette R1 motor driver direction bit 1 – direction 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_ROULETTE_DIR2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO for roulette R1 motor driver direction bit 2 – direction 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ROULETTE_TOP1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI for roulette R1 open position hall sensors – top 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ROULETTE_TOP2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI for roulette R1 open position hall sensors – top 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ROULETTE_BOT1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI for roulette R1 close position hall sensors – bottom 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ROULETTE_BOT2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI for roulette R1 close position hall sensors – bottom 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SPARE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spare pin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESP-IDF TIMERS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SYS_DRAIN_VENT_PWM_TIME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LEDC_TIMER_0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drainage vent servo PWM timer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESP-IDF CHANNELS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SYS_DRAIN_VENT_PWM_CHNL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LEDC_CHANNEL_0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drainage vent servo PWM channel.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRAINAGE VENT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STRUCTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FILE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ATRIBUTE TYPE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ATRIBUTE NAME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ledc_timer_config_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vsrp_dataset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ledc.h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ledc_mode_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">speed_mode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configuration structure for LEDC TIMER.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ledc_timer_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">timer_num</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ledc_timer_bit_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">duty_resolution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uint32_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">freq_hz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ledc_clk_cfg_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">clk_cfg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ledc_channel_config_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configuration structure for LEDC CHANNEL.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ledc_channel_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">channel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">timer_sel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ledc_intr_type_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">intr_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">int</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gpio_num</t>
-  </si>
-  <si>
-    <t xml:space="preserve">duty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hpoint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pwm_generator_config_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">timer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configuration structure for PWM GENERATOR.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">out_pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drainage_vent_dataset_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TickType_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">action_start_tick</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dataset structure which store drainage vent runtime properties.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v1_opn_ms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v1_cls_ms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v2_opn_ms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v2_cls_ms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v1_opn_duty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v1_cls_duty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v2_opn_duty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v2_cls_duty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uint16_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">err_word</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uint8_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">io_byte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ctrl_byte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BIT STRUCTURES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BYTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BIT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DATA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">READ BIN MASK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">READ HEX MASK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROCESS CODE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0b0000 0011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0x03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STRUCTURE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VENT 1 ENABLED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0b0001 0000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0x10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ATRIBUTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VENT 2 ENABLED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0b0010 0000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0x20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DATA TYPE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FSM STATES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FSM STATE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0b0000 1111</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0x0F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IDLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OFF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">START 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPEN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOVING 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLOSE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">START 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TMP PROCESS CODE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0b0011 0000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0x30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOVING 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FINISH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DUPONT &amp; UTP CABLE CONNECTION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CABLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COLOR 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COLOR 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DUPONT terminal – TOP view</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+10V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+6V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PWM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARROW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">roulette_dataset_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dataset structure which store roulette runtime properties.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">r1_opn_ms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">r1_cls_ms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROULETTE 1 ENABLED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACKNOWLEDGE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COLOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DUPONT connector – TOP view</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIGNAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VENT 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRAINAGE VENT DRIVER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VENT 2</t>
   </si>
   <si>
     <t xml:space="preserve">ESP32</t>
@@ -2641,11 +2641,11 @@
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
       <c r="E7" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F7" s="8"/>
       <c r="G7" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
@@ -2667,16 +2667,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
       <c r="E8" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F8" s="8"/>
       <c r="G8" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
@@ -2698,16 +2698,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
       <c r="E9" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F9" s="11"/>
       <c r="G9" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
@@ -2717,7 +2717,7 @@
       <c r="M9" s="11"/>
       <c r="N9" s="11"/>
       <c r="O9" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P9" s="11"/>
       <c r="Q9" s="11"/>
@@ -2731,16 +2731,16 @@
         <v>5</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
       <c r="E10" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F10" s="11"/>
       <c r="G10" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H10" s="11"/>
       <c r="I10" s="11"/>
@@ -2762,16 +2762,16 @@
         <v>6</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
       <c r="E11" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F11" s="13"/>
       <c r="G11" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H11" s="13"/>
       <c r="I11" s="13"/>
@@ -2781,7 +2781,7 @@
       <c r="M11" s="13"/>
       <c r="N11" s="13"/>
       <c r="O11" s="13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P11" s="13"/>
       <c r="Q11" s="13"/>
@@ -2795,16 +2795,16 @@
         <v>7</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
       <c r="E12" s="13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F12" s="13"/>
       <c r="G12" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H12" s="13"/>
       <c r="I12" s="13"/>
@@ -2826,16 +2826,16 @@
         <v>8</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H13" s="13"/>
       <c r="I13" s="13"/>
@@ -2857,16 +2857,16 @@
         <v>9</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F14" s="13"/>
       <c r="G14" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H14" s="13"/>
       <c r="I14" s="13"/>
@@ -2888,16 +2888,16 @@
         <v>10</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
       <c r="E15" s="13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F15" s="13"/>
       <c r="G15" s="13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H15" s="13"/>
       <c r="I15" s="13"/>
@@ -2919,16 +2919,16 @@
         <v>11</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F16" s="13"/>
       <c r="G16" s="13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H16" s="13"/>
       <c r="I16" s="13"/>
@@ -2950,16 +2950,16 @@
         <v>12</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
       <c r="E17" s="13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H17" s="13"/>
       <c r="I17" s="13"/>
@@ -2981,16 +2981,16 @@
         <v>13</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
       <c r="E18" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H18" s="15"/>
       <c r="I18" s="15"/>
@@ -3000,7 +3000,7 @@
       <c r="M18" s="15"/>
       <c r="N18" s="15"/>
       <c r="O18" s="15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="P18" s="15"/>
       <c r="Q18" s="15"/>
@@ -3014,16 +3014,16 @@
         <v>14</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C19" s="15"/>
       <c r="D19" s="15"/>
       <c r="E19" s="15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F19" s="15"/>
       <c r="G19" s="15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H19" s="15"/>
       <c r="I19" s="15"/>
@@ -3045,16 +3045,16 @@
         <v>15</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C20" s="15"/>
       <c r="D20" s="15"/>
       <c r="E20" s="15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F20" s="15"/>
       <c r="G20" s="15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H20" s="15"/>
       <c r="I20" s="15"/>
@@ -3076,16 +3076,16 @@
         <v>16</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C21" s="15"/>
       <c r="D21" s="15"/>
       <c r="E21" s="15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F21" s="15"/>
       <c r="G21" s="15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H21" s="15"/>
       <c r="I21" s="15"/>
@@ -3107,16 +3107,16 @@
         <v>17</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C22" s="15"/>
       <c r="D22" s="15"/>
       <c r="E22" s="15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F22" s="15"/>
       <c r="G22" s="15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H22" s="15"/>
       <c r="I22" s="15"/>
@@ -3138,16 +3138,16 @@
         <v>18</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C23" s="15"/>
       <c r="D23" s="15"/>
       <c r="E23" s="15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F23" s="15"/>
       <c r="G23" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H23" s="15"/>
       <c r="I23" s="15"/>
@@ -3169,16 +3169,16 @@
         <v>19</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
       <c r="E24" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F24" s="15"/>
       <c r="G24" s="15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H24" s="15"/>
       <c r="I24" s="15"/>
@@ -3200,16 +3200,16 @@
         <v>20</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
       <c r="E25" s="17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F25" s="17"/>
       <c r="G25" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H25" s="17"/>
       <c r="I25" s="17"/>
@@ -3219,7 +3219,7 @@
       <c r="M25" s="17"/>
       <c r="N25" s="17"/>
       <c r="O25" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P25" s="17"/>
       <c r="Q25" s="17"/>
@@ -3233,16 +3233,16 @@
         <v>21</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
       <c r="E26" s="17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F26" s="17"/>
       <c r="G26" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H26" s="17"/>
       <c r="I26" s="17"/>
@@ -3264,16 +3264,16 @@
         <v>22</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
       <c r="E27" s="17" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F27" s="17"/>
       <c r="G27" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H27" s="17"/>
       <c r="I27" s="17"/>
@@ -3295,16 +3295,16 @@
         <v>23</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C28" s="17"/>
       <c r="D28" s="17"/>
       <c r="E28" s="17" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F28" s="17"/>
       <c r="G28" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H28" s="17"/>
       <c r="I28" s="17"/>
@@ -3346,7 +3346,7 @@
     </row>
     <row r="30" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -3403,16 +3403,16 @@
         <v>1</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
       <c r="E32" s="13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F32" s="13"/>
       <c r="G32" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H32" s="13"/>
       <c r="I32" s="13"/>
@@ -3422,7 +3422,7 @@
       <c r="M32" s="13"/>
       <c r="N32" s="13"/>
       <c r="O32" s="13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P32" s="13"/>
       <c r="Q32" s="13"/>
@@ -3452,7 +3452,7 @@
     </row>
     <row r="34" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
@@ -3509,16 +3509,16 @@
         <v>1</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
       <c r="E36" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F36" s="13"/>
       <c r="G36" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H36" s="13"/>
       <c r="I36" s="13"/>
@@ -3528,7 +3528,7 @@
       <c r="M36" s="13"/>
       <c r="N36" s="13"/>
       <c r="O36" s="13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P36" s="13"/>
       <c r="Q36" s="13"/>
@@ -3558,7 +3558,7 @@
     </row>
     <row r="38" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B38" s="18"/>
       <c r="C38" s="18"/>
@@ -3583,7 +3583,7 @@
     </row>
     <row r="39" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
@@ -3616,17 +3616,17 @@
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
       <c r="E40" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L40" s="4"/>
       <c r="M40" s="4"/>
@@ -3646,31 +3646,31 @@
         <v>1</v>
       </c>
       <c r="B41" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="D41" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E41" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>123</v>
       </c>
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
       <c r="H41" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
       <c r="K41" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L41" s="5"/>
       <c r="M41" s="5"/>
       <c r="N41" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="O41" s="5"/>
       <c r="P41" s="5"/>
@@ -3689,12 +3689,12 @@
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
       <c r="H42" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
       <c r="K42" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="L42" s="5"/>
       <c r="M42" s="5"/>
@@ -3716,12 +3716,12 @@
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
       <c r="H43" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
       <c r="K43" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L43" s="5"/>
       <c r="M43" s="5"/>
@@ -3743,12 +3743,12 @@
       <c r="F44" s="5"/>
       <c r="G44" s="5"/>
       <c r="H44" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I44" s="5"/>
       <c r="J44" s="5"/>
       <c r="K44" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L44" s="5"/>
       <c r="M44" s="5"/>
@@ -3770,12 +3770,12 @@
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
       <c r="H45" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
       <c r="K45" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L45" s="5"/>
       <c r="M45" s="5"/>
@@ -3793,7 +3793,7 @@
         <v>2</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5"/>
@@ -3801,17 +3801,17 @@
       <c r="F46" s="5"/>
       <c r="G46" s="5"/>
       <c r="H46" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
       <c r="K46" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L46" s="5"/>
       <c r="M46" s="5"/>
       <c r="N46" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="O46" s="5"/>
       <c r="P46" s="5"/>
@@ -3830,12 +3830,12 @@
       <c r="F47" s="5"/>
       <c r="G47" s="5"/>
       <c r="H47" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
       <c r="K47" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L47" s="5"/>
       <c r="M47" s="5"/>
@@ -3857,12 +3857,12 @@
       <c r="F48" s="5"/>
       <c r="G48" s="5"/>
       <c r="H48" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I48" s="5"/>
       <c r="J48" s="5"/>
       <c r="K48" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L48" s="5"/>
       <c r="M48" s="5"/>
@@ -3884,12 +3884,12 @@
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
       <c r="H49" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
       <c r="K49" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L49" s="5"/>
       <c r="M49" s="5"/>
@@ -3911,12 +3911,12 @@
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
       <c r="H50" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I50" s="5"/>
       <c r="J50" s="5"/>
       <c r="K50" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L50" s="5"/>
       <c r="M50" s="5"/>
@@ -3938,12 +3938,12 @@
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
       <c r="H51" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I51" s="5"/>
       <c r="J51" s="5"/>
       <c r="K51" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="L51" s="5"/>
       <c r="M51" s="5"/>
@@ -3965,12 +3965,12 @@
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
       <c r="H52" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I52" s="5"/>
       <c r="J52" s="5"/>
       <c r="K52" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="L52" s="5"/>
       <c r="M52" s="5"/>
@@ -3988,7 +3988,7 @@
         <v>3</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5"/>
@@ -3998,17 +3998,17 @@
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
       <c r="H53" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I53" s="5"/>
       <c r="J53" s="5"/>
       <c r="K53" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="L53" s="5"/>
       <c r="M53" s="5"/>
       <c r="N53" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="O53" s="5"/>
       <c r="P53" s="5"/>
@@ -4027,12 +4027,12 @@
       <c r="F54" s="5"/>
       <c r="G54" s="5"/>
       <c r="H54" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I54" s="5"/>
       <c r="J54" s="5"/>
       <c r="K54" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L54" s="5"/>
       <c r="M54" s="5"/>
@@ -4054,12 +4054,12 @@
       <c r="F55" s="5"/>
       <c r="G55" s="5"/>
       <c r="H55" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I55" s="5"/>
       <c r="J55" s="5"/>
       <c r="K55" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L55" s="5"/>
       <c r="M55" s="5"/>
@@ -4081,12 +4081,12 @@
       <c r="F56" s="5"/>
       <c r="G56" s="5"/>
       <c r="H56" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I56" s="5"/>
       <c r="J56" s="5"/>
       <c r="K56" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="L56" s="5"/>
       <c r="M56" s="5"/>
@@ -4104,13 +4104,13 @@
         <v>4</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E57" s="5" t="s">
         <v>18</v>
@@ -4118,17 +4118,17 @@
       <c r="F57" s="5"/>
       <c r="G57" s="5"/>
       <c r="H57" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I57" s="5"/>
       <c r="J57" s="5"/>
       <c r="K57" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L57" s="5"/>
       <c r="M57" s="5"/>
       <c r="N57" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="O57" s="5"/>
       <c r="P57" s="5"/>
@@ -4147,12 +4147,12 @@
       <c r="F58" s="5"/>
       <c r="G58" s="5"/>
       <c r="H58" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I58" s="5"/>
       <c r="J58" s="5"/>
       <c r="K58" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="L58" s="5"/>
       <c r="M58" s="5"/>
@@ -4174,12 +4174,12 @@
       <c r="F59" s="5"/>
       <c r="G59" s="5"/>
       <c r="H59" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I59" s="5"/>
       <c r="J59" s="5"/>
       <c r="K59" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="L59" s="5"/>
       <c r="M59" s="5"/>
@@ -4201,12 +4201,12 @@
       <c r="F60" s="5"/>
       <c r="G60" s="5"/>
       <c r="H60" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I60" s="5"/>
       <c r="J60" s="5"/>
       <c r="K60" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L60" s="5"/>
       <c r="M60" s="5"/>
@@ -4228,12 +4228,12 @@
       <c r="F61" s="5"/>
       <c r="G61" s="5"/>
       <c r="H61" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I61" s="5"/>
       <c r="J61" s="5"/>
       <c r="K61" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L61" s="5"/>
       <c r="M61" s="5"/>
@@ -4255,12 +4255,12 @@
       <c r="F62" s="5"/>
       <c r="G62" s="5"/>
       <c r="H62" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I62" s="5"/>
       <c r="J62" s="5"/>
       <c r="K62" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L62" s="5"/>
       <c r="M62" s="5"/>
@@ -4282,12 +4282,12 @@
       <c r="F63" s="5"/>
       <c r="G63" s="5"/>
       <c r="H63" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I63" s="5"/>
       <c r="J63" s="5"/>
       <c r="K63" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L63" s="5"/>
       <c r="M63" s="5"/>
@@ -4309,12 +4309,12 @@
       <c r="F64" s="5"/>
       <c r="G64" s="5"/>
       <c r="H64" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I64" s="5"/>
       <c r="J64" s="5"/>
       <c r="K64" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L64" s="5"/>
       <c r="M64" s="5"/>
@@ -4336,12 +4336,12 @@
       <c r="F65" s="5"/>
       <c r="G65" s="5"/>
       <c r="H65" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I65" s="5"/>
       <c r="J65" s="5"/>
       <c r="K65" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L65" s="5"/>
       <c r="M65" s="5"/>
@@ -4363,12 +4363,12 @@
       <c r="F66" s="5"/>
       <c r="G66" s="5"/>
       <c r="H66" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I66" s="5"/>
       <c r="J66" s="5"/>
       <c r="K66" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L66" s="5"/>
       <c r="M66" s="5"/>
@@ -4390,12 +4390,12 @@
       <c r="F67" s="5"/>
       <c r="G67" s="5"/>
       <c r="H67" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I67" s="5"/>
       <c r="J67" s="5"/>
       <c r="K67" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="L67" s="5"/>
       <c r="M67" s="5"/>
@@ -4417,12 +4417,12 @@
       <c r="F68" s="5"/>
       <c r="G68" s="5"/>
       <c r="H68" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I68" s="5"/>
       <c r="J68" s="5"/>
       <c r="K68" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="L68" s="5"/>
       <c r="M68" s="5"/>
@@ -4460,7 +4460,7 @@
     </row>
     <row r="70" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B70" s="6"/>
       <c r="C70" s="6"/>
@@ -4497,21 +4497,21 @@
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D71" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="D71" s="4" t="s">
+      <c r="E71" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="E71" s="4" t="s">
-        <v>170</v>
       </c>
       <c r="F71" s="4"/>
       <c r="G71" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H71" s="4"/>
       <c r="I71" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J71" s="4"/>
       <c r="L71" s="4" t="s">
@@ -4519,21 +4519,21 @@
       </c>
       <c r="M71" s="4"/>
       <c r="N71" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="O71" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="O71" s="4" t="s">
+      <c r="P71" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="P71" s="4" t="s">
-        <v>170</v>
       </c>
       <c r="Q71" s="4"/>
       <c r="R71" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S71" s="4"/>
       <c r="T71" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U71" s="4"/>
     </row>
@@ -4546,10 +4546,10 @@
         <v>1</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E72" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F72" s="9"/>
       <c r="G72" s="9"/>
@@ -4564,28 +4564,28 @@
         <v>1</v>
       </c>
       <c r="O72" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="P72" s="5" t="s">
         <v>173</v>
-      </c>
-      <c r="P72" s="5" t="s">
-        <v>174</v>
       </c>
       <c r="Q72" s="5"/>
       <c r="R72" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="S72" s="5"/>
       <c r="T72" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U72" s="5"/>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C73" s="9"/>
       <c r="D73" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
@@ -4594,7 +4594,7 @@
       <c r="J73" s="9"/>
       <c r="N73" s="9"/>
       <c r="O73" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="P73" s="5"/>
       <c r="Q73" s="5"/>
@@ -4605,15 +4605,15 @@
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B74" s="4"/>
       <c r="C74" s="9"/>
       <c r="D74" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
@@ -4621,15 +4621,15 @@
       <c r="I74" s="9"/>
       <c r="J74" s="9"/>
       <c r="L74" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="M74" s="4"/>
       <c r="N74" s="9"/>
       <c r="O74" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="P74" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q74" s="9"/>
       <c r="R74" s="9"/>
@@ -4639,15 +4639,15 @@
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B75" s="5"/>
       <c r="C75" s="9"/>
       <c r="D75" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F75" s="9"/>
       <c r="G75" s="9"/>
@@ -4655,15 +4655,15 @@
       <c r="I75" s="9"/>
       <c r="J75" s="9"/>
       <c r="L75" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="M75" s="5"/>
       <c r="N75" s="9"/>
       <c r="O75" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q75" s="9"/>
       <c r="R75" s="9"/>
@@ -4674,10 +4674,10 @@
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C76" s="9"/>
       <c r="D76" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E76" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F76" s="9"/>
       <c r="G76" s="9"/>
@@ -4686,32 +4686,32 @@
       <c r="J76" s="9"/>
       <c r="N76" s="9"/>
       <c r="O76" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="P76" s="9" t="s">
         <v>181</v>
-      </c>
-      <c r="P76" s="9" t="s">
-        <v>182</v>
       </c>
       <c r="Q76" s="9"/>
       <c r="R76" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="S76" s="9"/>
       <c r="T76" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="U76" s="9"/>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="9"/>
       <c r="D77" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
@@ -4719,37 +4719,37 @@
       <c r="I77" s="9"/>
       <c r="J77" s="9"/>
       <c r="L77" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="M77" s="4"/>
       <c r="N77" s="9"/>
       <c r="O77" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="P77" s="9" t="s">
         <v>186</v>
-      </c>
-      <c r="P77" s="9" t="s">
-        <v>187</v>
       </c>
       <c r="Q77" s="9"/>
       <c r="R77" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="S77" s="9"/>
       <c r="T77" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="U77" s="9"/>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B78" s="5"/>
       <c r="C78" s="9"/>
       <c r="D78" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E78" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
@@ -4757,15 +4757,15 @@
       <c r="I78" s="9"/>
       <c r="J78" s="9"/>
       <c r="L78" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="M78" s="5"/>
       <c r="N78" s="9"/>
       <c r="O78" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P78" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q78" s="9"/>
       <c r="R78" s="9"/>
@@ -4776,10 +4776,10 @@
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C79" s="9"/>
       <c r="D79" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
@@ -4788,10 +4788,10 @@
       <c r="J79" s="9"/>
       <c r="N79" s="9"/>
       <c r="O79" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q79" s="9"/>
       <c r="R79" s="9"/>
@@ -4801,17 +4801,17 @@
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="9" t="n">
         <v>2</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E80" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F80" s="9"/>
       <c r="G80" s="9"/>
@@ -4819,7 +4819,7 @@
       <c r="I80" s="9"/>
       <c r="J80" s="9"/>
       <c r="L80" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="M80" s="4"/>
       <c r="N80" s="9"/>
@@ -4833,15 +4833,15 @@
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B81" s="5"/>
       <c r="C81" s="9"/>
       <c r="D81" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F81" s="9"/>
       <c r="G81" s="9"/>
@@ -4849,7 +4849,7 @@
       <c r="I81" s="9"/>
       <c r="J81" s="9"/>
       <c r="L81" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="M81" s="5"/>
       <c r="N81" s="9"/>
@@ -4864,10 +4864,10 @@
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C82" s="9"/>
       <c r="D82" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E82" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F82" s="9"/>
       <c r="G82" s="9"/>
@@ -4886,10 +4886,10 @@
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C83" s="9"/>
       <c r="D83" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E83" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F83" s="9"/>
       <c r="G83" s="9"/>
@@ -4908,10 +4908,10 @@
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C84" s="9"/>
       <c r="D84" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E84" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F84" s="9"/>
       <c r="G84" s="9"/>
@@ -4930,10 +4930,10 @@
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C85" s="9"/>
       <c r="D85" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F85" s="9"/>
       <c r="G85" s="9"/>
@@ -4952,10 +4952,10 @@
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C86" s="9"/>
       <c r="D86" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E86" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F86" s="9"/>
       <c r="G86" s="9"/>
@@ -4974,10 +4974,10 @@
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C87" s="9"/>
       <c r="D87" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E87" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F87" s="9"/>
       <c r="G87" s="9"/>
@@ -4999,29 +4999,29 @@
       </c>
       <c r="B89" s="4"/>
       <c r="C89" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D89" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="D89" s="4" t="s">
+      <c r="E89" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="E89" s="4" t="s">
-        <v>170</v>
       </c>
       <c r="F89" s="4"/>
       <c r="G89" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H89" s="4"/>
       <c r="I89" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J89" s="4"/>
       <c r="L89" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="M89" s="4"/>
       <c r="O89" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="P89" s="4"/>
     </row>
@@ -5034,37 +5034,37 @@
         <v>1</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F90" s="5"/>
       <c r="G90" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H90" s="5"/>
       <c r="I90" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="J90" s="5"/>
       <c r="L90" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M90" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O90" s="9" t="n">
         <v>0</v>
       </c>
       <c r="P90" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C91" s="9"/>
       <c r="D91" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E91" s="5"/>
       <c r="F91" s="5"/>
@@ -5076,23 +5076,23 @@
         <v>1</v>
       </c>
       <c r="M91" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="O91" s="9" t="n">
         <v>1</v>
       </c>
       <c r="P91" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B92" s="4"/>
       <c r="C92" s="9"/>
       <c r="D92" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
@@ -5104,23 +5104,23 @@
         <v>2</v>
       </c>
       <c r="M92" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="O92" s="9" t="n">
         <v>2</v>
       </c>
       <c r="P92" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B93" s="5"/>
       <c r="C93" s="9"/>
       <c r="D93" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E93" s="5"/>
       <c r="F93" s="5"/>
@@ -5132,47 +5132,47 @@
         <v>3</v>
       </c>
       <c r="M93" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="O93" s="9" t="n">
         <v>3</v>
       </c>
       <c r="P93" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C94" s="9"/>
       <c r="D94" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F94" s="5"/>
       <c r="G94" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H94" s="5"/>
       <c r="I94" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J94" s="5"/>
       <c r="L94" s="9" t="n">
         <v>4</v>
       </c>
       <c r="M94" s="9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B95" s="4"/>
       <c r="C95" s="9"/>
       <c r="D95" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E95" s="5"/>
       <c r="F95" s="5"/>
@@ -5184,20 +5184,20 @@
         <v>5</v>
       </c>
       <c r="M95" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B96" s="5"/>
       <c r="C96" s="9"/>
       <c r="D96" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E96" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F96" s="9"/>
       <c r="G96" s="9"/>
@@ -5208,10 +5208,10 @@
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C97" s="9"/>
       <c r="D97" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E97" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F97" s="9"/>
       <c r="G97" s="9"/>
@@ -5221,7 +5221,7 @@
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B98" s="4"/>
       <c r="C98" s="9"/>
@@ -5235,7 +5235,7 @@
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B99" s="5"/>
       <c r="C99" s="9"/>
@@ -5332,7 +5332,7 @@
     </row>
     <row r="107" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B107" s="6"/>
       <c r="C107" s="6"/>
@@ -5357,13 +5357,13 @@
     </row>
     <row r="108" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B108" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="B108" s="4" t="s">
+      <c r="C108" s="4" t="s">
         <v>219</v>
-      </c>
-      <c r="C108" s="4" t="s">
-        <v>220</v>
       </c>
       <c r="D108" s="4" t="s">
         <v>41</v>
@@ -5371,7 +5371,7 @@
       <c r="E108" s="4"/>
       <c r="F108" s="4"/>
       <c r="H108" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I108" s="4"/>
       <c r="J108" s="4"/>
@@ -5388,24 +5388,24 @@
       <c r="B109" s="19"/>
       <c r="C109" s="9"/>
       <c r="D109" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E109" s="5"/>
       <c r="F109" s="5"/>
       <c r="H109" s="20" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I109" s="21"/>
       <c r="J109" s="22" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="K109" s="21"/>
       <c r="L109" s="23" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="M109" s="21"/>
       <c r="N109" s="24" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="O109" s="21"/>
     </row>
@@ -5416,24 +5416,24 @@
       <c r="B110" s="19"/>
       <c r="C110" s="19"/>
       <c r="D110" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E110" s="5"/>
       <c r="F110" s="5"/>
       <c r="H110" s="20" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I110" s="25"/>
       <c r="J110" s="22" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="K110" s="26"/>
       <c r="L110" s="23" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="M110" s="27"/>
       <c r="N110" s="24" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="O110" s="28"/>
     </row>
@@ -5444,12 +5444,12 @@
       <c r="B111" s="29"/>
       <c r="C111" s="9"/>
       <c r="D111" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E111" s="5"/>
       <c r="F111" s="5"/>
       <c r="O111" s="30" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5459,7 +5459,7 @@
       <c r="B112" s="29"/>
       <c r="C112" s="29"/>
       <c r="D112" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E112" s="5"/>
       <c r="F112" s="5"/>
@@ -5475,7 +5475,7 @@
       <c r="B113" s="33"/>
       <c r="C113" s="9"/>
       <c r="D113" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E113" s="5"/>
       <c r="F113" s="5"/>
@@ -5489,7 +5489,7 @@
       <c r="B114" s="33"/>
       <c r="C114" s="33"/>
       <c r="D114" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E114" s="5"/>
       <c r="F114" s="5"/>
@@ -5501,7 +5501,7 @@
       <c r="B115" s="34"/>
       <c r="C115" s="9"/>
       <c r="D115" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E115" s="5"/>
       <c r="F115" s="5"/>
@@ -5513,7 +5513,7 @@
       <c r="B116" s="34"/>
       <c r="C116" s="34"/>
       <c r="D116" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E116" s="5"/>
       <c r="F116" s="5"/>
@@ -5543,7 +5543,7 @@
     </row>
     <row r="118" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B118" s="18"/>
       <c r="C118" s="18"/>
@@ -5568,7 +5568,7 @@
     </row>
     <row r="119" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B119" s="6"/>
       <c r="C119" s="6"/>
@@ -5601,17 +5601,17 @@
       <c r="C120" s="4"/>
       <c r="D120" s="4"/>
       <c r="E120" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F120" s="4"/>
       <c r="G120" s="4"/>
       <c r="H120" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I120" s="4"/>
       <c r="J120" s="4"/>
       <c r="K120" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L120" s="4"/>
       <c r="M120" s="4"/>
@@ -5631,7 +5631,7 @@
         <v>1</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C121" s="5"/>
       <c r="D121" s="5"/>
@@ -5641,21 +5641,21 @@
       <c r="F121" s="5"/>
       <c r="G121" s="5"/>
       <c r="H121" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="I121" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="J121" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="K121" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="I121" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="J121" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="K121" s="5" t="s">
-        <v>152</v>
       </c>
       <c r="L121" s="5"/>
       <c r="M121" s="5"/>
       <c r="N121" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="O121" s="5"/>
       <c r="P121" s="5"/>
@@ -5674,12 +5674,12 @@
       <c r="F122" s="5"/>
       <c r="G122" s="5"/>
       <c r="H122" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I122" s="5"/>
       <c r="J122" s="5"/>
       <c r="K122" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L122" s="5"/>
       <c r="M122" s="5"/>
@@ -5701,12 +5701,12 @@
       <c r="F123" s="5"/>
       <c r="G123" s="5"/>
       <c r="H123" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I123" s="5"/>
       <c r="J123" s="5"/>
       <c r="K123" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L123" s="5"/>
       <c r="M123" s="5"/>
@@ -5728,12 +5728,12 @@
       <c r="F124" s="5"/>
       <c r="G124" s="5"/>
       <c r="H124" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I124" s="5"/>
       <c r="J124" s="5"/>
       <c r="K124" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L124" s="5"/>
       <c r="M124" s="5"/>
@@ -5755,12 +5755,12 @@
       <c r="F125" s="5"/>
       <c r="G125" s="5"/>
       <c r="H125" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I125" s="5"/>
       <c r="J125" s="5"/>
       <c r="K125" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="L125" s="5"/>
       <c r="M125" s="5"/>
@@ -5782,12 +5782,12 @@
       <c r="F126" s="5"/>
       <c r="G126" s="5"/>
       <c r="H126" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I126" s="5"/>
       <c r="J126" s="5"/>
       <c r="K126" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="L126" s="5"/>
       <c r="M126" s="5"/>
@@ -5825,7 +5825,7 @@
     </row>
     <row r="128" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="6"/>
@@ -5862,21 +5862,21 @@
       </c>
       <c r="B129" s="4"/>
       <c r="C129" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D129" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="D129" s="4" t="s">
+      <c r="E129" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="E129" s="4" t="s">
-        <v>170</v>
       </c>
       <c r="F129" s="4"/>
       <c r="G129" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H129" s="4"/>
       <c r="I129" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J129" s="4"/>
       <c r="L129" s="4" t="s">
@@ -5884,21 +5884,21 @@
       </c>
       <c r="M129" s="4"/>
       <c r="N129" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="O129" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="O129" s="4" t="s">
+      <c r="P129" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="P129" s="4" t="s">
-        <v>170</v>
       </c>
       <c r="Q129" s="4"/>
       <c r="R129" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S129" s="4"/>
       <c r="T129" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U129" s="4"/>
     </row>
@@ -5911,10 +5911,10 @@
         <v>1</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E130" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F130" s="9"/>
       <c r="G130" s="9"/>
@@ -5929,28 +5929,28 @@
         <v>1</v>
       </c>
       <c r="O130" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="P130" s="5" t="s">
         <v>173</v>
-      </c>
-      <c r="P130" s="5" t="s">
-        <v>174</v>
       </c>
       <c r="Q130" s="5"/>
       <c r="R130" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="S130" s="5"/>
       <c r="T130" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U130" s="5"/>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C131" s="9"/>
       <c r="D131" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E131" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F131" s="9"/>
       <c r="G131" s="9"/>
@@ -5959,7 +5959,7 @@
       <c r="J131" s="9"/>
       <c r="N131" s="9"/>
       <c r="O131" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="P131" s="5"/>
       <c r="Q131" s="5"/>
@@ -5970,15 +5970,15 @@
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B132" s="4"/>
       <c r="C132" s="9"/>
       <c r="D132" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E132" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F132" s="9"/>
       <c r="G132" s="9"/>
@@ -5986,15 +5986,15 @@
       <c r="I132" s="9"/>
       <c r="J132" s="9"/>
       <c r="L132" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="M132" s="4"/>
       <c r="N132" s="9"/>
       <c r="O132" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="P132" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q132" s="9"/>
       <c r="R132" s="9"/>
@@ -6004,15 +6004,15 @@
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B133" s="5"/>
       <c r="C133" s="9"/>
       <c r="D133" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E133" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F133" s="9"/>
       <c r="G133" s="9"/>
@@ -6020,15 +6020,15 @@
       <c r="I133" s="9"/>
       <c r="J133" s="9"/>
       <c r="L133" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="M133" s="5"/>
       <c r="N133" s="9"/>
       <c r="O133" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="P133" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q133" s="9"/>
       <c r="R133" s="9"/>
@@ -6039,10 +6039,10 @@
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C134" s="9"/>
       <c r="D134" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E134" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F134" s="9"/>
       <c r="G134" s="9"/>
@@ -6051,32 +6051,32 @@
       <c r="J134" s="9"/>
       <c r="N134" s="9"/>
       <c r="O134" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P134" s="9" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="Q134" s="9"/>
       <c r="R134" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="S134" s="9"/>
       <c r="T134" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="U134" s="9"/>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B135" s="4"/>
       <c r="C135" s="9"/>
       <c r="D135" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E135" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F135" s="9"/>
       <c r="G135" s="9"/>
@@ -6084,15 +6084,15 @@
       <c r="I135" s="9"/>
       <c r="J135" s="9"/>
       <c r="L135" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="M135" s="4"/>
       <c r="N135" s="9"/>
       <c r="O135" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="P135" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q135" s="9"/>
       <c r="R135" s="9"/>
@@ -6102,15 +6102,15 @@
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B136" s="5"/>
       <c r="C136" s="9"/>
       <c r="D136" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E136" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F136" s="9"/>
       <c r="G136" s="9"/>
@@ -6118,15 +6118,15 @@
       <c r="I136" s="9"/>
       <c r="J136" s="9"/>
       <c r="L136" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="M136" s="5"/>
       <c r="N136" s="9"/>
       <c r="O136" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P136" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q136" s="9"/>
       <c r="R136" s="9"/>
@@ -6137,10 +6137,10 @@
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C137" s="9"/>
       <c r="D137" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E137" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F137" s="9"/>
       <c r="G137" s="9"/>
@@ -6149,10 +6149,10 @@
       <c r="J137" s="9"/>
       <c r="N137" s="9"/>
       <c r="O137" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P137" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q137" s="9"/>
       <c r="R137" s="9"/>
@@ -6162,17 +6162,17 @@
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B138" s="4"/>
       <c r="C138" s="9" t="n">
         <v>2</v>
       </c>
       <c r="D138" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E138" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F138" s="9"/>
       <c r="G138" s="9"/>
@@ -6180,7 +6180,7 @@
       <c r="I138" s="9"/>
       <c r="J138" s="9"/>
       <c r="L138" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="M138" s="4"/>
       <c r="N138" s="9"/>
@@ -6194,15 +6194,15 @@
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B139" s="5"/>
       <c r="C139" s="9"/>
       <c r="D139" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E139" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F139" s="9"/>
       <c r="G139" s="9"/>
@@ -6210,7 +6210,7 @@
       <c r="I139" s="9"/>
       <c r="J139" s="9"/>
       <c r="L139" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="M139" s="5"/>
       <c r="N139" s="9"/>
@@ -6225,10 +6225,10 @@
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C140" s="9"/>
       <c r="D140" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E140" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F140" s="9"/>
       <c r="G140" s="9"/>
@@ -6247,10 +6247,10 @@
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C141" s="9"/>
       <c r="D141" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E141" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F141" s="9"/>
       <c r="G141" s="9"/>
@@ -6269,10 +6269,10 @@
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C142" s="9"/>
       <c r="D142" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E142" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F142" s="9"/>
       <c r="G142" s="9"/>
@@ -6291,10 +6291,10 @@
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C143" s="9"/>
       <c r="D143" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E143" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F143" s="9"/>
       <c r="G143" s="9"/>
@@ -6313,10 +6313,10 @@
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C144" s="9"/>
       <c r="D144" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E144" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F144" s="9"/>
       <c r="G144" s="9"/>
@@ -6335,10 +6335,10 @@
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C145" s="9"/>
       <c r="D145" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E145" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F145" s="9"/>
       <c r="G145" s="9"/>
@@ -6360,30 +6360,30 @@
       </c>
       <c r="B147" s="4"/>
       <c r="C147" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D147" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="D147" s="4" t="s">
+      <c r="E147" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="E147" s="4" t="s">
-        <v>170</v>
       </c>
       <c r="F147" s="4"/>
       <c r="G147" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H147" s="4"/>
       <c r="I147" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J147" s="4"/>
       <c r="L147" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="M147" s="4"/>
       <c r="N147" s="4"/>
       <c r="P147" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="Q147" s="4"/>
     </row>
@@ -6396,38 +6396,38 @@
         <v>1</v>
       </c>
       <c r="D148" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E148" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F148" s="5"/>
       <c r="G148" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H148" s="5"/>
       <c r="I148" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="J148" s="5"/>
       <c r="L148" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M148" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="N148" s="9"/>
       <c r="P148" s="9" t="n">
         <v>0</v>
       </c>
       <c r="Q148" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C149" s="9"/>
       <c r="D149" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E149" s="5"/>
       <c r="F149" s="5"/>
@@ -6439,24 +6439,24 @@
         <v>1</v>
       </c>
       <c r="M149" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N149" s="9"/>
       <c r="P149" s="9" t="n">
         <v>1</v>
       </c>
       <c r="Q149" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B150" s="4"/>
       <c r="C150" s="9"/>
       <c r="D150" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E150" s="5"/>
       <c r="F150" s="5"/>
@@ -6468,24 +6468,24 @@
         <v>2</v>
       </c>
       <c r="M150" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="N150" s="9"/>
       <c r="P150" s="9" t="n">
         <v>2</v>
       </c>
       <c r="Q150" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B151" s="5"/>
       <c r="C151" s="9"/>
       <c r="D151" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E151" s="5"/>
       <c r="F151" s="5"/>
@@ -6497,49 +6497,49 @@
         <v>3</v>
       </c>
       <c r="M151" s="9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="N151" s="9"/>
       <c r="P151" s="9" t="n">
         <v>3</v>
       </c>
       <c r="Q151" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C152" s="9"/>
       <c r="D152" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E152" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F152" s="5"/>
       <c r="G152" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H152" s="5"/>
       <c r="I152" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J152" s="5"/>
       <c r="L152" s="9" t="n">
         <v>4</v>
       </c>
       <c r="M152" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="N152" s="9"/>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B153" s="4"/>
       <c r="C153" s="9"/>
       <c r="D153" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E153" s="5"/>
       <c r="F153" s="5"/>
@@ -6552,15 +6552,15 @@
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B154" s="5"/>
       <c r="C154" s="9"/>
       <c r="D154" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E154" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F154" s="9"/>
       <c r="G154" s="9"/>
@@ -6571,10 +6571,10 @@
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C155" s="9"/>
       <c r="D155" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E155" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F155" s="9"/>
       <c r="G155" s="9"/>
@@ -6584,7 +6584,7 @@
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B156" s="4"/>
       <c r="C156" s="9"/>
@@ -6598,7 +6598,7 @@
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B157" s="5"/>
       <c r="C157" s="9"/>
@@ -6695,7 +6695,7 @@
     </row>
     <row r="165" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="6"/>
@@ -6720,10 +6720,10 @@
     </row>
     <row r="166" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C166" s="4"/>
       <c r="D166" s="4" t="s">
@@ -6732,7 +6732,7 @@
       <c r="E166" s="4"/>
       <c r="F166" s="4"/>
       <c r="H166" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="I166" s="4"/>
       <c r="J166" s="4"/>
@@ -6747,20 +6747,20 @@
       <c r="B167" s="36"/>
       <c r="C167" s="36"/>
       <c r="D167" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E167" s="5"/>
       <c r="F167" s="5"/>
       <c r="H167" s="23" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I167" s="27"/>
       <c r="J167" s="37" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="K167" s="38"/>
       <c r="L167" s="39" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="M167" s="40"/>
     </row>
@@ -6771,12 +6771,12 @@
       <c r="B168" s="41"/>
       <c r="C168" s="41"/>
       <c r="D168" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E168" s="5"/>
       <c r="F168" s="5"/>
       <c r="M168" s="30" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6786,7 +6786,7 @@
       <c r="B169" s="33"/>
       <c r="C169" s="33"/>
       <c r="D169" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E169" s="5"/>
       <c r="F169" s="5"/>
@@ -7451,7 +7451,7 @@
       <c r="B3" s="46"/>
       <c r="C3" s="42"/>
       <c r="D3" s="47" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E3" s="47"/>
       <c r="F3" s="42"/>
@@ -7527,13 +7527,13 @@
       <c r="A6" s="42"/>
       <c r="B6" s="46"/>
       <c r="C6" s="51" t="s">
+        <v>237</v>
+      </c>
+      <c r="D6" s="52" t="s">
         <v>238</v>
       </c>
-      <c r="D6" s="52" t="s">
-        <v>239</v>
-      </c>
       <c r="E6" s="53" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F6" s="42"/>
       <c r="G6" s="42"/>
@@ -7559,10 +7559,10 @@
       <c r="B7" s="46"/>
       <c r="C7" s="51"/>
       <c r="D7" s="54" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E7" s="55" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F7" s="42"/>
       <c r="G7" s="42"/>
@@ -7588,10 +7588,10 @@
       <c r="B8" s="46"/>
       <c r="C8" s="51"/>
       <c r="D8" s="56" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E8" s="57" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F8" s="42"/>
       <c r="G8" s="42"/>
@@ -7605,7 +7605,7 @@
       <c r="O8" s="42"/>
       <c r="P8" s="42"/>
       <c r="Q8" s="58" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="R8" s="58"/>
       <c r="S8" s="58"/>
@@ -7619,10 +7619,10 @@
       <c r="B9" s="46"/>
       <c r="C9" s="51"/>
       <c r="D9" s="59" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E9" s="60" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F9" s="42"/>
       <c r="G9" s="42"/>
@@ -7672,13 +7672,13 @@
       <c r="A11" s="42"/>
       <c r="B11" s="46"/>
       <c r="C11" s="51" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D11" s="59" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E11" s="60" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F11" s="42"/>
       <c r="G11" s="42"/>
@@ -7704,10 +7704,10 @@
       <c r="B12" s="61"/>
       <c r="C12" s="51"/>
       <c r="D12" s="56" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E12" s="57" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V12" s="62"/>
       <c r="W12" s="42"/>
@@ -7717,10 +7717,10 @@
       <c r="B13" s="46"/>
       <c r="C13" s="51"/>
       <c r="D13" s="54" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E13" s="55" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F13" s="42"/>
       <c r="G13" s="42"/>
@@ -7737,7 +7737,7 @@
       <c r="R13" s="42"/>
       <c r="T13" s="36"/>
       <c r="U13" s="63" t="s">
-        <v>47</v>
+        <v>241</v>
       </c>
       <c r="V13" s="62"/>
       <c r="W13" s="42"/>
@@ -7747,10 +7747,10 @@
       <c r="B14" s="46"/>
       <c r="C14" s="51"/>
       <c r="D14" s="52" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E14" s="53" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F14" s="64"/>
       <c r="G14" s="64"/>
@@ -7832,7 +7832,7 @@
       <c r="N18" s="73"/>
       <c r="O18" s="73"/>
       <c r="P18" s="74" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="R18" s="42"/>
       <c r="T18" s="75"/>
@@ -7862,7 +7862,7 @@
       <c r="G20" s="76"/>
       <c r="H20" s="76"/>
       <c r="K20" s="77" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="L20" s="78"/>
       <c r="M20" s="79"/>
@@ -7921,7 +7921,7 @@
         <v>252</v>
       </c>
       <c r="K23" s="77" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="L23" s="78"/>
       <c r="M23" s="79"/>
@@ -7954,11 +7954,11 @@
     <row r="25" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="46"/>
       <c r="F25" s="86" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G25" s="87"/>
       <c r="H25" s="88" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="K25" s="76" t="s">
         <v>244</v>
@@ -8015,7 +8015,7 @@
       <c r="D28" s="49"/>
       <c r="E28" s="50"/>
       <c r="K28" s="83" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="L28" s="85"/>
       <c r="O28" s="49"/>

</xml_diff>